<commit_message>
redid lorentzian fits with 350ms (slight change), started ARO figures
</commit_message>
<xml_diff>
--- a/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
+++ b/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
@@ -555,13 +555,13 @@
         <v>38.29669189453125</v>
       </c>
       <c r="N2" t="n">
-        <v>13.49874031691002</v>
+        <v>13.76357921407892</v>
       </c>
       <c r="O2" t="n">
-        <v>5.701998066238218e-11</v>
+        <v>2.813538798148832e-11</v>
       </c>
       <c r="P2" t="n">
-        <v>1233.124453344375</v>
+        <v>1233.00912198773</v>
       </c>
     </row>
     <row r="3">
@@ -609,13 +609,13 @@
         <v>49.51171875</v>
       </c>
       <c r="N3" t="n">
-        <v>17.4228878035034</v>
+        <v>17.48944487684902</v>
       </c>
       <c r="O3" t="n">
-        <v>5.486692993972195e-11</v>
+        <v>2.735008223368497e-11</v>
       </c>
       <c r="P3" t="n">
-        <v>2155.309038931057</v>
+        <v>2155.319437958638</v>
       </c>
     </row>
     <row r="4">
@@ -663,13 +663,13 @@
         <v>77.76953125</v>
       </c>
       <c r="N4" t="n">
-        <v>18.5501801752043</v>
+        <v>18.37701490468909</v>
       </c>
       <c r="O4" t="n">
-        <v>2.457713479874036e-10</v>
+        <v>1.235028563709804e-10</v>
       </c>
       <c r="P4" t="n">
-        <v>3704.379755594088</v>
+        <v>3704.297679527263</v>
       </c>
     </row>
     <row r="5">
@@ -717,13 +717,13 @@
         <v>47.24951171875</v>
       </c>
       <c r="N5" t="n">
-        <v>34.66239683732749</v>
+        <v>34.76595543223775</v>
       </c>
       <c r="O5" t="n">
-        <v>1.357314261232701e-11</v>
+        <v>6.755779864268177e-12</v>
       </c>
       <c r="P5" t="n">
-        <v>4501.005395273555</v>
+        <v>4501.129974561822</v>
       </c>
     </row>
     <row r="6">
@@ -771,13 +771,13 @@
         <v>17.3978271484375</v>
       </c>
       <c r="N6" t="n">
-        <v>23.64426939454631</v>
+        <v>24.10412405477431</v>
       </c>
       <c r="O6" t="n">
-        <v>4.166610049075284e-11</v>
+        <v>2.059603196508205e-11</v>
       </c>
       <c r="P6" t="n">
-        <v>966.55485068773</v>
+        <v>966.5721338914575</v>
       </c>
     </row>
     <row r="7">
@@ -825,13 +825,13 @@
         <v>39.27484130859375</v>
       </c>
       <c r="N7" t="n">
-        <v>37.50996729651273</v>
+        <v>37.96421643976429</v>
       </c>
       <c r="O7" t="n">
-        <v>6.882964472826868e-11</v>
+        <v>3.395653054995207e-11</v>
       </c>
       <c r="P7" t="n">
-        <v>3028.626325285753</v>
+        <v>3028.875033791051</v>
       </c>
     </row>
     <row r="8">
@@ -879,13 +879,13 @@
         <v>52.03173828125001</v>
       </c>
       <c r="N8" t="n">
-        <v>23.2635660706599</v>
+        <v>23.35091952012064</v>
       </c>
       <c r="O8" t="n">
-        <v>3.176311143956635e-10</v>
+        <v>1.583734146407318e-10</v>
       </c>
       <c r="P8" t="n">
-        <v>3152.610821201952</v>
+        <v>3152.508980960771</v>
       </c>
     </row>
     <row r="9">
@@ -933,13 +933,13 @@
         <v>39.54034423828125</v>
       </c>
       <c r="N9" t="n">
-        <v>33.94081083081656</v>
+        <v>33.73452550992971</v>
       </c>
       <c r="O9" t="n">
-        <v>9.783328709239504e-11</v>
+        <v>4.926773925604347e-11</v>
       </c>
       <c r="P9" t="n">
-        <v>3945.227870712746</v>
+        <v>3944.963974235252</v>
       </c>
     </row>
     <row r="10">
@@ -987,13 +987,13 @@
         <v>72.459228515625</v>
       </c>
       <c r="N10" t="n">
-        <v>47.20527813440874</v>
+        <v>47.13257191358234</v>
       </c>
       <c r="O10" t="n">
-        <v>2.728374981284834e-11</v>
+        <v>1.369598844786981e-11</v>
       </c>
       <c r="P10" t="n">
-        <v>1801.595382692145</v>
+        <v>1801.655626397607</v>
       </c>
     </row>
     <row r="11">
@@ -1041,13 +1041,13 @@
         <v>56.63592529296875</v>
       </c>
       <c r="N11" t="n">
-        <v>14.17292855092692</v>
+        <v>14.21023832975533</v>
       </c>
       <c r="O11" t="n">
-        <v>1.939760310133725e-10</v>
+        <v>9.650500119140539e-11</v>
       </c>
       <c r="P11" t="n">
-        <v>2175.140023101672</v>
+        <v>2175.246197569066</v>
       </c>
     </row>
     <row r="12">
@@ -1095,13 +1095,13 @@
         <v>48.2607421875</v>
       </c>
       <c r="N12" t="n">
-        <v>24.04997435018094</v>
+        <v>24.17271670332591</v>
       </c>
       <c r="O12" t="n">
-        <v>1.421525365522831e-10</v>
+        <v>7.06937906864068e-11</v>
       </c>
       <c r="P12" t="n">
-        <v>3112.790751149034</v>
+        <v>3112.93841005744</v>
       </c>
     </row>
     <row r="13">
@@ -1149,13 +1149,13 @@
         <v>50.389892578125</v>
       </c>
       <c r="N13" t="n">
-        <v>24.36015673799121</v>
+        <v>24.60793692397083</v>
       </c>
       <c r="O13" t="n">
-        <v>1.028995778531184e-10</v>
+        <v>5.100088038041753e-11</v>
       </c>
       <c r="P13" t="n">
-        <v>3477.954975752495</v>
+        <v>3478.017965968106</v>
       </c>
     </row>
     <row r="14">
@@ -1203,13 +1203,13 @@
         <v>29.681640625</v>
       </c>
       <c r="N14" t="n">
-        <v>23.42245472006664</v>
+        <v>23.55275459339331</v>
       </c>
       <c r="O14" t="n">
-        <v>3.539291193544394e-11</v>
+        <v>1.759269509509833e-11</v>
       </c>
       <c r="P14" t="n">
-        <v>1793.19663419541</v>
+        <v>1793.479704400886</v>
       </c>
     </row>
     <row r="15">
@@ -1257,13 +1257,13 @@
         <v>17.12860107421875</v>
       </c>
       <c r="N15" t="n">
-        <v>41.13536799564929</v>
+        <v>41.30265573954974</v>
       </c>
       <c r="O15" t="n">
-        <v>7.102693742763213e-12</v>
+        <v>3.539373210432152e-12</v>
       </c>
       <c r="P15" t="n">
-        <v>2141.206698806877</v>
+        <v>2141.354446457694</v>
       </c>
     </row>
     <row r="16">
@@ -1311,13 +1311,13 @@
         <v>18.1419677734375</v>
       </c>
       <c r="N16" t="n">
-        <v>42.50273593021302</v>
+        <v>42.34817726778903</v>
       </c>
       <c r="O16" t="n">
-        <v>5.782920652556695e-12</v>
+        <v>2.902234163120909e-12</v>
       </c>
       <c r="P16" t="n">
-        <v>2413.916814391103</v>
+        <v>2413.939743194736</v>
       </c>
     </row>
     <row r="17">
@@ -1365,13 +1365,13 @@
         <v>69.547607421875</v>
       </c>
       <c r="N17" t="n">
-        <v>46.28212381639919</v>
+        <v>46.27969260680279</v>
       </c>
       <c r="O17" t="n">
-        <v>7.179066528684823e-12</v>
+        <v>3.577109007377321e-12</v>
       </c>
       <c r="P17" t="n">
-        <v>2784.485016813617</v>
+        <v>2784.865043070137</v>
       </c>
     </row>
     <row r="18">
@@ -1419,13 +1419,13 @@
         <v>10.7421875</v>
       </c>
       <c r="N18" t="n">
-        <v>42.43192224937608</v>
+        <v>42.66633598035457</v>
       </c>
       <c r="O18" t="n">
-        <v>6.387922355298556e-11</v>
+        <v>3.152433682764227e-11</v>
       </c>
       <c r="P18" t="n">
-        <v>1345.35643547757</v>
+        <v>1345.558150501267</v>
       </c>
     </row>
     <row r="19">
@@ -1473,13 +1473,13 @@
         <v>24.01885986328125</v>
       </c>
       <c r="N19" t="n">
-        <v>29.40023479776275</v>
+        <v>29.42202178338179</v>
       </c>
       <c r="O19" t="n">
-        <v>9.618238651727223e-11</v>
+        <v>4.771729493735052e-11</v>
       </c>
       <c r="P19" t="n">
-        <v>1782.520741488091</v>
+        <v>1782.379762773272</v>
       </c>
     </row>
     <row r="20">
@@ -1527,13 +1527,13 @@
         <v>31.024169921875</v>
       </c>
       <c r="N20" t="n">
-        <v>38.0453005907239</v>
+        <v>38.44768429616745</v>
       </c>
       <c r="O20" t="n">
-        <v>3.567629700403809e-11</v>
+        <v>1.774343353631128e-11</v>
       </c>
       <c r="P20" t="n">
-        <v>3644.343499219396</v>
+        <v>3644.432330447859</v>
       </c>
     </row>
     <row r="21">
@@ -1581,13 +1581,13 @@
         <v>80.01708984374999</v>
       </c>
       <c r="N21" t="n">
-        <v>23.25321642635075</v>
+        <v>23.01318201212892</v>
       </c>
       <c r="O21" t="n">
-        <v>4.348084875991019e-11</v>
+        <v>2.192222132226324e-11</v>
       </c>
       <c r="P21" t="n">
-        <v>4210.535049636132</v>
+        <v>4210.422772491951</v>
       </c>
     </row>
     <row r="22">
@@ -1635,13 +1635,13 @@
         <v>10.23101806640625</v>
       </c>
       <c r="N22" t="n">
-        <v>42.52731823436151</v>
+        <v>42.21255991974764</v>
       </c>
       <c r="O22" t="n">
-        <v>3.407190040037541e-11</v>
+        <v>1.71600307853262e-11</v>
       </c>
       <c r="P22" t="n">
-        <v>1361.167622259814</v>
+        <v>1360.86966387402</v>
       </c>
     </row>
     <row r="23">
@@ -1689,13 +1689,13 @@
         <v>15.0970458984375</v>
       </c>
       <c r="N23" t="n">
-        <v>39.7329860750773</v>
+        <v>39.77002884196471</v>
       </c>
       <c r="O23" t="n">
-        <v>4.203383502861764e-11</v>
+        <v>2.101229297986004e-11</v>
       </c>
       <c r="P23" t="n">
-        <v>1777.13636546578</v>
+        <v>1777.323367602554</v>
       </c>
     </row>
     <row r="24">
@@ -1743,13 +1743,13 @@
         <v>55.91125488281249</v>
       </c>
       <c r="N24" t="n">
-        <v>25.36364828994446</v>
+        <v>25.50541865779515</v>
       </c>
       <c r="O24" t="n">
-        <v>7.60903197647116e-11</v>
+        <v>3.783068554544835e-11</v>
       </c>
       <c r="P24" t="n">
-        <v>3604.698157424685</v>
+        <v>3604.758004675124</v>
       </c>
     </row>
     <row r="25">
@@ -1797,13 +1797,13 @@
         <v>37.35351562499999</v>
       </c>
       <c r="N25" t="n">
-        <v>39.00656358010245</v>
+        <v>39.16627633705617</v>
       </c>
       <c r="O25" t="n">
-        <v>1.972760643713383e-11</v>
+        <v>9.845293129520055e-12</v>
       </c>
       <c r="P25" t="n">
-        <v>4390.435377240718</v>
+        <v>4390.472362905448</v>
       </c>
     </row>
     <row r="26">
@@ -1851,13 +1851,13 @@
         <v>20.1171875</v>
       </c>
       <c r="N26" t="n">
-        <v>26.82594700506083</v>
+        <v>26.78638101426216</v>
       </c>
       <c r="O26" t="n">
-        <v>5.362201724144603e-11</v>
+        <v>2.689083012062509e-11</v>
       </c>
       <c r="P26" t="n">
-        <v>1256.960007381276</v>
+        <v>1256.959658401852</v>
       </c>
     </row>
     <row r="27">
@@ -1905,13 +1905,13 @@
         <v>12.860107421875</v>
       </c>
       <c r="N27" t="n">
-        <v>44.89910219652642</v>
+        <v>45.09541545147014</v>
       </c>
       <c r="O27" t="n">
-        <v>3.238278432155652e-11</v>
+        <v>1.609361979514102e-11</v>
       </c>
       <c r="P27" t="n">
-        <v>1839.357708970227</v>
+        <v>1839.488305202574</v>
       </c>
     </row>
     <row r="28">
@@ -1959,13 +1959,13 @@
         <v>18.0511474609375</v>
       </c>
       <c r="N28" t="n">
-        <v>43.5534635931605</v>
+        <v>43.57426733179351</v>
       </c>
       <c r="O28" t="n">
-        <v>1.750986941562969e-11</v>
+        <v>8.757415282657275e-12</v>
       </c>
       <c r="P28" t="n">
-        <v>2573.086521837186</v>
+        <v>2572.886713729026</v>
       </c>
     </row>
     <row r="29">
@@ -2013,13 +2013,13 @@
         <v>46.37756347656249</v>
       </c>
       <c r="N29" t="n">
-        <v>28.65389346138159</v>
+        <v>28.54024203390058</v>
       </c>
       <c r="O29" t="n">
-        <v>3.512408565127503e-11</v>
+        <v>1.757871137128941e-11</v>
       </c>
       <c r="P29" t="n">
-        <v>3559.281782220796</v>
+        <v>3559.172952959399</v>
       </c>
     </row>
     <row r="30">
@@ -2067,13 +2067,13 @@
         <v>20.6451416015625</v>
       </c>
       <c r="N30" t="n">
-        <v>24.71837056218591</v>
+        <v>24.92820201618651</v>
       </c>
       <c r="O30" t="n">
-        <v>7.686499052157489e-11</v>
+        <v>3.834120878250849e-11</v>
       </c>
       <c r="P30" t="n">
-        <v>1251.205006488157</v>
+        <v>1251.287838447055</v>
       </c>
     </row>
     <row r="31">
@@ -2121,13 +2121,13 @@
         <v>27.20489501953125</v>
       </c>
       <c r="N31" t="n">
-        <v>31.39880304265806</v>
+        <v>31.27955333718139</v>
       </c>
       <c r="O31" t="n">
-        <v>4.100477372317999e-11</v>
+        <v>2.053361281504691e-11</v>
       </c>
       <c r="P31" t="n">
-        <v>2591.363959375077</v>
+        <v>2591.805130181283</v>
       </c>
     </row>
     <row r="32">
@@ -2175,13 +2175,13 @@
         <v>24.1241455078125</v>
       </c>
       <c r="N32" t="n">
-        <v>40.44577822285396</v>
+        <v>40.60474868382574</v>
       </c>
       <c r="O32" t="n">
-        <v>1.151139691059027e-11</v>
+        <v>5.761462717113044e-12</v>
       </c>
       <c r="P32" t="n">
-        <v>3220.120349829717</v>
+        <v>3220.389925054321</v>
       </c>
     </row>
     <row r="33">
@@ -2229,13 +2229,13 @@
         <v>35.82763671874999</v>
       </c>
       <c r="N33" t="n">
-        <v>33.66392465289412</v>
+        <v>33.43948673382051</v>
       </c>
       <c r="O33" t="n">
-        <v>3.862470882993179e-11</v>
+        <v>1.950103839622597e-11</v>
       </c>
       <c r="P33" t="n">
-        <v>3583.640453835764</v>
+        <v>3584.025592853023</v>
       </c>
     </row>
     <row r="34">
@@ -2283,13 +2283,13 @@
         <v>15.22705078125</v>
       </c>
       <c r="N34" t="n">
-        <v>88.04686450596937</v>
+        <v>87.64883889212321</v>
       </c>
       <c r="O34" t="n">
-        <v>3.597180564459571e-13</v>
+        <v>1.806475847363449e-13</v>
       </c>
       <c r="P34" t="n">
-        <v>4346.828152195468</v>
+        <v>4347.72734487957</v>
       </c>
     </row>
     <row r="35">
@@ -2337,13 +2337,13 @@
         <v>37.265625</v>
       </c>
       <c r="N35" t="n">
-        <v>67.85515544987975</v>
+        <v>68.22161768748448</v>
       </c>
       <c r="O35" t="n">
-        <v>1.26189758663374e-12</v>
+        <v>6.30085870083755e-13</v>
       </c>
       <c r="P35" t="n">
-        <v>7456.96221043282</v>
+        <v>7456.907112586428</v>
       </c>
     </row>
     <row r="36">
@@ -2391,13 +2391,13 @@
         <v>46.48681640625</v>
       </c>
       <c r="N36" t="n">
-        <v>60.03149730150874</v>
+        <v>60.09398519868756</v>
       </c>
       <c r="O36" t="n">
-        <v>3.555192550123271e-12</v>
+        <v>1.784690547665494e-12</v>
       </c>
       <c r="P36" t="n">
-        <v>8444.898188380446</v>
+        <v>8445.060419516562</v>
       </c>
     </row>
     <row r="37">
@@ -2445,13 +2445,13 @@
         <v>72.2109375</v>
       </c>
       <c r="N37" t="n">
-        <v>48.1155010115467</v>
+        <v>48.17177549386727</v>
       </c>
       <c r="O37" t="n">
-        <v>4.091123796662425e-12</v>
+        <v>2.045822095595467e-12</v>
       </c>
       <c r="P37" t="n">
-        <v>9030.619519845581</v>
+        <v>9030.795774783386</v>
       </c>
     </row>
     <row r="38">
@@ -2499,13 +2499,13 @@
         <v>27.3515625</v>
       </c>
       <c r="N38" t="n">
-        <v>77.00428622253314</v>
+        <v>76.67818748697763</v>
       </c>
       <c r="O38" t="n">
-        <v>7.722440708880625e-13</v>
+        <v>3.885635794226587e-13</v>
       </c>
       <c r="P38" t="n">
-        <v>6840.659444440797</v>
+        <v>6840.757442741772</v>
       </c>
     </row>
     <row r="39">
@@ -2553,13 +2553,13 @@
         <v>63.2109375</v>
       </c>
       <c r="N39" t="n">
-        <v>51.67437961669827</v>
+        <v>51.7303391195944</v>
       </c>
       <c r="O39" t="n">
-        <v>1.393890798981966e-12</v>
+        <v>6.977991565512491e-13</v>
       </c>
       <c r="P39" t="n">
-        <v>7901.211008017457</v>
+        <v>7901.190467312519</v>
       </c>
     </row>
     <row r="40">
@@ -2607,13 +2607,13 @@
         <v>70.6875</v>
       </c>
       <c r="N40" t="n">
-        <v>49.4686715984015</v>
+        <v>49.42569815474504</v>
       </c>
       <c r="O40" t="n">
-        <v>2.577618012957903e-12</v>
+        <v>1.292541591210098e-12</v>
       </c>
       <c r="P40" t="n">
-        <v>8845.345193607762</v>
+        <v>8845.361149512852</v>
       </c>
     </row>
     <row r="41">
@@ -2661,13 +2661,13 @@
         <v>134.23828125</v>
       </c>
       <c r="N41" t="n">
-        <v>89.47811797763433</v>
+        <v>89.73515677713675</v>
       </c>
       <c r="O41" t="n">
-        <v>1.537070170817859e-12</v>
+        <v>7.664901288177202e-13</v>
       </c>
       <c r="P41" t="n">
-        <v>9253.719655990404</v>
+        <v>9253.893064877439</v>
       </c>
     </row>
     <row r="42">
@@ -2715,13 +2715,13 @@
         <v>53.4490966796875</v>
       </c>
       <c r="N42" t="n">
-        <v>55.63156172241037</v>
+        <v>55.38194222549402</v>
       </c>
       <c r="O42" t="n">
-        <v>1.588033309690506e-10</v>
+        <v>7.975997509325952e-11</v>
       </c>
       <c r="P42" t="n">
-        <v>5623.301707548723</v>
+        <v>5623.316734238025</v>
       </c>
     </row>
     <row r="43">
@@ -2769,13 +2769,13 @@
         <v>48.65234375</v>
       </c>
       <c r="N43" t="n">
-        <v>58.59552907829816</v>
+        <v>58.78366132431848</v>
       </c>
       <c r="O43" t="n">
-        <v>2.598374680921007e-10</v>
+        <v>1.299537582437962e-10</v>
       </c>
       <c r="P43" t="n">
-        <v>8098.389244124367</v>
+        <v>8098.586383255675</v>
       </c>
     </row>
     <row r="44">
@@ -2823,13 +2823,13 @@
         <v>127.438232421875</v>
       </c>
       <c r="N44" t="n">
-        <v>24.65121885617466</v>
+        <v>24.82765613524692</v>
       </c>
       <c r="O44" t="n">
-        <v>7.426545525735238e-10</v>
+        <v>3.706405454296643e-10</v>
       </c>
       <c r="P44" t="n">
-        <v>8486.990976232802</v>
+        <v>8486.907248855707</v>
       </c>
     </row>
     <row r="45">
@@ -2877,13 +2877,13 @@
         <v>49.43634033203125</v>
       </c>
       <c r="N45" t="n">
-        <v>64.04212616111205</v>
+        <v>63.90181081181339</v>
       </c>
       <c r="O45" t="n">
-        <v>1.931726648220092e-10</v>
+        <v>9.69195629278402e-11</v>
       </c>
       <c r="P45" t="n">
-        <v>9857.012236195154</v>
+        <v>9856.932898275971</v>
       </c>
     </row>
     <row r="46">
@@ -2931,13 +2931,13 @@
         <v>22.2000732421875</v>
       </c>
       <c r="N46" t="n">
-        <v>73.48509442051802</v>
+        <v>73.82638021620554</v>
       </c>
       <c r="O46" t="n">
-        <v>9.288702845355572e-11</v>
+        <v>4.610246676062042e-11</v>
       </c>
       <c r="P46" t="n">
-        <v>4954.788686667887</v>
+        <v>4954.457814883755</v>
       </c>
     </row>
     <row r="47">
@@ -2985,13 +2985,13 @@
         <v>86.5885009765625</v>
       </c>
       <c r="N47" t="n">
-        <v>26.50530117044341</v>
+        <v>26.63568621305765</v>
       </c>
       <c r="O47" t="n">
-        <v>4.067304936525313e-10</v>
+        <v>2.037326814883841e-10</v>
       </c>
       <c r="P47" t="n">
-        <v>5766.3279789766</v>
+        <v>5766.206632270292</v>
       </c>
     </row>
     <row r="48">
@@ -3039,13 +3039,13 @@
         <v>463.295654296875</v>
       </c>
       <c r="N48" t="n">
-        <v>5.56825361287411</v>
+        <v>5.600274938598027</v>
       </c>
       <c r="O48" t="n">
-        <v>1.100894634208016e-08</v>
+        <v>5.484176416186218e-09</v>
       </c>
       <c r="P48" t="n">
-        <v>7182.023695604765</v>
+        <v>7182.063356605612</v>
       </c>
     </row>
     <row r="49">
@@ -3093,13 +3093,13 @@
         <v>317.8372192382812</v>
       </c>
       <c r="N49" t="n">
-        <v>11.84121353021598</v>
+        <v>12.07424623307133</v>
       </c>
       <c r="O49" t="n">
-        <v>3.857816204061241e-09</v>
+        <v>1.899439743021853e-09</v>
       </c>
       <c r="P49" t="n">
-        <v>9634.434320710956</v>
+        <v>9634.460544446882</v>
       </c>
     </row>
     <row r="50">
@@ -3147,13 +3147,13 @@
         <v>62.536865234375</v>
       </c>
       <c r="N50" t="n">
-        <v>13.37569700231536</v>
+        <v>13.39453994590456</v>
       </c>
       <c r="O50" t="n">
-        <v>4.387388411543119e-12</v>
+        <v>2.196421233614644e-12</v>
       </c>
       <c r="P50" t="n">
-        <v>2659.812159338104</v>
+        <v>2659.676701636059</v>
       </c>
     </row>
     <row r="51">
@@ -3201,13 +3201,13 @@
         <v>283.268310546875</v>
       </c>
       <c r="N51" t="n">
-        <v>4.396755746018324</v>
+        <v>4.548385840690079</v>
       </c>
       <c r="O51" t="n">
-        <v>1.580118125759308e-11</v>
+        <v>7.782864418659612e-12</v>
       </c>
       <c r="P51" t="n">
-        <v>2804.051171728255</v>
+        <v>2804.093986490997</v>
       </c>
     </row>
     <row r="52">
@@ -3255,13 +3255,13 @@
         <v>470.7158203125</v>
       </c>
       <c r="N52" t="n">
-        <v>3.20347974555013</v>
+        <v>3.385749687296979</v>
       </c>
       <c r="O52" t="n">
-        <v>3.471135036038896e-11</v>
+        <v>1.649522971510552e-11</v>
       </c>
       <c r="P52" t="n">
-        <v>2943.07516048353</v>
+        <v>2943.013811279915</v>
       </c>
     </row>
     <row r="53">
@@ -3309,13 +3309,13 @@
         <v>741.5859985351562</v>
       </c>
       <c r="N53" t="n">
-        <v>2.924789762497687</v>
+        <v>3.045758270631805</v>
       </c>
       <c r="O53" t="n">
-        <v>5.721370416804932e-11</v>
+        <v>2.7509079510722e-11</v>
       </c>
       <c r="P53" t="n">
-        <v>3862.782205536074</v>
+        <v>3862.739037311213</v>
       </c>
     </row>
     <row r="54">
@@ -3363,13 +3363,13 @@
         <v>1849.011779785156</v>
       </c>
       <c r="N54" t="n">
-        <v>1.199989206411956</v>
+        <v>1.700255064897827</v>
       </c>
       <c r="O54" t="n">
-        <v>4.005964519290518e-10</v>
+        <v>1.219344120318504e-10</v>
       </c>
       <c r="P54" t="n">
-        <v>2340.272845939905</v>
+        <v>2340.388090027172</v>
       </c>
     </row>
     <row r="55">
@@ -3417,13 +3417,13 @@
         <v>1918.085021972656</v>
       </c>
       <c r="N55" t="n">
-        <v>1.676873230797176</v>
+        <v>1.28095518819708</v>
       </c>
       <c r="O55" t="n">
-        <v>4.9076822679619e-11</v>
+        <v>3.398105938092607e-11</v>
       </c>
       <c r="P55" t="n">
-        <v>4050.173672412683</v>
+        <v>4050.203365680363</v>
       </c>
     </row>
     <row r="56">
@@ -3471,13 +3471,13 @@
         <v>1173.462890625</v>
       </c>
       <c r="N56" t="n">
-        <v>2.671077526653983</v>
+        <v>2.935485532484775</v>
       </c>
       <c r="O56" t="n">
-        <v>6.024852360282668e-11</v>
+        <v>2.796867277425509e-11</v>
       </c>
       <c r="P56" t="n">
-        <v>5839.384508310388</v>
+        <v>5839.230198622787</v>
       </c>
     </row>
     <row r="57">
@@ -3525,13 +3525,13 @@
         <v>3734.960998535156</v>
       </c>
       <c r="N57" t="n">
-        <v>1.15072627530995</v>
+        <v>1.387349873576789</v>
       </c>
       <c r="O57" t="n">
-        <v>2.139880006016499e-09</v>
+        <v>9.021792532535704e-10</v>
       </c>
       <c r="P57" t="n">
-        <v>8310.263470697417</v>
+        <v>8309.988515326677</v>
       </c>
     </row>
     <row r="58">
@@ -3579,13 +3579,13 @@
         <v>863.912109375</v>
       </c>
       <c r="N58" t="n">
-        <v>1.822014315463064</v>
+        <v>1.869358907589715</v>
       </c>
       <c r="O58" t="n">
-        <v>1.697379656316001e-10</v>
+        <v>8.443746198615233e-11</v>
       </c>
       <c r="P58" t="n">
-        <v>733.1087229617199</v>
+        <v>732.9333705336513</v>
       </c>
     </row>
     <row r="59">
@@ -3633,13 +3633,13 @@
         <v>1348.664428710938</v>
       </c>
       <c r="N59" t="n">
-        <v>2.033610502307091</v>
+        <v>2.111207187761406</v>
       </c>
       <c r="O59" t="n">
-        <v>9.001391189393193e-11</v>
+        <v>4.54303482517407e-11</v>
       </c>
       <c r="P59" t="n">
-        <v>984.5673723153527</v>
+        <v>984.581668316362</v>
       </c>
     </row>
     <row r="60">
@@ -3687,13 +3687,13 @@
         <v>177.2763061523438</v>
       </c>
       <c r="N60" t="n">
-        <v>5.767663439898371</v>
+        <v>5.527666438818121</v>
       </c>
       <c r="O60" t="n">
-        <v>1.762617398163122e-11</v>
+        <v>9.064826848430388e-12</v>
       </c>
       <c r="P60" t="n">
-        <v>1634.52111418689</v>
+        <v>1634.412669824537</v>
       </c>
     </row>
     <row r="61">
@@ -3741,13 +3741,13 @@
         <v>1410.150085449219</v>
       </c>
       <c r="N61" t="n">
-        <v>1.880640892936283</v>
+        <v>1.833350440871084</v>
       </c>
       <c r="O61" t="n">
-        <v>5.923811919470027e-11</v>
+        <v>3.090843463916614e-11</v>
       </c>
       <c r="P61" t="n">
-        <v>2226.341842484205</v>
+        <v>2226.429989231169</v>
       </c>
     </row>
     <row r="62">
@@ -3795,13 +3795,13 @@
         <v>587.8564453125</v>
       </c>
       <c r="N62" t="n">
-        <v>2.209909336702901</v>
+        <v>2.545154730379255</v>
       </c>
       <c r="O62" t="n">
-        <v>1.575130906454158e-08</v>
+        <v>7.161708852846133e-09</v>
       </c>
       <c r="P62" t="n">
-        <v>905.0584409282009</v>
+        <v>904.9686777906261</v>
       </c>
     </row>
     <row r="63">
@@ -3849,13 +3849,13 @@
         <v>1394.56787109375</v>
       </c>
       <c r="N63" t="n">
-        <v>1.575827832325747</v>
+        <v>1.952430412995464</v>
       </c>
       <c r="O63" t="n">
-        <v>1.882751022310289e-08</v>
+        <v>7.462411328533061e-09</v>
       </c>
       <c r="P63" t="n">
-        <v>1519.908625157091</v>
+        <v>1520.304279797999</v>
       </c>
     </row>
     <row r="64">
@@ -3903,13 +3903,13 @@
         <v>847.6514892578125</v>
       </c>
       <c r="N64" t="n">
-        <v>1.995825703258068</v>
+        <v>1.725143363002918</v>
       </c>
       <c r="O64" t="n">
-        <v>1.428661381424328e-08</v>
+        <v>8.231508706457555e-09</v>
       </c>
       <c r="P64" t="n">
-        <v>2038.049182456879</v>
+        <v>2038.146974608225</v>
       </c>
     </row>
     <row r="65">
@@ -3957,13 +3957,13 @@
         <v>98.3648681640625</v>
       </c>
       <c r="N65" t="n">
-        <v>9.883714629885734</v>
+        <v>9.907909797259302</v>
       </c>
       <c r="O65" t="n">
-        <v>5.177606603663085e-10</v>
+        <v>2.614181286759171e-10</v>
       </c>
       <c r="P65" t="n">
-        <v>2695.97693516991</v>
+        <v>2696.097771353126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
switched over Qerb, finished incorporating notes on poster
</commit_message>
<xml_diff>
--- a/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
+++ b/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,60 +451,65 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Frequency (Rounded)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>N_xi</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>N_xi_std</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>T_xi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>T_xi_std</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>A_xi</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>A_xi_std</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>MSE</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Decayed Xi</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Decayed Num Cycles</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>L_gamma</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>L_amp</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>L_f0</t>
         </is>
@@ -528,39 +533,42 @@
         <v>1235.467529296875</v>
       </c>
       <c r="E2" t="n">
+        <v>1235</v>
+      </c>
+      <c r="F2" t="n">
         <v>16.27045348324553</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.1604725269936995</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.01316947074481619</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.0001298880975730921</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.9985519516693381</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.007620958622036293</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.0001611813450498767</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.03099773242630385</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>38.29669189453125</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>13.76357921407892</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>2.813538798148832e-11</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>1233.00912198773</v>
       </c>
     </row>
@@ -582,39 +590,42 @@
         <v>2153.3203125</v>
       </c>
       <c r="E3" t="n">
+        <v>2153</v>
+      </c>
+      <c r="F3" t="n">
         <v>19.32091238876069</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.1191495762712399</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.008972614188703376</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>5.533295514818578e-05</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1.138955073099183</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.005973835603635176</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>4.912864377187464e-05</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.02299319727891156</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>49.51171875</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>17.48944487684902</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>2.735008223368497e-11</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>2155.319437958638</v>
       </c>
     </row>
@@ -636,39 +647,42 @@
         <v>3703.7109375</v>
       </c>
       <c r="E4" t="n">
+        <v>3704</v>
+      </c>
+      <c r="F4" t="n">
         <v>31.46322969314967</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.1427470844557601</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.008495055425245283</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>3.854163752641942e-05</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>1.206275863016083</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.004677101758986906</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>2.622069975168253e-05</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.02099773242630385</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>77.76953125</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>18.37701490468909</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>1.235028563709804e-10</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>3704.297679527263</v>
       </c>
     </row>
@@ -690,39 +704,42 @@
         <v>4500.439453125</v>
       </c>
       <c r="E5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F5" t="n">
         <v>18.73891316765203</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0.5111525313559319</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.004163796305411945</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.0001135783597757324</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>1.331207539183221</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.03210092064674847</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.0004891674757343065</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>0.01049886621315193</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>47.24951171875</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>34.76595543223775</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>6.755779864268177e-12</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>4501.129974561822</v>
       </c>
     </row>
@@ -744,39 +761,42 @@
         <v>966.302490234375</v>
       </c>
       <c r="E6" t="n">
+        <v>966</v>
+      </c>
+      <c r="F6" t="n">
         <v>6.137620528466492</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>0.1872804185843038</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>0.006351655501765107</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>0.0001938113794355215</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>1.072079156092322</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.02693463093490572</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.0009077351656215396</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>0.01800453514739229</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>17.3978271484375</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>24.10412405477431</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>2.059603196508205e-11</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>966.5721338914575</v>
       </c>
     </row>
@@ -795,43 +815,46 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3022.723388671875</v>
+        <v>3151.922607421875</v>
       </c>
       <c r="E7" t="n">
-        <v>10.73828304736731</v>
+        <v>3152</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6264526162404236</v>
+        <v>20.46677603291103</v>
       </c>
       <c r="G7" t="n">
-        <v>0.003552519257174074</v>
+        <v>0.2005660799087317</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002072477483676316</v>
+        <v>0.006493425944126177</v>
       </c>
       <c r="I7" t="n">
-        <v>1.213076971725806</v>
+        <v>6.363293293955125e-05</v>
       </c>
       <c r="J7" t="n">
-        <v>0.06904941171546593</v>
+        <v>1.243291384815935</v>
       </c>
       <c r="K7" t="n">
-        <v>0.001860346665208865</v>
+        <v>0.01051288534168879</v>
       </c>
       <c r="L7" t="n">
-        <v>0.01299319727891157</v>
+        <v>9.893151436961653e-05</v>
       </c>
       <c r="M7" t="n">
-        <v>39.27484130859375</v>
+        <v>0.01650793650793651</v>
       </c>
       <c r="N7" t="n">
-        <v>37.96421643976429</v>
+        <v>52.03173828125001</v>
       </c>
       <c r="O7" t="n">
-        <v>3.395653054995207e-11</v>
+        <v>23.35091952012064</v>
       </c>
       <c r="P7" t="n">
-        <v>3028.875033791051</v>
+        <v>1.583734146407318e-10</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3152.508980960771</v>
       </c>
     </row>
     <row r="8">
@@ -849,43 +872,46 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3151.922607421875</v>
+        <v>3954.034423828125</v>
       </c>
       <c r="E8" t="n">
-        <v>20.46677603291103</v>
+        <v>3954</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2005660799087317</v>
+        <v>15.53825647486</v>
       </c>
       <c r="G8" t="n">
-        <v>0.006493425944126177</v>
+        <v>0.5098892675341249</v>
       </c>
       <c r="H8" t="n">
-        <v>6.363293293955125e-05</v>
+        <v>0.003929722103890167</v>
       </c>
       <c r="I8" t="n">
-        <v>1.243291384815935</v>
+        <v>0.0001289541801814846</v>
       </c>
       <c r="J8" t="n">
-        <v>0.01051288534168879</v>
+        <v>1.460311260664919</v>
       </c>
       <c r="K8" t="n">
-        <v>9.893151436961653e-05</v>
+        <v>0.04805708251155821</v>
       </c>
       <c r="L8" t="n">
-        <v>0.01650793650793651</v>
+        <v>0.0005595649156774294</v>
       </c>
       <c r="M8" t="n">
-        <v>52.03173828125001</v>
+        <v>0.01</v>
       </c>
       <c r="N8" t="n">
-        <v>23.35091952012064</v>
+        <v>39.54034423828125</v>
       </c>
       <c r="O8" t="n">
-        <v>1.583734146407318e-10</v>
+        <v>33.73452550992971</v>
       </c>
       <c r="P8" t="n">
-        <v>3152.508980960771</v>
+        <v>4.926773925604347e-11</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3944.963974235252</v>
       </c>
     </row>
     <row r="9">
@@ -895,51 +921,54 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ACsb4rearSOAEwf1.mat</t>
+          <t>ACsb24rearSOAEwfA1.mat</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3954.034423828125</v>
+        <v>2177.545166015625</v>
       </c>
       <c r="E9" t="n">
-        <v>15.53825647486</v>
+        <v>2178</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5098892675341249</v>
+        <v>23.87533611430924</v>
       </c>
       <c r="G9" t="n">
-        <v>0.003929722103890167</v>
+        <v>0.199603620443464</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0001289541801814846</v>
+        <v>0.01096433565968014</v>
       </c>
       <c r="I9" t="n">
-        <v>1.460311260664919</v>
+        <v>9.166451449945803e-05</v>
       </c>
       <c r="J9" t="n">
-        <v>0.04805708251155821</v>
+        <v>1.229145680085068</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0005595649156774294</v>
+        <v>0.008954135430953924</v>
       </c>
       <c r="L9" t="n">
-        <v>0.01</v>
+        <v>0.0001070512298754903</v>
       </c>
       <c r="M9" t="n">
-        <v>39.54034423828125</v>
+        <v>0.02600907029478458</v>
       </c>
       <c r="N9" t="n">
-        <v>33.73452550992971</v>
+        <v>56.63592529296875</v>
       </c>
       <c r="O9" t="n">
-        <v>4.926773925604347e-11</v>
+        <v>14.21023832975533</v>
       </c>
       <c r="P9" t="n">
-        <v>3944.963974235252</v>
+        <v>9.650500119140539e-11</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>2175.246197569066</v>
       </c>
     </row>
     <row r="10">
@@ -957,43 +986,46 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1811.480712890625</v>
+        <v>3111.5478515625</v>
       </c>
       <c r="E10" t="n">
-        <v>29.52024959362215</v>
+        <v>3112</v>
       </c>
       <c r="F10" t="n">
-        <v>2.060378082277679</v>
+        <v>18.1369995145824</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01629619867523511</v>
+        <v>0.2432247810841414</v>
       </c>
       <c r="H10" t="n">
-        <v>0.001137399955525821</v>
+        <v>0.005828931573549382</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2163530574655104</v>
+        <v>7.816842056984703e-05</v>
       </c>
       <c r="J10" t="n">
-        <v>0.02005055343144353</v>
+        <v>1.360869933351719</v>
       </c>
       <c r="K10" t="n">
-        <v>8.616871130929551e-05</v>
+        <v>0.01761179210471739</v>
       </c>
       <c r="L10" t="n">
-        <v>0.04</v>
+        <v>0.0001563171901731081</v>
       </c>
       <c r="M10" t="n">
-        <v>72.459228515625</v>
+        <v>0.01551020408163265</v>
       </c>
       <c r="N10" t="n">
-        <v>47.13257191358234</v>
+        <v>48.2607421875</v>
       </c>
       <c r="O10" t="n">
-        <v>1.369598844786981e-11</v>
+        <v>24.17271670332591</v>
       </c>
       <c r="P10" t="n">
-        <v>1801.655626397607</v>
+        <v>7.06937906864068e-11</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3112.93841005744</v>
       </c>
     </row>
     <row r="11">
@@ -1011,43 +1043,46 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2177.545166015625</v>
+        <v>3477.6123046875</v>
       </c>
       <c r="E11" t="n">
-        <v>23.87533611430924</v>
+        <v>3478</v>
       </c>
       <c r="F11" t="n">
-        <v>0.199603620443464</v>
+        <v>21.11625766221708</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01096433565968014</v>
+        <v>0.3180059870534072</v>
       </c>
       <c r="H11" t="n">
-        <v>9.166451449945803e-05</v>
+        <v>0.006072056288090055</v>
       </c>
       <c r="I11" t="n">
-        <v>1.229145680085068</v>
+        <v>9.144377210328032e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>0.008954135430953924</v>
+        <v>1.279115198918998</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0001070512298754903</v>
+        <v>0.01665715461241262</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02600907029478458</v>
+        <v>0.0002044789298814027</v>
       </c>
       <c r="M11" t="n">
-        <v>56.63592529296875</v>
+        <v>0.01448979591836735</v>
       </c>
       <c r="N11" t="n">
-        <v>14.21023832975533</v>
+        <v>50.389892578125</v>
       </c>
       <c r="O11" t="n">
-        <v>9.650500119140539e-11</v>
+        <v>24.60793692397083</v>
       </c>
       <c r="P11" t="n">
-        <v>2175.246197569066</v>
+        <v>5.100088038041753e-11</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3478.017965968106</v>
       </c>
     </row>
     <row r="12">
@@ -1057,51 +1092,54 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ACsb24rearSOAEwfA1.mat</t>
+          <t>ACsb30learSOAEwfA2.mat</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3111.5478515625</v>
+        <v>1798.0224609375</v>
       </c>
       <c r="E12" t="n">
-        <v>18.1369995145824</v>
+        <v>1798</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2432247810841414</v>
+        <v>10.83138782180633</v>
       </c>
       <c r="G12" t="n">
-        <v>0.005828931573549382</v>
+        <v>0.1189343580154598</v>
       </c>
       <c r="H12" t="n">
-        <v>7.816842056984703e-05</v>
+        <v>0.006024055904262052</v>
       </c>
       <c r="I12" t="n">
-        <v>1.360869933351719</v>
+        <v>6.614731495258778e-05</v>
       </c>
       <c r="J12" t="n">
-        <v>0.01761179210471739</v>
+        <v>1.233487856175178</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0001563171901731081</v>
+        <v>0.01208949815066053</v>
       </c>
       <c r="L12" t="n">
-        <v>0.01551020408163265</v>
+        <v>0.0001152929336444951</v>
       </c>
       <c r="M12" t="n">
-        <v>48.2607421875</v>
+        <v>0.01650793650793651</v>
       </c>
       <c r="N12" t="n">
-        <v>24.17271670332591</v>
+        <v>29.681640625</v>
       </c>
       <c r="O12" t="n">
-        <v>7.06937906864068e-11</v>
+        <v>23.55275459339331</v>
       </c>
       <c r="P12" t="n">
-        <v>3112.93841005744</v>
+        <v>1.759269509509833e-11</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1793.479704400886</v>
       </c>
     </row>
     <row r="13">
@@ -1111,51 +1149,54 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ACsb24rearSOAEwfA1.mat</t>
+          <t>ACsb30learSOAEwfA2.mat</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3477.6123046875</v>
+        <v>2139.862060546875</v>
       </c>
       <c r="E13" t="n">
-        <v>21.11625766221708</v>
+        <v>2140</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3180059870534072</v>
+        <v>7.383225339650395</v>
       </c>
       <c r="G13" t="n">
-        <v>0.006072056288090055</v>
+        <v>0.3977289205921791</v>
       </c>
       <c r="H13" t="n">
-        <v>9.144377210328032e-05</v>
+        <v>0.003450327699049675</v>
       </c>
       <c r="I13" t="n">
-        <v>1.279115198918998</v>
+        <v>0.0001858666163231724</v>
       </c>
       <c r="J13" t="n">
-        <v>0.01665715461241262</v>
+        <v>1.418070862340206</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0002044789298814027</v>
+        <v>0.06976038352038443</v>
       </c>
       <c r="L13" t="n">
-        <v>0.01448979591836735</v>
+        <v>0.001307088889552022</v>
       </c>
       <c r="M13" t="n">
-        <v>50.389892578125</v>
+        <v>0.008004535147392289</v>
       </c>
       <c r="N13" t="n">
-        <v>24.60793692397083</v>
+        <v>17.12860107421875</v>
       </c>
       <c r="O13" t="n">
-        <v>5.100088038041753e-11</v>
+        <v>41.30265573954974</v>
       </c>
       <c r="P13" t="n">
-        <v>3478.017965968106</v>
+        <v>3.539373210432152e-12</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>2141.354446457694</v>
       </c>
     </row>
     <row r="14">
@@ -1173,43 +1214,46 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1798.0224609375</v>
+        <v>2417.10205078125</v>
       </c>
       <c r="E14" t="n">
-        <v>10.83138782180633</v>
+        <v>2417</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1189343580154598</v>
+        <v>7.685360244948903</v>
       </c>
       <c r="G14" t="n">
-        <v>0.006024055904262052</v>
+        <v>0.4288062054925163</v>
       </c>
       <c r="H14" t="n">
-        <v>6.614731495258778e-05</v>
+        <v>0.003179576237778152</v>
       </c>
       <c r="I14" t="n">
-        <v>1.233487856175178</v>
+        <v>0.0001774050894350607</v>
       </c>
       <c r="J14" t="n">
-        <v>0.01208949815066053</v>
+        <v>1.44421366723964</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0001152929336444951</v>
+        <v>0.07587432245996721</v>
       </c>
       <c r="L14" t="n">
-        <v>0.01650793650793651</v>
+        <v>0.00123986853948281</v>
       </c>
       <c r="M14" t="n">
-        <v>29.681640625</v>
+        <v>0.007505668934240363</v>
       </c>
       <c r="N14" t="n">
-        <v>23.55275459339331</v>
+        <v>18.1419677734375</v>
       </c>
       <c r="O14" t="n">
-        <v>1.759269509509833e-11</v>
+        <v>42.34817726778903</v>
       </c>
       <c r="P14" t="n">
-        <v>1793.479704400886</v>
+        <v>2.902234163120909e-12</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>2413.939743194736</v>
       </c>
     </row>
     <row r="15">
@@ -1227,151 +1271,160 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2139.862060546875</v>
+        <v>2783.16650390625</v>
       </c>
       <c r="E15" t="n">
-        <v>7.383225339650395</v>
+        <v>2783</v>
       </c>
       <c r="F15" t="n">
-        <v>0.3977289205921791</v>
+        <v>222580056.6111855</v>
       </c>
       <c r="G15" t="n">
-        <v>0.003450327699049675</v>
+        <v>212851825869879.1</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0001858666163231724</v>
+        <v>79973.67613428384</v>
       </c>
       <c r="I15" t="n">
-        <v>1.418070862340206</v>
+        <v>76478293904.13248</v>
       </c>
       <c r="J15" t="n">
-        <v>0.06976038352038443</v>
+        <v>0.01931650088908909</v>
       </c>
       <c r="K15" t="n">
-        <v>0.001307088889552022</v>
+        <v>0.004113185546243618</v>
       </c>
       <c r="L15" t="n">
-        <v>0.008004535147392289</v>
+        <v>2.729313132736339e-05</v>
       </c>
       <c r="M15" t="n">
-        <v>17.12860107421875</v>
+        <v>0.02498866213151927</v>
       </c>
       <c r="N15" t="n">
-        <v>41.30265573954974</v>
+        <v>69.547607421875</v>
       </c>
       <c r="O15" t="n">
-        <v>3.539373210432152e-12</v>
+        <v>46.27969260680279</v>
       </c>
       <c r="P15" t="n">
-        <v>2141.354446457694</v>
+        <v>3.577109007377321e-12</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2784.865043070137</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Anole</t>
+          <t>Tokay</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ACsb30learSOAEwfA2.mat</t>
+          <t>tokay_GG1rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2417.10205078125</v>
+        <v>1342.7734375</v>
       </c>
       <c r="E16" t="n">
-        <v>7.685360244948903</v>
+        <v>1343</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4288062054925163</v>
+        <v>4.460025553747603</v>
       </c>
       <c r="G16" t="n">
-        <v>0.003179576237778152</v>
+        <v>0.2083667218300633</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0001774050894350607</v>
+        <v>0.003321502666936397</v>
       </c>
       <c r="I16" t="n">
-        <v>1.44421366723964</v>
+        <v>0.0001551763804756254</v>
       </c>
       <c r="J16" t="n">
-        <v>0.07587432245996721</v>
+        <v>1.423530552657516</v>
       </c>
       <c r="K16" t="n">
-        <v>0.00123986853948281</v>
+        <v>0.06219363852230954</v>
       </c>
       <c r="L16" t="n">
-        <v>0.007505668934240363</v>
+        <v>0.0009635734659170579</v>
       </c>
       <c r="M16" t="n">
-        <v>18.1419677734375</v>
+        <v>0.008</v>
       </c>
       <c r="N16" t="n">
-        <v>42.34817726778903</v>
+        <v>10.7421875</v>
       </c>
       <c r="O16" t="n">
-        <v>2.902234163120909e-12</v>
+        <v>42.66633598035457</v>
       </c>
       <c r="P16" t="n">
-        <v>2413.939743194736</v>
+        <v>3.152433682764227e-11</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1345.558150501267</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Anole</t>
+          <t>Tokay</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ACsb30learSOAEwfA2.mat</t>
+          <t>tokay_GG1rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2783.16650390625</v>
+        <v>1779.1748046875</v>
       </c>
       <c r="E17" t="n">
-        <v>222580056.6111855</v>
+        <v>1779</v>
       </c>
       <c r="F17" t="n">
-        <v>212851825869879.1</v>
+        <v>8.448976852641636</v>
       </c>
       <c r="G17" t="n">
-        <v>79973.67613428384</v>
+        <v>0.1296501109855726</v>
       </c>
       <c r="H17" t="n">
-        <v>76478293904.13248</v>
+        <v>0.004748817727398991</v>
       </c>
       <c r="I17" t="n">
-        <v>0.01931650088908909</v>
+        <v>7.287092344382921e-05</v>
       </c>
       <c r="J17" t="n">
-        <v>0.004113185546243618</v>
+        <v>1.239216578257107</v>
       </c>
       <c r="K17" t="n">
-        <v>2.729313132736339e-05</v>
+        <v>0.01667045906770272</v>
       </c>
       <c r="L17" t="n">
-        <v>0.02498866213151927</v>
+        <v>0.0001916137841558003</v>
       </c>
       <c r="M17" t="n">
-        <v>69.547607421875</v>
+        <v>0.0135</v>
       </c>
       <c r="N17" t="n">
-        <v>46.27969260680279</v>
+        <v>24.01885986328125</v>
       </c>
       <c r="O17" t="n">
-        <v>3.577109007377321e-12</v>
+        <v>29.42202178338179</v>
       </c>
       <c r="P17" t="n">
-        <v>2784.865043070137</v>
+        <v>4.771729493735052e-11</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1782.379762773272</v>
       </c>
     </row>
     <row r="18">
@@ -1389,43 +1442,46 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1342.7734375</v>
+        <v>3649.90234375</v>
       </c>
       <c r="E18" t="n">
-        <v>4.460025553747603</v>
+        <v>3650</v>
       </c>
       <c r="F18" t="n">
-        <v>0.2083667218300633</v>
+        <v>12.83125968722967</v>
       </c>
       <c r="G18" t="n">
-        <v>0.003321502666936397</v>
+        <v>0.5629645986041236</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0001551763804756254</v>
+        <v>0.003515507670828946</v>
       </c>
       <c r="I18" t="n">
-        <v>1.423530552657516</v>
+        <v>0.0001542410030690629</v>
       </c>
       <c r="J18" t="n">
-        <v>0.06219363852230954</v>
+        <v>1.396707260296086</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0009635734659170579</v>
+        <v>0.05635726268570131</v>
       </c>
       <c r="L18" t="n">
-        <v>0.008</v>
+        <v>0.0009325137695151844</v>
       </c>
       <c r="M18" t="n">
-        <v>10.7421875</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>42.66633598035457</v>
+        <v>31.024169921875</v>
       </c>
       <c r="O18" t="n">
-        <v>3.152433682764227e-11</v>
+        <v>38.44768429616745</v>
       </c>
       <c r="P18" t="n">
-        <v>1345.558150501267</v>
+        <v>1.774343353631128e-11</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3644.432330447859</v>
       </c>
     </row>
     <row r="19">
@@ -1443,43 +1499,46 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1779.1748046875</v>
+        <v>4211.425781249999</v>
       </c>
       <c r="E19" t="n">
-        <v>8.448976852641636</v>
+        <v>4211</v>
       </c>
       <c r="F19" t="n">
-        <v>0.1296501109855726</v>
+        <v>29.45316993193493</v>
       </c>
       <c r="G19" t="n">
-        <v>0.004748817727398991</v>
+        <v>1.068493130930639</v>
       </c>
       <c r="H19" t="n">
-        <v>7.287092344382921e-05</v>
+        <v>0.006993633857461188</v>
       </c>
       <c r="I19" t="n">
-        <v>1.239216578257107</v>
+        <v>0.0002537129196690955</v>
       </c>
       <c r="J19" t="n">
-        <v>0.01667045906770272</v>
+        <v>1.054240455752225</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0001916137841558003</v>
+        <v>0.03288075129920257</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0135</v>
+        <v>0.00117551605348218</v>
       </c>
       <c r="M19" t="n">
-        <v>24.01885986328125</v>
+        <v>0.019</v>
       </c>
       <c r="N19" t="n">
-        <v>29.42202178338179</v>
+        <v>80.01708984374999</v>
       </c>
       <c r="O19" t="n">
-        <v>4.771729493735052e-11</v>
+        <v>23.01318201212892</v>
       </c>
       <c r="P19" t="n">
-        <v>1782.379762773272</v>
+        <v>2.192222132226324e-11</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>4210.422772491951</v>
       </c>
     </row>
     <row r="20">
@@ -1489,51 +1548,54 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tokay_GG1rearSOAEwf.mat</t>
+          <t>tokay_GG2rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3649.90234375</v>
+        <v>1364.1357421875</v>
       </c>
       <c r="E20" t="n">
-        <v>12.83125968722967</v>
+        <v>1364</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5629645986041236</v>
+        <v>4.324112552004121</v>
       </c>
       <c r="G20" t="n">
-        <v>0.003515507670828946</v>
+        <v>0.1804466842198701</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0001542410030690629</v>
+        <v>0.003169855035885259</v>
       </c>
       <c r="I20" t="n">
-        <v>1.396707260296086</v>
+        <v>0.000132279126365027</v>
       </c>
       <c r="J20" t="n">
-        <v>0.05635726268570131</v>
+        <v>1.406366121009048</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0009325137695151844</v>
+        <v>0.05546019479220759</v>
       </c>
       <c r="L20" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0006551646695073318</v>
       </c>
       <c r="M20" t="n">
-        <v>31.024169921875</v>
+        <v>0.0075</v>
       </c>
       <c r="N20" t="n">
-        <v>38.44768429616745</v>
+        <v>10.23101806640625</v>
       </c>
       <c r="O20" t="n">
-        <v>1.774343353631128e-11</v>
+        <v>42.21255991974764</v>
       </c>
       <c r="P20" t="n">
-        <v>3644.432330447859</v>
+        <v>1.71600307853262e-11</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1360.86966387402</v>
       </c>
     </row>
     <row r="21">
@@ -1543,51 +1605,54 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tokay_GG1rearSOAEwf.mat</t>
+          <t>tokay_GG2rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4211.425781249999</v>
+        <v>1776.123046875</v>
       </c>
       <c r="E21" t="n">
-        <v>29.45316993193493</v>
+        <v>1776</v>
       </c>
       <c r="F21" t="n">
-        <v>1.068493130930639</v>
+        <v>5.771388687597842</v>
       </c>
       <c r="G21" t="n">
-        <v>0.006993633857461188</v>
+        <v>0.2101942134629494</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0002537129196690955</v>
+        <v>0.003249430661773301</v>
       </c>
       <c r="I21" t="n">
-        <v>1.054240455752225</v>
+        <v>0.0001183443983978338</v>
       </c>
       <c r="J21" t="n">
-        <v>0.03288075129920257</v>
+        <v>1.412328663391503</v>
       </c>
       <c r="K21" t="n">
-        <v>0.00117551605348218</v>
+        <v>0.04939513644597964</v>
       </c>
       <c r="L21" t="n">
-        <v>0.019</v>
+        <v>0.0006169226326571957</v>
       </c>
       <c r="M21" t="n">
-        <v>80.01708984374999</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N21" t="n">
-        <v>23.01318201212892</v>
+        <v>15.0970458984375</v>
       </c>
       <c r="O21" t="n">
-        <v>2.192222132226324e-11</v>
+        <v>39.77002884196471</v>
       </c>
       <c r="P21" t="n">
-        <v>4210.422772491951</v>
+        <v>2.101229297986004e-11</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1777.323367602554</v>
       </c>
     </row>
     <row r="22">
@@ -1605,43 +1670,46 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1364.1357421875</v>
+        <v>3607.177734375</v>
       </c>
       <c r="E22" t="n">
-        <v>4.324112552004121</v>
+        <v>3607</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1804466842198701</v>
+        <v>19.88328931692195</v>
       </c>
       <c r="G22" t="n">
-        <v>0.003169855035885259</v>
+        <v>0.2461295240289038</v>
       </c>
       <c r="H22" t="n">
-        <v>0.000132279126365027</v>
+        <v>0.005512145721970378</v>
       </c>
       <c r="I22" t="n">
-        <v>1.406366121009048</v>
+        <v>6.823326771048325e-05</v>
       </c>
       <c r="J22" t="n">
-        <v>0.05546019479220759</v>
+        <v>1.246398345349658</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0006551646695073318</v>
+        <v>0.01417945958124356</v>
       </c>
       <c r="L22" t="n">
-        <v>0.0075</v>
+        <v>0.0001301261287241322</v>
       </c>
       <c r="M22" t="n">
-        <v>10.23101806640625</v>
+        <v>0.0155</v>
       </c>
       <c r="N22" t="n">
-        <v>42.21255991974764</v>
+        <v>55.91125488281249</v>
       </c>
       <c r="O22" t="n">
-        <v>1.71600307853262e-11</v>
+        <v>25.50541865779515</v>
       </c>
       <c r="P22" t="n">
-        <v>1360.86966387402</v>
+        <v>3.783068554544835e-11</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>3604.758004675124</v>
       </c>
     </row>
     <row r="23">
@@ -1659,43 +1727,46 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1776.123046875</v>
+        <v>4394.531249999999</v>
       </c>
       <c r="E23" t="n">
-        <v>5.771388687597842</v>
+        <v>4395</v>
       </c>
       <c r="F23" t="n">
-        <v>0.2101942134629494</v>
+        <v>15.63666789306943</v>
       </c>
       <c r="G23" t="n">
-        <v>0.003249430661773301</v>
+        <v>0.6139322808409924</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0001183443983978338</v>
+        <v>0.003558210649445134</v>
       </c>
       <c r="I23" t="n">
-        <v>1.412328663391503</v>
+        <v>0.0001397037012402614</v>
       </c>
       <c r="J23" t="n">
-        <v>0.04939513644597964</v>
+        <v>1.371835470709829</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0006169226326571957</v>
+        <v>0.04920085661051307</v>
       </c>
       <c r="L23" t="n">
+        <v>0.0007264618189268275</v>
+      </c>
+      <c r="M23" t="n">
         <v>0.008500000000000001</v>
       </c>
-      <c r="M23" t="n">
-        <v>15.0970458984375</v>
-      </c>
       <c r="N23" t="n">
-        <v>39.77002884196471</v>
+        <v>37.35351562499999</v>
       </c>
       <c r="O23" t="n">
-        <v>2.101229297986004e-11</v>
+        <v>39.16627633705617</v>
       </c>
       <c r="P23" t="n">
-        <v>1777.323367602554</v>
+        <v>9.845293129520055e-12</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>4390.472362905448</v>
       </c>
     </row>
     <row r="24">
@@ -1705,51 +1776,54 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tokay_GG2rearSOAEwf.mat</t>
+          <t>tokay_GG3rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3607.177734375</v>
+        <v>1257.32421875</v>
       </c>
       <c r="E24" t="n">
-        <v>19.88328931692195</v>
+        <v>1257</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2461295240289038</v>
+        <v>6.159950049409389</v>
       </c>
       <c r="G24" t="n">
-        <v>0.005512145721970378</v>
+        <v>0.2030486871761092</v>
       </c>
       <c r="H24" t="n">
-        <v>6.823326771048325e-05</v>
+        <v>0.004899253476190459</v>
       </c>
       <c r="I24" t="n">
-        <v>1.246398345349658</v>
+        <v>0.0001614927034317172</v>
       </c>
       <c r="J24" t="n">
-        <v>0.01417945958124356</v>
+        <v>1.177873109107223</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0001301261287241322</v>
+        <v>0.03442875031901588</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0155</v>
+        <v>0.0009265966075376635</v>
       </c>
       <c r="M24" t="n">
-        <v>55.91125488281249</v>
+        <v>0.016</v>
       </c>
       <c r="N24" t="n">
-        <v>25.50541865779515</v>
+        <v>20.1171875</v>
       </c>
       <c r="O24" t="n">
-        <v>3.783068554544835e-11</v>
+        <v>26.78638101426216</v>
       </c>
       <c r="P24" t="n">
-        <v>3604.758004675124</v>
+        <v>2.689083012062509e-11</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>1256.959658401852</v>
       </c>
     </row>
     <row r="25">
@@ -1759,51 +1833,54 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tokay_GG2rearSOAEwf.mat</t>
+          <t>tokay_GG3rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4394.531249999999</v>
+        <v>2578.7353515625</v>
       </c>
       <c r="E25" t="n">
-        <v>15.63666789306943</v>
+        <v>2579</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6139322808409924</v>
+        <v>7.628241318316572</v>
       </c>
       <c r="G25" t="n">
-        <v>0.003558210649445134</v>
+        <v>0.4484300526328838</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0001397037012402614</v>
+        <v>0.002958132680693461</v>
       </c>
       <c r="I25" t="n">
-        <v>1.371835470709829</v>
+        <v>0.0001738953368600514</v>
       </c>
       <c r="J25" t="n">
-        <v>0.04920085661051307</v>
+        <v>1.470670867844325</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0007264618189268275</v>
+        <v>0.08363272398763569</v>
       </c>
       <c r="L25" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.001203545420941607</v>
       </c>
       <c r="M25" t="n">
-        <v>37.35351562499999</v>
+        <v>0.007</v>
       </c>
       <c r="N25" t="n">
-        <v>39.16627633705617</v>
+        <v>18.0511474609375</v>
       </c>
       <c r="O25" t="n">
-        <v>9.845293129520055e-12</v>
+        <v>43.57426733179351</v>
       </c>
       <c r="P25" t="n">
-        <v>4390.472362905448</v>
+        <v>8.757415282657275e-12</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>2572.886713729026</v>
       </c>
     </row>
     <row r="26">
@@ -1821,43 +1898,46 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1257.32421875</v>
+        <v>3567.5048828125</v>
       </c>
       <c r="E26" t="n">
-        <v>6.159950049409389</v>
+        <v>3568</v>
       </c>
       <c r="F26" t="n">
-        <v>0.2030486871761092</v>
+        <v>16.97342499260922</v>
       </c>
       <c r="G26" t="n">
-        <v>0.004899253476190459</v>
+        <v>0.1965609959724034</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0001614927034317172</v>
+        <v>0.004757786057808547</v>
       </c>
       <c r="I26" t="n">
-        <v>1.177873109107223</v>
+        <v>5.509761091551509e-05</v>
       </c>
       <c r="J26" t="n">
-        <v>0.03442875031901588</v>
+        <v>1.28980127584304</v>
       </c>
       <c r="K26" t="n">
-        <v>0.0009265966075376635</v>
+        <v>0.01426855130046424</v>
       </c>
       <c r="L26" t="n">
-        <v>0.016</v>
+        <v>8.938702772880043e-05</v>
       </c>
       <c r="M26" t="n">
-        <v>20.1171875</v>
+        <v>0.013</v>
       </c>
       <c r="N26" t="n">
-        <v>26.78638101426216</v>
+        <v>46.37756347656249</v>
       </c>
       <c r="O26" t="n">
-        <v>2.689083012062509e-11</v>
+        <v>28.54024203390058</v>
       </c>
       <c r="P26" t="n">
-        <v>1256.959658401852</v>
+        <v>1.757871137128941e-11</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>3559.172952959399</v>
       </c>
     </row>
     <row r="27">
@@ -1867,51 +1947,54 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1837.158203125</v>
+        <v>1251.220703125</v>
       </c>
       <c r="E27" t="n">
-        <v>5.454804620331305</v>
+        <v>1251</v>
       </c>
       <c r="F27" t="n">
-        <v>0.3022607368537311</v>
+        <v>6.968943536799011</v>
       </c>
       <c r="G27" t="n">
-        <v>0.002969153451810901</v>
+        <v>0.2097396321474185</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0001645262429439047</v>
+        <v>0.005569715653995854</v>
       </c>
       <c r="I27" t="n">
-        <v>1.462355788436553</v>
+        <v>0.0001676280064928442</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0782078009490524</v>
+        <v>1.128208953686543</v>
       </c>
       <c r="K27" t="n">
-        <v>0.001060205099203275</v>
+        <v>0.02890609544874574</v>
       </c>
       <c r="L27" t="n">
-        <v>0.007</v>
+        <v>0.0008208035871424071</v>
       </c>
       <c r="M27" t="n">
-        <v>12.860107421875</v>
+        <v>0.0165</v>
       </c>
       <c r="N27" t="n">
-        <v>45.09541545147014</v>
+        <v>20.6451416015625</v>
       </c>
       <c r="O27" t="n">
-        <v>1.609361979514102e-11</v>
+        <v>24.92820201618651</v>
       </c>
       <c r="P27" t="n">
-        <v>1839.488305202574</v>
+        <v>3.834120878250849e-11</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1251.287838447055</v>
       </c>
     </row>
     <row r="28">
@@ -1921,51 +2004,54 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2578.7353515625</v>
+        <v>2590.9423828125</v>
       </c>
       <c r="E28" t="n">
-        <v>7.628241318316572</v>
+        <v>2591</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4484300526328838</v>
+        <v>10.98963182361519</v>
       </c>
       <c r="G28" t="n">
-        <v>0.002958132680693461</v>
+        <v>0.3092448683018977</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0001738953368600514</v>
+        <v>0.004241557780874234</v>
       </c>
       <c r="I28" t="n">
-        <v>1.470670867844325</v>
+        <v>0.0001193561347999598</v>
       </c>
       <c r="J28" t="n">
-        <v>0.08363272398763569</v>
+        <v>1.32768769695136</v>
       </c>
       <c r="K28" t="n">
-        <v>0.001203545420941607</v>
+        <v>0.03276803607911022</v>
       </c>
       <c r="L28" t="n">
-        <v>0.007</v>
+        <v>0.0005233411782563589</v>
       </c>
       <c r="M28" t="n">
-        <v>18.0511474609375</v>
+        <v>0.0105</v>
       </c>
       <c r="N28" t="n">
-        <v>43.57426733179351</v>
+        <v>27.20489501953125</v>
       </c>
       <c r="O28" t="n">
-        <v>8.757415282657275e-12</v>
+        <v>31.27955333718139</v>
       </c>
       <c r="P28" t="n">
-        <v>2572.886713729026</v>
+        <v>2.053361281504691e-11</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>2591.805130181283</v>
       </c>
     </row>
     <row r="29">
@@ -1975,51 +2061,54 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3567.5048828125</v>
+        <v>3216.552734375</v>
       </c>
       <c r="E29" t="n">
-        <v>16.97342499260922</v>
+        <v>3217</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1965609959724034</v>
+        <v>10.18586891539348</v>
       </c>
       <c r="G29" t="n">
-        <v>0.004757786057808547</v>
+        <v>0.5054175690872295</v>
       </c>
       <c r="H29" t="n">
-        <v>5.509761091551509e-05</v>
+        <v>0.003166703535290452</v>
       </c>
       <c r="I29" t="n">
-        <v>1.28980127584304</v>
+        <v>0.0001571301983287508</v>
       </c>
       <c r="J29" t="n">
-        <v>0.01426855130046424</v>
+        <v>1.439482130378261</v>
       </c>
       <c r="K29" t="n">
-        <v>8.938702772880043e-05</v>
+        <v>0.06753790519768502</v>
       </c>
       <c r="L29" t="n">
-        <v>0.013</v>
+        <v>0.0009697510280074862</v>
       </c>
       <c r="M29" t="n">
-        <v>46.37756347656249</v>
+        <v>0.0075</v>
       </c>
       <c r="N29" t="n">
-        <v>28.54024203390058</v>
+        <v>24.1241455078125</v>
       </c>
       <c r="O29" t="n">
-        <v>1.757871137128941e-11</v>
+        <v>40.60474868382574</v>
       </c>
       <c r="P29" t="n">
-        <v>3559.172952959399</v>
+        <v>5.761462717113044e-12</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>3220.389925054321</v>
       </c>
     </row>
     <row r="30">
@@ -2037,205 +2126,217 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1251.220703125</v>
+        <v>3582.763671875</v>
       </c>
       <c r="E30" t="n">
-        <v>6.968943536799011</v>
+        <v>3583</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2097396321474185</v>
+        <v>14.31809874100298</v>
       </c>
       <c r="G30" t="n">
-        <v>0.005569715653995854</v>
+        <v>0.4232403169228528</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0001676280064928442</v>
+        <v>0.003996383812139571</v>
       </c>
       <c r="I30" t="n">
-        <v>1.128208953686543</v>
+        <v>0.0001181323569414654</v>
       </c>
       <c r="J30" t="n">
-        <v>0.02890609544874574</v>
+        <v>1.348669525122197</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0008208035871424071</v>
+        <v>0.03562087547215192</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0165</v>
+        <v>0.0005381260333174574</v>
       </c>
       <c r="M30" t="n">
-        <v>20.6451416015625</v>
+        <v>0.01</v>
       </c>
       <c r="N30" t="n">
-        <v>24.92820201618651</v>
+        <v>35.82763671874999</v>
       </c>
       <c r="O30" t="n">
-        <v>3.834120878250849e-11</v>
+        <v>33.43948673382051</v>
       </c>
       <c r="P30" t="n">
-        <v>1251.287838447055</v>
+        <v>1.950103839622597e-11</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>3584.025592853023</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2590.9423828125</v>
+        <v>4350.5859375</v>
       </c>
       <c r="E31" t="n">
-        <v>10.98963182361519</v>
+        <v>4351</v>
       </c>
       <c r="F31" t="n">
-        <v>0.3092448683018977</v>
+        <v>6.200537234175052</v>
       </c>
       <c r="G31" t="n">
-        <v>0.004241557780874234</v>
+        <v>0.503620119972046</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0001193561347999598</v>
+        <v>0.001425218883904658</v>
       </c>
       <c r="I31" t="n">
-        <v>1.32768769695136</v>
+        <v>0.000115759147665853</v>
       </c>
       <c r="J31" t="n">
-        <v>0.03276803607911022</v>
+        <v>1.556984711577556</v>
       </c>
       <c r="K31" t="n">
-        <v>0.0005233411782563589</v>
+        <v>0.1342492179820402</v>
       </c>
       <c r="L31" t="n">
-        <v>0.0105</v>
+        <v>0.0006445582041643389</v>
       </c>
       <c r="M31" t="n">
-        <v>27.20489501953125</v>
+        <v>0.0035</v>
       </c>
       <c r="N31" t="n">
-        <v>31.27955333718139</v>
+        <v>15.22705078125</v>
       </c>
       <c r="O31" t="n">
-        <v>2.053361281504691e-11</v>
+        <v>87.64883889212321</v>
       </c>
       <c r="P31" t="n">
-        <v>2591.805130181283</v>
+        <v>1.806475847363449e-13</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>4347.72734487957</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3216.552734375</v>
+        <v>7453.125</v>
       </c>
       <c r="E32" t="n">
-        <v>10.18586891539348</v>
+        <v>7453</v>
       </c>
       <c r="F32" t="n">
-        <v>0.5054175690872295</v>
+        <v>13.52609931227873</v>
       </c>
       <c r="G32" t="n">
-        <v>0.003166703535290452</v>
+        <v>0.3830227078285064</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0001571301983287508</v>
+        <v>0.001814822549236559</v>
       </c>
       <c r="I32" t="n">
-        <v>1.439482130378261</v>
+        <v>5.139088742353127e-05</v>
       </c>
       <c r="J32" t="n">
-        <v>0.06753790519768502</v>
+        <v>1.387782360319679</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0009697510280074862</v>
+        <v>0.03911632563287751</v>
       </c>
       <c r="L32" t="n">
-        <v>0.0075</v>
+        <v>0.0001643147067307164</v>
       </c>
       <c r="M32" t="n">
-        <v>24.1241455078125</v>
+        <v>0.005</v>
       </c>
       <c r="N32" t="n">
-        <v>40.60474868382574</v>
+        <v>37.265625</v>
       </c>
       <c r="O32" t="n">
-        <v>5.761462717113044e-12</v>
+        <v>68.22161768748448</v>
       </c>
       <c r="P32" t="n">
-        <v>3220.389925054321</v>
+        <v>6.30085870083755e-13</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>7456.907112586428</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3582.763671875</v>
+        <v>8452.1484375</v>
       </c>
       <c r="E33" t="n">
-        <v>14.31809874100298</v>
+        <v>8452</v>
       </c>
       <c r="F33" t="n">
-        <v>0.4232403169228528</v>
+        <v>17.85863955129348</v>
       </c>
       <c r="G33" t="n">
-        <v>0.003996383812139571</v>
+        <v>0.7019742548644242</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0001181323569414654</v>
+        <v>0.002112911253671233</v>
       </c>
       <c r="I33" t="n">
-        <v>1.348669525122197</v>
+        <v>8.30527599053923e-05</v>
       </c>
       <c r="J33" t="n">
-        <v>0.03562087547215192</v>
+        <v>1.370490614141937</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0005381260333174574</v>
+        <v>0.05037830177731586</v>
       </c>
       <c r="L33" t="n">
-        <v>0.01</v>
+        <v>0.0004109910990382773</v>
       </c>
       <c r="M33" t="n">
-        <v>35.82763671874999</v>
+        <v>0.0055</v>
       </c>
       <c r="N33" t="n">
-        <v>33.43948673382051</v>
+        <v>46.48681640625</v>
       </c>
       <c r="O33" t="n">
-        <v>1.950103839622597e-11</v>
+        <v>60.09398519868756</v>
       </c>
       <c r="P33" t="n">
-        <v>3584.025592853023</v>
+        <v>1.784690547665494e-12</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>8445.060419516562</v>
       </c>
     </row>
     <row r="34">
@@ -2253,43 +2354,46 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>4350.5859375</v>
+        <v>9026.3671875</v>
       </c>
       <c r="E34" t="n">
-        <v>6.200537234175052</v>
+        <v>9026</v>
       </c>
       <c r="F34" t="n">
-        <v>0.503620119972046</v>
+        <v>25.26965690636864</v>
       </c>
       <c r="G34" t="n">
-        <v>0.001425218883904658</v>
+        <v>0.4451316147322679</v>
       </c>
       <c r="H34" t="n">
-        <v>0.000115759147665853</v>
+        <v>0.002799537885115383</v>
       </c>
       <c r="I34" t="n">
-        <v>1.556984711577556</v>
+        <v>4.931459195995264e-05</v>
       </c>
       <c r="J34" t="n">
-        <v>0.1342492179820402</v>
+        <v>1.21040516136573</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0006445582041643389</v>
+        <v>0.01878987637047191</v>
       </c>
       <c r="L34" t="n">
-        <v>0.0035</v>
+        <v>0.0001291071634474768</v>
       </c>
       <c r="M34" t="n">
-        <v>15.22705078125</v>
+        <v>0.008</v>
       </c>
       <c r="N34" t="n">
-        <v>87.64883889212321</v>
+        <v>72.2109375</v>
       </c>
       <c r="O34" t="n">
-        <v>1.806475847363449e-13</v>
+        <v>48.17177549386727</v>
       </c>
       <c r="P34" t="n">
-        <v>4347.72734487957</v>
+        <v>2.045822095595467e-12</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>9030.795774783386</v>
       </c>
     </row>
     <row r="35">
@@ -2299,51 +2403,54 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7453.125</v>
+        <v>6837.890625</v>
       </c>
       <c r="E35" t="n">
-        <v>13.52609931227873</v>
+        <v>6838</v>
       </c>
       <c r="F35" t="n">
-        <v>0.3830227078285064</v>
+        <v>10.5977698983937</v>
       </c>
       <c r="G35" t="n">
-        <v>0.001814822549236559</v>
+        <v>0.6331896030148532</v>
       </c>
       <c r="H35" t="n">
-        <v>5.139088742353127e-05</v>
+        <v>0.00154985952241576</v>
       </c>
       <c r="I35" t="n">
-        <v>1.387782360319679</v>
+        <v>9.260013617355179e-05</v>
       </c>
       <c r="J35" t="n">
-        <v>0.03911632563287751</v>
+        <v>1.489588780119523</v>
       </c>
       <c r="K35" t="n">
-        <v>0.0001643147067307164</v>
+        <v>0.09255996511278757</v>
       </c>
       <c r="L35" t="n">
-        <v>0.005</v>
+        <v>0.0004790623519389627</v>
       </c>
       <c r="M35" t="n">
-        <v>37.265625</v>
+        <v>0.004</v>
       </c>
       <c r="N35" t="n">
-        <v>68.22161768748448</v>
+        <v>27.3515625</v>
       </c>
       <c r="O35" t="n">
-        <v>6.30085870083755e-13</v>
+        <v>76.67818748697763</v>
       </c>
       <c r="P35" t="n">
-        <v>7456.907112586428</v>
+        <v>3.885635794226587e-13</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>6840.757442741772</v>
       </c>
     </row>
     <row r="36">
@@ -2353,51 +2460,54 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8452.1484375</v>
+        <v>7901.3671875</v>
       </c>
       <c r="E36" t="n">
-        <v>17.85863955129348</v>
+        <v>7901</v>
       </c>
       <c r="F36" t="n">
-        <v>0.7019742548644242</v>
+        <v>19.12436303910451</v>
       </c>
       <c r="G36" t="n">
-        <v>0.002112911253671233</v>
+        <v>1.032548472683028</v>
       </c>
       <c r="H36" t="n">
-        <v>8.30527599053923e-05</v>
+        <v>0.002420386571751701</v>
       </c>
       <c r="I36" t="n">
-        <v>1.370490614141937</v>
+        <v>0.0001306797226581906</v>
       </c>
       <c r="J36" t="n">
-        <v>0.05037830177731586</v>
+        <v>1.174421851631025</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0004109910990382773</v>
+        <v>0.05926269821551847</v>
       </c>
       <c r="L36" t="n">
-        <v>0.0055</v>
+        <v>0.0009800467979355896</v>
       </c>
       <c r="M36" t="n">
-        <v>46.48681640625</v>
+        <v>0.008</v>
       </c>
       <c r="N36" t="n">
-        <v>60.09398519868756</v>
+        <v>63.2109375</v>
       </c>
       <c r="O36" t="n">
-        <v>1.784690547665494e-12</v>
+        <v>51.7303391195944</v>
       </c>
       <c r="P36" t="n">
-        <v>8445.060419516562</v>
+        <v>6.977991565512491e-13</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>7901.190467312519</v>
       </c>
     </row>
     <row r="37">
@@ -2407,51 +2517,54 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9026.3671875</v>
+        <v>8835.9375</v>
       </c>
       <c r="E37" t="n">
-        <v>25.26965690636864</v>
+        <v>8836</v>
       </c>
       <c r="F37" t="n">
-        <v>0.4451316147322679</v>
+        <v>22.98015480698477</v>
       </c>
       <c r="G37" t="n">
-        <v>0.002799537885115383</v>
+        <v>0.678522834599649</v>
       </c>
       <c r="H37" t="n">
-        <v>4.931459195995264e-05</v>
+        <v>0.002600760225724183</v>
       </c>
       <c r="I37" t="n">
-        <v>1.21040516136573</v>
+        <v>7.679126686892579e-05</v>
       </c>
       <c r="J37" t="n">
-        <v>0.01878987637047191</v>
+        <v>1.215681358694547</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0001291071634474768</v>
+        <v>0.0326037303704333</v>
       </c>
       <c r="L37" t="n">
+        <v>0.0003405400154561213</v>
+      </c>
+      <c r="M37" t="n">
         <v>0.008</v>
       </c>
-      <c r="M37" t="n">
-        <v>72.2109375</v>
-      </c>
       <c r="N37" t="n">
-        <v>48.17177549386727</v>
+        <v>70.6875</v>
       </c>
       <c r="O37" t="n">
-        <v>2.045822095595467e-12</v>
+        <v>49.42569815474504</v>
       </c>
       <c r="P37" t="n">
-        <v>9030.795774783386</v>
+        <v>1.292541591210098e-12</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>8845.361149512852</v>
       </c>
     </row>
     <row r="38">
@@ -2469,43 +2582,46 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>6837.890625</v>
+        <v>9257.8125</v>
       </c>
       <c r="E38" t="n">
-        <v>10.5977698983937</v>
+        <v>9258</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6331896030148532</v>
+        <v>57.96893269989882</v>
       </c>
       <c r="G38" t="n">
-        <v>0.00154985952241576</v>
+        <v>6.118874950467526</v>
       </c>
       <c r="H38" t="n">
-        <v>9.260013617355179e-05</v>
+        <v>0.006261623110200042</v>
       </c>
       <c r="I38" t="n">
-        <v>1.489588780119523</v>
+        <v>0.0006609417668015556</v>
       </c>
       <c r="J38" t="n">
-        <v>0.09255996511278757</v>
+        <v>0.06859142883780221</v>
       </c>
       <c r="K38" t="n">
-        <v>0.0004790623519389627</v>
+        <v>0.009411778969351539</v>
       </c>
       <c r="L38" t="n">
-        <v>0.004</v>
+        <v>6.093241765296857e-06</v>
       </c>
       <c r="M38" t="n">
-        <v>27.3515625</v>
+        <v>0.0145</v>
       </c>
       <c r="N38" t="n">
-        <v>76.67818748697763</v>
+        <v>134.23828125</v>
       </c>
       <c r="O38" t="n">
-        <v>3.885635794226587e-13</v>
+        <v>89.73515677713675</v>
       </c>
       <c r="P38" t="n">
-        <v>6840.757442741772</v>
+        <v>7.664901288177202e-13</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>9253.893064877439</v>
       </c>
     </row>
     <row r="39">
@@ -2515,51 +2631,54 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7901.3671875</v>
+        <v>5625.54931640625</v>
       </c>
       <c r="E39" t="n">
-        <v>19.12436303910451</v>
+        <v>5626</v>
       </c>
       <c r="F39" t="n">
-        <v>1.032548472683028</v>
+        <v>13.7025908628672</v>
       </c>
       <c r="G39" t="n">
-        <v>0.002420386571751701</v>
+        <v>1.23349974496892</v>
       </c>
       <c r="H39" t="n">
-        <v>0.0001306797226581906</v>
+        <v>0.002435778284425524</v>
       </c>
       <c r="I39" t="n">
-        <v>1.174421851631025</v>
+        <v>0.0002192674307149995</v>
       </c>
       <c r="J39" t="n">
-        <v>0.05926269821551847</v>
+        <v>1.123193040757176</v>
       </c>
       <c r="K39" t="n">
-        <v>0.0009800467979355896</v>
+        <v>0.09542756147256611</v>
       </c>
       <c r="L39" t="n">
-        <v>0.008</v>
+        <v>0.002768955551456496</v>
       </c>
       <c r="M39" t="n">
-        <v>63.2109375</v>
+        <v>0.009501133786848073</v>
       </c>
       <c r="N39" t="n">
-        <v>51.7303391195944</v>
+        <v>53.4490966796875</v>
       </c>
       <c r="O39" t="n">
-        <v>6.977991565512491e-13</v>
+        <v>55.38194222549402</v>
       </c>
       <c r="P39" t="n">
-        <v>7901.190467312519</v>
+        <v>7.975997509325952e-11</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>5623.316734238025</v>
       </c>
     </row>
     <row r="40">
@@ -2569,51 +2688,54 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8835.9375</v>
+        <v>8096.484375</v>
       </c>
       <c r="E40" t="n">
-        <v>22.98015480698477</v>
+        <v>8096</v>
       </c>
       <c r="F40" t="n">
-        <v>0.678522834599649</v>
+        <v>16.61126643733448</v>
       </c>
       <c r="G40" t="n">
-        <v>0.002600760225724183</v>
+        <v>0.3634184788855256</v>
       </c>
       <c r="H40" t="n">
-        <v>7.679126686892579e-05</v>
+        <v>0.002051664113454734</v>
       </c>
       <c r="I40" t="n">
-        <v>1.215681358694547</v>
+        <v>4.488596062850125e-05</v>
       </c>
       <c r="J40" t="n">
-        <v>0.0326037303704333</v>
+        <v>1.326748703747682</v>
       </c>
       <c r="K40" t="n">
-        <v>0.0003405400154561213</v>
+        <v>0.0279915396108054</v>
       </c>
       <c r="L40" t="n">
-        <v>0.008</v>
+        <v>0.0001302866375262261</v>
       </c>
       <c r="M40" t="n">
-        <v>70.6875</v>
+        <v>0.00600907029478458</v>
       </c>
       <c r="N40" t="n">
-        <v>49.42569815474504</v>
+        <v>48.65234375</v>
       </c>
       <c r="O40" t="n">
-        <v>1.292541591210098e-12</v>
+        <v>58.78366132431848</v>
       </c>
       <c r="P40" t="n">
-        <v>8845.361149512852</v>
+        <v>1.299537582437962e-10</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>8098.586383255675</v>
       </c>
     </row>
     <row r="41">
@@ -2623,51 +2745,54 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9257.8125</v>
+        <v>8489.46533203125</v>
       </c>
       <c r="E41" t="n">
-        <v>57.96893269989882</v>
+        <v>8489</v>
       </c>
       <c r="F41" t="n">
-        <v>6.118874950467526</v>
+        <v>54.8932366315176</v>
       </c>
       <c r="G41" t="n">
-        <v>0.006261623110200042</v>
+        <v>2.019460731392774</v>
       </c>
       <c r="H41" t="n">
-        <v>0.0006609417668015556</v>
+        <v>0.006466041674544828</v>
       </c>
       <c r="I41" t="n">
-        <v>0.06859142883780221</v>
+        <v>0.0002378784354973723</v>
       </c>
       <c r="J41" t="n">
-        <v>0.009411778969351539</v>
+        <v>0.842857790203811</v>
       </c>
       <c r="K41" t="n">
-        <v>6.093241765296857e-06</v>
+        <v>0.02437092987453587</v>
       </c>
       <c r="L41" t="n">
-        <v>0.0145</v>
+        <v>0.0006957767539891147</v>
       </c>
       <c r="M41" t="n">
-        <v>134.23828125</v>
+        <v>0.01501133786848073</v>
       </c>
       <c r="N41" t="n">
-        <v>89.73515677713675</v>
+        <v>127.438232421875</v>
       </c>
       <c r="O41" t="n">
-        <v>7.664901288177202e-13</v>
+        <v>24.82765613524692</v>
       </c>
       <c r="P41" t="n">
-        <v>9253.893064877439</v>
+        <v>3.706405454296643e-10</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>8486.907248855707</v>
       </c>
     </row>
     <row r="42">
@@ -2685,43 +2810,46 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5625.54931640625</v>
+        <v>9864.898681640625</v>
       </c>
       <c r="E42" t="n">
-        <v>13.7025908628672</v>
+        <v>9865</v>
       </c>
       <c r="F42" t="n">
-        <v>1.23349974496892</v>
+        <v>17.55744318502499</v>
       </c>
       <c r="G42" t="n">
-        <v>0.002435778284425524</v>
+        <v>0.7706878262572214</v>
       </c>
       <c r="H42" t="n">
-        <v>0.0002192674307149995</v>
+        <v>0.001779789509414913</v>
       </c>
       <c r="I42" t="n">
-        <v>1.123193040757176</v>
+        <v>7.812425156393484e-05</v>
       </c>
       <c r="J42" t="n">
-        <v>0.09542756147256611</v>
+        <v>1.430540075178475</v>
       </c>
       <c r="K42" t="n">
-        <v>0.002768955551456496</v>
+        <v>0.06310040276667497</v>
       </c>
       <c r="L42" t="n">
-        <v>0.009501133786848073</v>
+        <v>0.0004119904486747436</v>
       </c>
       <c r="M42" t="n">
-        <v>53.4490966796875</v>
+        <v>0.005011337868480726</v>
       </c>
       <c r="N42" t="n">
-        <v>55.38194222549402</v>
+        <v>49.43634033203125</v>
       </c>
       <c r="O42" t="n">
-        <v>7.975997509325952e-11</v>
+        <v>63.90181081181339</v>
       </c>
       <c r="P42" t="n">
-        <v>5623.316734238025</v>
+        <v>9.69195629278402e-11</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>9856.932898275971</v>
       </c>
     </row>
     <row r="43">
@@ -2731,51 +2859,54 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>8096.484375</v>
+        <v>4944.561767578125</v>
       </c>
       <c r="E43" t="n">
-        <v>16.61126643733448</v>
+        <v>4945</v>
       </c>
       <c r="F43" t="n">
-        <v>0.3634184788855256</v>
+        <v>7.915838219591966</v>
       </c>
       <c r="G43" t="n">
-        <v>0.002051664113454734</v>
+        <v>0.3683099505358468</v>
       </c>
       <c r="H43" t="n">
-        <v>4.488596062850125e-05</v>
+        <v>0.001600918057389177</v>
       </c>
       <c r="I43" t="n">
-        <v>1.326748703747682</v>
+        <v>7.448788544838973e-05</v>
       </c>
       <c r="J43" t="n">
-        <v>0.0279915396108054</v>
+        <v>1.484261017007512</v>
       </c>
       <c r="K43" t="n">
-        <v>0.0001302866375262261</v>
+        <v>0.07218371225140059</v>
       </c>
       <c r="L43" t="n">
-        <v>0.00600907029478458</v>
+        <v>0.000374978253079178</v>
       </c>
       <c r="M43" t="n">
-        <v>48.65234375</v>
+        <v>0.004489795918367347</v>
       </c>
       <c r="N43" t="n">
-        <v>58.78366132431848</v>
+        <v>22.2000732421875</v>
       </c>
       <c r="O43" t="n">
-        <v>1.299537582437962e-10</v>
+        <v>73.82638021620554</v>
       </c>
       <c r="P43" t="n">
-        <v>8098.586383255675</v>
+        <v>4.610246676062042e-11</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>4954.457814883755</v>
       </c>
     </row>
     <row r="44">
@@ -2785,51 +2916,54 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8489.46533203125</v>
+        <v>5768.206787109375</v>
       </c>
       <c r="E44" t="n">
-        <v>54.8932366315176</v>
+        <v>5768</v>
       </c>
       <c r="F44" t="n">
-        <v>2.019460731392774</v>
+        <v>31.92543080459712</v>
       </c>
       <c r="G44" t="n">
-        <v>0.006466041674544828</v>
+        <v>2.402161376318801</v>
       </c>
       <c r="H44" t="n">
-        <v>0.0002378784354973723</v>
+        <v>0.005534723698870014</v>
       </c>
       <c r="I44" t="n">
-        <v>0.842857790203811</v>
+        <v>0.0004164485541134001</v>
       </c>
       <c r="J44" t="n">
-        <v>0.02437092987453587</v>
+        <v>0.8224411756415669</v>
       </c>
       <c r="K44" t="n">
-        <v>0.0006957767539891147</v>
+        <v>0.04763836043567797</v>
       </c>
       <c r="L44" t="n">
+        <v>0.003106225350922567</v>
+      </c>
+      <c r="M44" t="n">
         <v>0.01501133786848073</v>
       </c>
-      <c r="M44" t="n">
-        <v>127.438232421875</v>
-      </c>
       <c r="N44" t="n">
-        <v>24.82765613524692</v>
+        <v>86.5885009765625</v>
       </c>
       <c r="O44" t="n">
-        <v>3.706405454296643e-10</v>
+        <v>26.63568621305765</v>
       </c>
       <c r="P44" t="n">
-        <v>8486.907248855707</v>
+        <v>2.037326814883841e-10</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>5766.206632270292</v>
       </c>
     </row>
     <row r="45">
@@ -2839,51 +2973,54 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>9864.898681640625</v>
+        <v>7184.014892578125</v>
       </c>
       <c r="E45" t="n">
-        <v>17.55744318502499</v>
+        <v>7184</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7706878262572214</v>
+        <v>236.2795024146108</v>
       </c>
       <c r="G45" t="n">
-        <v>0.001779789509414913</v>
+        <v>2.40489004794071</v>
       </c>
       <c r="H45" t="n">
-        <v>7.812425156393484e-05</v>
+        <v>0.03288961756729004</v>
       </c>
       <c r="I45" t="n">
-        <v>1.430540075178475</v>
+        <v>0.0003347557158358936</v>
       </c>
       <c r="J45" t="n">
-        <v>0.06310040276667497</v>
+        <v>0.9717468225374449</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0004119904486747436</v>
+        <v>0.006551192460712446</v>
       </c>
       <c r="L45" t="n">
-        <v>0.005011337868480726</v>
+        <v>0.0004427735154623166</v>
       </c>
       <c r="M45" t="n">
-        <v>49.43634033203125</v>
+        <v>0.06448979591836734</v>
       </c>
       <c r="N45" t="n">
-        <v>63.90181081181339</v>
+        <v>463.295654296875</v>
       </c>
       <c r="O45" t="n">
-        <v>9.69195629278402e-11</v>
+        <v>5.600274938598027</v>
       </c>
       <c r="P45" t="n">
-        <v>9856.932898275971</v>
+        <v>5.484176416186218e-09</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>7182.063356605612</v>
       </c>
     </row>
     <row r="46">
@@ -2901,205 +3038,217 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4944.561767578125</v>
+        <v>9633.416748046875</v>
       </c>
       <c r="E46" t="n">
-        <v>7.915838219591966</v>
+        <v>9633</v>
       </c>
       <c r="F46" t="n">
-        <v>0.3683099505358468</v>
+        <v>135.779151684903</v>
       </c>
       <c r="G46" t="n">
-        <v>0.001600918057389177</v>
+        <v>1.304228554709577</v>
       </c>
       <c r="H46" t="n">
-        <v>7.448788544838973e-05</v>
+        <v>0.01409459958352072</v>
       </c>
       <c r="I46" t="n">
-        <v>1.484261017007512</v>
+        <v>0.0001353858748998897</v>
       </c>
       <c r="J46" t="n">
-        <v>0.07218371225140059</v>
+        <v>0.9042606428263641</v>
       </c>
       <c r="K46" t="n">
-        <v>0.000374978253079178</v>
+        <v>0.00619267527097353</v>
       </c>
       <c r="L46" t="n">
-        <v>0.004489795918367347</v>
+        <v>0.0001631920864378598</v>
       </c>
       <c r="M46" t="n">
-        <v>22.2000732421875</v>
+        <v>0.03299319727891156</v>
       </c>
       <c r="N46" t="n">
-        <v>73.82638021620554</v>
+        <v>317.8372192382812</v>
       </c>
       <c r="O46" t="n">
-        <v>4.610246676062042e-11</v>
+        <v>12.07424623307133</v>
       </c>
       <c r="P46" t="n">
-        <v>4954.457814883755</v>
+        <v>1.899439743021853e-09</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>9634.460544446882</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5768.206787109375</v>
+        <v>2804.69970703125</v>
       </c>
       <c r="E47" t="n">
-        <v>31.92543080459712</v>
+        <v>2805</v>
       </c>
       <c r="F47" t="n">
-        <v>2.402161376318801</v>
+        <v>112.1591857637033</v>
       </c>
       <c r="G47" t="n">
-        <v>0.005534723698870014</v>
+        <v>3.116989985832063</v>
       </c>
       <c r="H47" t="n">
-        <v>0.0004164485541134001</v>
+        <v>0.03998973062339813</v>
       </c>
       <c r="I47" t="n">
-        <v>0.8224411756415669</v>
+        <v>0.001111345352950947</v>
       </c>
       <c r="J47" t="n">
-        <v>0.04763836043567797</v>
+        <v>0.7874208216893995</v>
       </c>
       <c r="K47" t="n">
-        <v>0.003106225350922567</v>
+        <v>0.01618327782969985</v>
       </c>
       <c r="L47" t="n">
-        <v>0.01501133786848073</v>
+        <v>0.003078120742162101</v>
       </c>
       <c r="M47" t="n">
-        <v>86.5885009765625</v>
+        <v>0.1009977324263039</v>
       </c>
       <c r="N47" t="n">
-        <v>26.63568621305765</v>
+        <v>283.268310546875</v>
       </c>
       <c r="O47" t="n">
-        <v>2.037326814883841e-10</v>
+        <v>4.548385840690079</v>
       </c>
       <c r="P47" t="n">
-        <v>5766.206632270292</v>
+        <v>7.782864418659612e-12</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2804.093986490997</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>7184.014892578125</v>
+        <v>2941.973876953125</v>
       </c>
       <c r="E48" t="n">
-        <v>236.2795024146108</v>
+        <v>2942</v>
       </c>
       <c r="F48" t="n">
-        <v>2.40489004794071</v>
+        <v>204.8053250741048</v>
       </c>
       <c r="G48" t="n">
-        <v>0.03288961756729004</v>
+        <v>2.090545044013624</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0003347557158358936</v>
+        <v>0.06961493665137938</v>
       </c>
       <c r="I48" t="n">
-        <v>0.9717468225374449</v>
+        <v>0.0007105926603871516</v>
       </c>
       <c r="J48" t="n">
-        <v>0.006551192460712446</v>
+        <v>0.8108312609039502</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0004427735154623166</v>
+        <v>0.005845507158385367</v>
       </c>
       <c r="L48" t="n">
-        <v>0.06448979591836734</v>
+        <v>0.0007536322401791502</v>
       </c>
       <c r="M48" t="n">
-        <v>463.295654296875</v>
+        <v>0.16</v>
       </c>
       <c r="N48" t="n">
-        <v>5.600274938598027</v>
+        <v>470.7158203125</v>
       </c>
       <c r="O48" t="n">
-        <v>5.484176416186218e-09</v>
+        <v>3.385749687296979</v>
       </c>
       <c r="P48" t="n">
-        <v>7182.063356605612</v>
+        <v>1.649522971510552e-11</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2943.013811279915</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>9633.416748046875</v>
+        <v>3862.518310546875</v>
       </c>
       <c r="E49" t="n">
-        <v>135.779151684903</v>
+        <v>3863</v>
       </c>
       <c r="F49" t="n">
-        <v>1.304228554709577</v>
+        <v>342.0198920001052</v>
       </c>
       <c r="G49" t="n">
-        <v>0.01409459958352072</v>
+        <v>2.265109638389958</v>
       </c>
       <c r="H49" t="n">
-        <v>0.0001353858748998897</v>
+        <v>0.08854841958061302</v>
       </c>
       <c r="I49" t="n">
-        <v>0.9042606428263641</v>
+        <v>0.0005864333722910564</v>
       </c>
       <c r="J49" t="n">
-        <v>0.00619267527097353</v>
+        <v>0.8301158019981648</v>
       </c>
       <c r="K49" t="n">
-        <v>0.0001631920864378598</v>
+        <v>0.003774163838770095</v>
       </c>
       <c r="L49" t="n">
-        <v>0.03299319727891156</v>
+        <v>0.0004130480838088269</v>
       </c>
       <c r="M49" t="n">
-        <v>317.8372192382812</v>
+        <v>0.1919954648526077</v>
       </c>
       <c r="N49" t="n">
-        <v>12.07424623307133</v>
+        <v>741.5859985351562</v>
       </c>
       <c r="O49" t="n">
-        <v>1.899439743021853e-09</v>
+        <v>3.045758270631805</v>
       </c>
       <c r="P49" t="n">
-        <v>9634.460544446882</v>
+        <v>2.7509079510722e-11</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>3862.739037311213</v>
       </c>
     </row>
     <row r="50">
@@ -3109,51 +3258,54 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2662.042236328125</v>
+        <v>2339.044189453125</v>
       </c>
       <c r="E50" t="n">
-        <v>26.80024350898403</v>
+        <v>2339</v>
       </c>
       <c r="F50" t="n">
-        <v>0.6634063282556106</v>
+        <v>833.5315642493954</v>
       </c>
       <c r="G50" t="n">
-        <v>0.01006755007236505</v>
+        <v>2.181040615102482</v>
       </c>
       <c r="H50" t="n">
-        <v>0.0002492095426595023</v>
+        <v>0.3563556293668301</v>
       </c>
       <c r="I50" t="n">
-        <v>1.374844633271292</v>
+        <v>0.0009324495128980077</v>
       </c>
       <c r="J50" t="n">
-        <v>0.03023452236352695</v>
+        <v>1.13292288867092</v>
       </c>
       <c r="K50" t="n">
-        <v>0.0009841833861590696</v>
+        <v>0.002252287858549144</v>
       </c>
       <c r="L50" t="n">
-        <v>0.02349206349206349</v>
+        <v>0.0003927868497291857</v>
       </c>
       <c r="M50" t="n">
-        <v>62.536865234375</v>
+        <v>0.7904988662131519</v>
       </c>
       <c r="N50" t="n">
-        <v>13.39453994590456</v>
+        <v>1849.011779785156</v>
       </c>
       <c r="O50" t="n">
-        <v>2.196421233614644e-12</v>
+        <v>1.700255064897827</v>
       </c>
       <c r="P50" t="n">
-        <v>2659.676701636059</v>
+        <v>1.219344120318504e-10</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>2340.388090027172</v>
       </c>
     </row>
     <row r="51">
@@ -3163,51 +3315,54 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2804.69970703125</v>
+        <v>4050.933837890625</v>
       </c>
       <c r="E51" t="n">
-        <v>112.1591857637033</v>
+        <v>4051</v>
       </c>
       <c r="F51" t="n">
-        <v>3.116989985832063</v>
+        <v>916.2758381885071</v>
       </c>
       <c r="G51" t="n">
-        <v>0.03998973062339813</v>
+        <v>3.395661205768661</v>
       </c>
       <c r="H51" t="n">
-        <v>0.001111345352950947</v>
+        <v>0.2261887937092609</v>
       </c>
       <c r="I51" t="n">
-        <v>0.7874208216893995</v>
+        <v>0.0008382415861762942</v>
       </c>
       <c r="J51" t="n">
-        <v>0.01618327782969985</v>
+        <v>0.9352741379327487</v>
       </c>
       <c r="K51" t="n">
-        <v>0.003078120742162101</v>
+        <v>0.002289990332693098</v>
       </c>
       <c r="L51" t="n">
-        <v>0.1009977324263039</v>
+        <v>0.0004352344504847237</v>
       </c>
       <c r="M51" t="n">
-        <v>283.268310546875</v>
+        <v>0.4734920634920635</v>
       </c>
       <c r="N51" t="n">
-        <v>4.548385840690079</v>
+        <v>1918.085021972656</v>
       </c>
       <c r="O51" t="n">
-        <v>7.782864418659612e-12</v>
+        <v>1.28095518819708</v>
       </c>
       <c r="P51" t="n">
-        <v>2804.093986490997</v>
+        <v>3.398105938092607e-11</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>4050.203365680363</v>
       </c>
     </row>
     <row r="52">
@@ -3217,51 +3372,54 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2941.973876953125</v>
+        <v>5838.189697265625</v>
       </c>
       <c r="E52" t="n">
-        <v>204.8053250741048</v>
+        <v>5838</v>
       </c>
       <c r="F52" t="n">
-        <v>2.090545044013624</v>
+        <v>555.1450293220936</v>
       </c>
       <c r="G52" t="n">
-        <v>0.06961493665137938</v>
+        <v>2.832061453128816</v>
       </c>
       <c r="H52" t="n">
-        <v>0.0007105926603871516</v>
+        <v>0.09508855623209732</v>
       </c>
       <c r="I52" t="n">
-        <v>0.8108312609039502</v>
+        <v>0.0004850924002101611</v>
       </c>
       <c r="J52" t="n">
-        <v>0.005845507158385367</v>
+        <v>0.8531948662396553</v>
       </c>
       <c r="K52" t="n">
-        <v>0.0007536322401791502</v>
+        <v>0.002966196585971969</v>
       </c>
       <c r="L52" t="n">
-        <v>0.16</v>
+        <v>0.0002708919184608968</v>
       </c>
       <c r="M52" t="n">
-        <v>470.7158203125</v>
+        <v>0.2009977324263039</v>
       </c>
       <c r="N52" t="n">
-        <v>3.385749687296979</v>
+        <v>1173.462890625</v>
       </c>
       <c r="O52" t="n">
-        <v>1.649522971510552e-11</v>
+        <v>2.935485532484775</v>
       </c>
       <c r="P52" t="n">
-        <v>2943.013811279915</v>
+        <v>2.796867277425509e-11</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>5839.230198622787</v>
       </c>
     </row>
     <row r="53">
@@ -3271,51 +3429,54 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3862.518310546875</v>
+        <v>8309.124755859375</v>
       </c>
       <c r="E53" t="n">
-        <v>342.0198920001052</v>
+        <v>8309</v>
       </c>
       <c r="F53" t="n">
-        <v>2.265109638389958</v>
+        <v>1501.91919676692</v>
       </c>
       <c r="G53" t="n">
-        <v>0.08854841958061302</v>
+        <v>4.696898412724011</v>
       </c>
       <c r="H53" t="n">
-        <v>0.0005864333722910564</v>
+        <v>0.1807554033543432</v>
       </c>
       <c r="I53" t="n">
-        <v>0.8301158019981648</v>
+        <v>0.0005652699352494236</v>
       </c>
       <c r="J53" t="n">
-        <v>0.003774163838770095</v>
+        <v>0.9896115551617721</v>
       </c>
       <c r="K53" t="n">
-        <v>0.0004130480838088269</v>
+        <v>0.002208303270317655</v>
       </c>
       <c r="L53" t="n">
-        <v>0.1919954648526077</v>
+        <v>0.0002996444111471889</v>
       </c>
       <c r="M53" t="n">
-        <v>741.5859985351562</v>
+        <v>0.4495011337868481</v>
       </c>
       <c r="N53" t="n">
-        <v>3.045758270631805</v>
+        <v>3734.960998535156</v>
       </c>
       <c r="O53" t="n">
-        <v>2.7509079510722e-11</v>
+        <v>1.387349873576789</v>
       </c>
       <c r="P53" t="n">
-        <v>3862.739037311213</v>
+        <v>9.021792532535704e-10</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>8309.988515326677</v>
       </c>
     </row>
     <row r="54">
@@ -3325,51 +3486,54 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2339.044189453125</v>
+        <v>732.12890625</v>
       </c>
       <c r="E54" t="n">
-        <v>833.5315642493954</v>
+        <v>732</v>
       </c>
       <c r="F54" t="n">
-        <v>2.181040615102482</v>
+        <v>426.0242234785599</v>
       </c>
       <c r="G54" t="n">
-        <v>0.3563556293668301</v>
+        <v>0.9465588900473837</v>
       </c>
       <c r="H54" t="n">
-        <v>0.0009324495128980077</v>
+        <v>0.5818978322556294</v>
       </c>
       <c r="I54" t="n">
-        <v>1.13292288867092</v>
+        <v>0.001292885558768202</v>
       </c>
       <c r="J54" t="n">
-        <v>0.002252287858549144</v>
+        <v>0.5703322494834494</v>
       </c>
       <c r="K54" t="n">
-        <v>0.0003927868497291857</v>
+        <v>0.001021537033707037</v>
       </c>
       <c r="L54" t="n">
-        <v>0.7904988662131519</v>
+        <v>8.321041434927589e-05</v>
       </c>
       <c r="M54" t="n">
-        <v>1849.011779785156</v>
+        <v>1.18</v>
       </c>
       <c r="N54" t="n">
-        <v>1.700255064897827</v>
+        <v>863.912109375</v>
       </c>
       <c r="O54" t="n">
-        <v>1.219344120318504e-10</v>
+        <v>1.869358907589715</v>
       </c>
       <c r="P54" t="n">
-        <v>2340.388090027172</v>
+        <v>8.443746198615233e-11</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>732.9333705336513</v>
       </c>
     </row>
     <row r="55">
@@ -3379,51 +3543,54 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4050.933837890625</v>
+        <v>985.14404296875</v>
       </c>
       <c r="E55" t="n">
-        <v>916.2758381885071</v>
+        <v>985</v>
       </c>
       <c r="F55" t="n">
-        <v>3.395661205768661</v>
+        <v>694.8643004530124</v>
       </c>
       <c r="G55" t="n">
-        <v>0.2261887937092609</v>
+        <v>2.539265973618143</v>
       </c>
       <c r="H55" t="n">
-        <v>0.0008382415861762942</v>
+        <v>0.7053428434272676</v>
       </c>
       <c r="I55" t="n">
-        <v>0.9352741379327487</v>
+        <v>0.002577558065484533</v>
       </c>
       <c r="J55" t="n">
-        <v>0.002289990332693098</v>
+        <v>0.4967652746459102</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0004352344504847237</v>
+        <v>0.001374978075252021</v>
       </c>
       <c r="L55" t="n">
-        <v>0.4734920634920635</v>
+        <v>0.0002234264096304524</v>
       </c>
       <c r="M55" t="n">
-        <v>1918.085021972656</v>
+        <v>1.369002267573696</v>
       </c>
       <c r="N55" t="n">
-        <v>1.28095518819708</v>
+        <v>1348.664428710938</v>
       </c>
       <c r="O55" t="n">
-        <v>3.398105938092607e-11</v>
+        <v>2.111207187761406</v>
       </c>
       <c r="P55" t="n">
-        <v>4050.203365680363</v>
+        <v>4.54303482517407e-11</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>984.581668316362</v>
       </c>
     </row>
     <row r="56">
@@ -3433,51 +3600,54 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5838.189697265625</v>
+        <v>1633.831787109375</v>
       </c>
       <c r="E56" t="n">
-        <v>555.1450293220936</v>
+        <v>1634</v>
       </c>
       <c r="F56" t="n">
-        <v>2.832061453128816</v>
+        <v>71.64584881729785</v>
       </c>
       <c r="G56" t="n">
-        <v>0.09508855623209732</v>
+        <v>2.798029810765954</v>
       </c>
       <c r="H56" t="n">
-        <v>0.0004850924002101611</v>
+        <v>0.04385142300607082</v>
       </c>
       <c r="I56" t="n">
-        <v>0.8531948662396553</v>
+        <v>0.001712556845106015</v>
       </c>
       <c r="J56" t="n">
-        <v>0.002966196585971969</v>
+        <v>0.687888065524211</v>
       </c>
       <c r="K56" t="n">
-        <v>0.0002708919184608968</v>
+        <v>0.01937478657080717</v>
       </c>
       <c r="L56" t="n">
-        <v>0.2009977324263039</v>
+        <v>0.005259074200213454</v>
       </c>
       <c r="M56" t="n">
-        <v>1173.462890625</v>
+        <v>0.1085034013605442</v>
       </c>
       <c r="N56" t="n">
-        <v>2.935485532484775</v>
+        <v>177.2763061523438</v>
       </c>
       <c r="O56" t="n">
-        <v>2.796867277425509e-11</v>
+        <v>5.527666438818121</v>
       </c>
       <c r="P56" t="n">
-        <v>5839.230198622787</v>
+        <v>9.064826848430388e-12</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>1634.412669824537</v>
       </c>
     </row>
     <row r="57">
@@ -3487,51 +3657,54 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8309.124755859375</v>
+        <v>2225.994873046875</v>
       </c>
       <c r="E57" t="n">
-        <v>1501.91919676692</v>
+        <v>2226</v>
       </c>
       <c r="F57" t="n">
-        <v>4.696898412724011</v>
+        <v>660.1708006533678</v>
       </c>
       <c r="G57" t="n">
-        <v>0.1807554033543432</v>
+        <v>2.006211577553995</v>
       </c>
       <c r="H57" t="n">
-        <v>0.0005652699352494236</v>
+        <v>0.2965733697983526</v>
       </c>
       <c r="I57" t="n">
-        <v>0.9896115551617721</v>
+        <v>0.0009012651384987032</v>
       </c>
       <c r="J57" t="n">
-        <v>0.002208303270317655</v>
+        <v>0.8058744981350021</v>
       </c>
       <c r="K57" t="n">
-        <v>0.0002996444111471889</v>
+        <v>0.001597878152246114</v>
       </c>
       <c r="L57" t="n">
-        <v>0.4495011337868481</v>
+        <v>0.0003043553852052328</v>
       </c>
       <c r="M57" t="n">
-        <v>3734.960998535156</v>
+        <v>0.6334920634920634</v>
       </c>
       <c r="N57" t="n">
-        <v>1.387349873576789</v>
+        <v>1410.150085449219</v>
       </c>
       <c r="O57" t="n">
-        <v>9.021792532535704e-10</v>
+        <v>1.833350440871084</v>
       </c>
       <c r="P57" t="n">
-        <v>8309.988515326677</v>
+        <v>3.090843463916614e-11</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>2226.429989231169</v>
       </c>
     </row>
     <row r="58">
@@ -3541,51 +3714,54 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>732.12890625</v>
+        <v>904.39453125</v>
       </c>
       <c r="E58" t="n">
-        <v>426.0242234785599</v>
+        <v>904</v>
       </c>
       <c r="F58" t="n">
-        <v>0.9465588900473837</v>
+        <v>343.9176201914185</v>
       </c>
       <c r="G58" t="n">
-        <v>0.5818978322556294</v>
+        <v>2.450073601578405</v>
       </c>
       <c r="H58" t="n">
-        <v>0.001292885558768202</v>
+        <v>0.3802738830320835</v>
       </c>
       <c r="I58" t="n">
-        <v>0.5703322494834494</v>
+        <v>0.002709076091152454</v>
       </c>
       <c r="J58" t="n">
-        <v>0.001021537033707037</v>
+        <v>0.5605367190463145</v>
       </c>
       <c r="K58" t="n">
-        <v>8.321041434927589e-05</v>
+        <v>0.002369263841942123</v>
       </c>
       <c r="L58" t="n">
-        <v>1.18</v>
+        <v>0.0008353972374226948</v>
       </c>
       <c r="M58" t="n">
-        <v>863.912109375</v>
+        <v>0.65</v>
       </c>
       <c r="N58" t="n">
-        <v>1.869358907589715</v>
+        <v>587.8564453125</v>
       </c>
       <c r="O58" t="n">
-        <v>8.443746198615233e-11</v>
+        <v>2.545154730379255</v>
       </c>
       <c r="P58" t="n">
-        <v>732.9333705336513</v>
+        <v>7.161708852846133e-09</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>904.9686777906261</v>
       </c>
     </row>
     <row r="59">
@@ -3595,51 +3771,54 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>985.14404296875</v>
+        <v>1520.782470703125</v>
       </c>
       <c r="E59" t="n">
-        <v>694.8643004530124</v>
+        <v>1521</v>
       </c>
       <c r="F59" t="n">
-        <v>2.539265973618143</v>
+        <v>724.8780094116786</v>
       </c>
       <c r="G59" t="n">
-        <v>0.7053428434272676</v>
+        <v>1.01886750048609</v>
       </c>
       <c r="H59" t="n">
-        <v>0.002577558065484533</v>
+        <v>0.4766480567576081</v>
       </c>
       <c r="I59" t="n">
-        <v>0.4967652746459102</v>
+        <v>0.0006699626804713384</v>
       </c>
       <c r="J59" t="n">
-        <v>0.001374978075252021</v>
+        <v>0.7933168937124105</v>
       </c>
       <c r="K59" t="n">
-        <v>0.0002234264096304524</v>
+        <v>0.0006971795280635326</v>
       </c>
       <c r="L59" t="n">
-        <v>1.369002267573696</v>
+        <v>9.284643772323053e-05</v>
       </c>
       <c r="M59" t="n">
-        <v>1348.664428710938</v>
+        <v>0.9170068027210885</v>
       </c>
       <c r="N59" t="n">
-        <v>2.111207187761406</v>
+        <v>1394.56787109375</v>
       </c>
       <c r="O59" t="n">
-        <v>4.54303482517407e-11</v>
+        <v>1.952430412995464</v>
       </c>
       <c r="P59" t="n">
-        <v>984.581668316362</v>
+        <v>7.462411328533061e-09</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1520.304279797999</v>
       </c>
     </row>
     <row r="60">
@@ -3649,321 +3828,54 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1633.831787109375</v>
+        <v>2037.579345703125</v>
       </c>
       <c r="E60" t="n">
-        <v>71.64584881729785</v>
+        <v>2038</v>
       </c>
       <c r="F60" t="n">
-        <v>2.798029810765954</v>
+        <v>403.363723287138</v>
       </c>
       <c r="G60" t="n">
-        <v>0.04385142300607082</v>
+        <v>0.6939979087577202</v>
       </c>
       <c r="H60" t="n">
-        <v>0.001712556845106015</v>
+        <v>0.1979622163611723</v>
       </c>
       <c r="I60" t="n">
-        <v>0.687888065524211</v>
+        <v>0.0003405992067112539</v>
       </c>
       <c r="J60" t="n">
-        <v>0.01937478657080717</v>
+        <v>0.9228832326415889</v>
       </c>
       <c r="K60" t="n">
-        <v>0.005259074200213454</v>
+        <v>0.001064998810228081</v>
       </c>
       <c r="L60" t="n">
-        <v>0.1085034013605442</v>
+        <v>7.753620886085926e-05</v>
       </c>
       <c r="M60" t="n">
-        <v>177.2763061523438</v>
+        <v>0.4160090702947846</v>
       </c>
       <c r="N60" t="n">
-        <v>5.527666438818121</v>
+        <v>847.6514892578125</v>
       </c>
       <c r="O60" t="n">
-        <v>9.064826848430388e-12</v>
+        <v>1.725143363002918</v>
       </c>
       <c r="P60" t="n">
-        <v>1634.412669824537</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>2</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>LSrearSOAEwf1.mat</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>2225.994873046875</v>
-      </c>
-      <c r="E61" t="n">
-        <v>660.1708006533678</v>
-      </c>
-      <c r="F61" t="n">
-        <v>2.006211577553995</v>
-      </c>
-      <c r="G61" t="n">
-        <v>0.2965733697983526</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0.0009012651384987032</v>
-      </c>
-      <c r="I61" t="n">
-        <v>0.8058744981350021</v>
-      </c>
-      <c r="J61" t="n">
-        <v>0.001597878152246114</v>
-      </c>
-      <c r="K61" t="n">
-        <v>0.0003043553852052328</v>
-      </c>
-      <c r="L61" t="n">
-        <v>0.6334920634920634</v>
-      </c>
-      <c r="M61" t="n">
-        <v>1410.150085449219</v>
-      </c>
-      <c r="N61" t="n">
-        <v>1.833350440871084</v>
-      </c>
-      <c r="O61" t="n">
-        <v>3.090843463916614e-11</v>
-      </c>
-      <c r="P61" t="n">
-        <v>2226.429989231169</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>3</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>904.39453125</v>
-      </c>
-      <c r="E62" t="n">
-        <v>343.9176201914185</v>
-      </c>
-      <c r="F62" t="n">
-        <v>2.450073601578405</v>
-      </c>
-      <c r="G62" t="n">
-        <v>0.3802738830320835</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0.002709076091152454</v>
-      </c>
-      <c r="I62" t="n">
-        <v>0.5605367190463145</v>
-      </c>
-      <c r="J62" t="n">
-        <v>0.002369263841942123</v>
-      </c>
-      <c r="K62" t="n">
-        <v>0.0008353972374226948</v>
-      </c>
-      <c r="L62" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="M62" t="n">
-        <v>587.8564453125</v>
-      </c>
-      <c r="N62" t="n">
-        <v>2.545154730379255</v>
-      </c>
-      <c r="O62" t="n">
-        <v>7.161708852846133e-09</v>
-      </c>
-      <c r="P62" t="n">
-        <v>904.9686777906261</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>1520.782470703125</v>
-      </c>
-      <c r="E63" t="n">
-        <v>724.8780094116786</v>
-      </c>
-      <c r="F63" t="n">
-        <v>1.01886750048609</v>
-      </c>
-      <c r="G63" t="n">
-        <v>0.4766480567576081</v>
-      </c>
-      <c r="H63" t="n">
-        <v>0.0006699626804713384</v>
-      </c>
-      <c r="I63" t="n">
-        <v>0.7933168937124105</v>
-      </c>
-      <c r="J63" t="n">
-        <v>0.0006971795280635326</v>
-      </c>
-      <c r="K63" t="n">
-        <v>9.284643772323053e-05</v>
-      </c>
-      <c r="L63" t="n">
-        <v>0.9170068027210885</v>
-      </c>
-      <c r="M63" t="n">
-        <v>1394.56787109375</v>
-      </c>
-      <c r="N63" t="n">
-        <v>1.952430412995464</v>
-      </c>
-      <c r="O63" t="n">
-        <v>7.462411328533061e-09</v>
-      </c>
-      <c r="P63" t="n">
-        <v>1520.304279797999</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>3</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>2037.579345703125</v>
-      </c>
-      <c r="E64" t="n">
-        <v>403.363723287138</v>
-      </c>
-      <c r="F64" t="n">
-        <v>0.6939979087577202</v>
-      </c>
-      <c r="G64" t="n">
-        <v>0.1979622163611723</v>
-      </c>
-      <c r="H64" t="n">
-        <v>0.0003405992067112539</v>
-      </c>
-      <c r="I64" t="n">
-        <v>0.9228832326415889</v>
-      </c>
-      <c r="J64" t="n">
-        <v>0.001064998810228081</v>
-      </c>
-      <c r="K64" t="n">
-        <v>7.753620886085926e-05</v>
-      </c>
-      <c r="L64" t="n">
-        <v>0.4160090702947846</v>
-      </c>
-      <c r="M64" t="n">
-        <v>847.6514892578125</v>
-      </c>
-      <c r="N64" t="n">
-        <v>1.725143363002918</v>
-      </c>
-      <c r="O64" t="n">
         <v>8.231508706457555e-09</v>
       </c>
-      <c r="P64" t="n">
+      <c r="Q60" t="n">
         <v>2038.146974608225</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>3</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>2694.342041015625</v>
-      </c>
-      <c r="E65" t="n">
-        <v>34.41335938393284</v>
-      </c>
-      <c r="F65" t="n">
-        <v>0.3729234884813598</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.01277245385332028</v>
-      </c>
-      <c r="H65" t="n">
-        <v>0.0001384098539845324</v>
-      </c>
-      <c r="I65" t="n">
-        <v>1.286343718669184</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0.01258520861402013</v>
-      </c>
-      <c r="K65" t="n">
-        <v>0.0002782269568808125</v>
-      </c>
-      <c r="L65" t="n">
-        <v>0.03650793650793651</v>
-      </c>
-      <c r="M65" t="n">
-        <v>98.3648681640625</v>
-      </c>
-      <c r="N65" t="n">
-        <v>9.907909797259302</v>
-      </c>
-      <c r="O65" t="n">
-        <v>2.614181286759171e-10</v>
-      </c>
-      <c r="P65" t="n">
-        <v>2696.097771353126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
switched over to 200 Hz static lizards
</commit_message>
<xml_diff>
--- a/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
+++ b/results/soae/SOAE Results (Static Flattop, BW=Species, Mode=phi)/SOAE N_xi Fitted Parameters (Static Flattop, BW=Species, Mode=phi).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q60"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,40 +536,40 @@
         <v>1235</v>
       </c>
       <c r="F2" t="n">
-        <v>16.27045348324553</v>
+        <v>16.28805780965003</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1604725269936995</v>
+        <v>0.2570100636312063</v>
       </c>
       <c r="H2" t="n">
-        <v>0.01316947074481619</v>
+        <v>0.01318371986588739</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0001298880975730921</v>
+        <v>0.0002080265628490253</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9985519516693381</v>
+        <v>0.8730865242162046</v>
       </c>
       <c r="K2" t="n">
-        <v>0.007620958622036293</v>
+        <v>0.01013263330912294</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0001611813450498767</v>
+        <v>0.0003290155909698478</v>
       </c>
       <c r="M2" t="n">
-        <v>0.03099773242630385</v>
+        <v>0.02950113378684807</v>
       </c>
       <c r="N2" t="n">
-        <v>38.29669189453125</v>
+        <v>36.44769287109375</v>
       </c>
       <c r="O2" t="n">
-        <v>13.76357921407892</v>
+        <v>14.30510016845546</v>
       </c>
       <c r="P2" t="n">
-        <v>2.813538798148832e-11</v>
+        <v>2.77729720474316e-11</v>
       </c>
       <c r="Q2" t="n">
-        <v>1233.00912198773</v>
+        <v>1232.98854275687</v>
       </c>
     </row>
     <row r="3">
@@ -593,40 +593,40 @@
         <v>2153</v>
       </c>
       <c r="F3" t="n">
-        <v>19.32091238876069</v>
+        <v>19.51723609601467</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1191495762712399</v>
+        <v>0.1801369017511076</v>
       </c>
       <c r="H3" t="n">
-        <v>0.008972614188703376</v>
+        <v>0.009063786740280737</v>
       </c>
       <c r="I3" t="n">
-        <v>5.533295514818578e-05</v>
+        <v>8.365541378373433e-05</v>
       </c>
       <c r="J3" t="n">
-        <v>1.138955073099183</v>
+        <v>1.03877647278039</v>
       </c>
       <c r="K3" t="n">
-        <v>0.005973835603635176</v>
+        <v>0.00762983014395034</v>
       </c>
       <c r="L3" t="n">
-        <v>4.912864377187464e-05</v>
+        <v>0.000100694483473601</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02299319727891156</v>
+        <v>0.02199546485260771</v>
       </c>
       <c r="N3" t="n">
-        <v>49.51171875</v>
+        <v>47.36328125</v>
       </c>
       <c r="O3" t="n">
-        <v>17.48944487684902</v>
+        <v>18.31682574313761</v>
       </c>
       <c r="P3" t="n">
-        <v>2.735008223368497e-11</v>
+        <v>2.696578289494421e-11</v>
       </c>
       <c r="Q3" t="n">
-        <v>2155.319437958638</v>
+        <v>2155.371051067194</v>
       </c>
     </row>
     <row r="4">
@@ -650,40 +650,40 @@
         <v>3704</v>
       </c>
       <c r="F4" t="n">
-        <v>31.46322969314967</v>
+        <v>31.18317918159503</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1427470844557601</v>
+        <v>0.1032097510305445</v>
       </c>
       <c r="H4" t="n">
-        <v>0.008495055425245283</v>
+        <v>0.008419441934808128</v>
       </c>
       <c r="I4" t="n">
-        <v>3.854163752641942e-05</v>
+        <v>2.786657835133618e-05</v>
       </c>
       <c r="J4" t="n">
-        <v>1.206275863016083</v>
+        <v>1.136588683818613</v>
       </c>
       <c r="K4" t="n">
-        <v>0.004677101758986906</v>
+        <v>0.003019260431203308</v>
       </c>
       <c r="L4" t="n">
-        <v>2.622069975168253e-05</v>
+        <v>1.35151629067455e-05</v>
       </c>
       <c r="M4" t="n">
-        <v>0.02099773242630385</v>
+        <v>0.02</v>
       </c>
       <c r="N4" t="n">
-        <v>77.76953125</v>
+        <v>74.07421875</v>
       </c>
       <c r="O4" t="n">
-        <v>18.37701490468909</v>
+        <v>19.03377135638383</v>
       </c>
       <c r="P4" t="n">
-        <v>1.235028563709804e-10</v>
+        <v>1.221877867257483e-10</v>
       </c>
       <c r="Q4" t="n">
-        <v>3704.297679527263</v>
+        <v>3704.29659206207</v>
       </c>
     </row>
     <row r="5">
@@ -707,40 +707,40 @@
         <v>4500</v>
       </c>
       <c r="F5" t="n">
-        <v>18.73891316765203</v>
+        <v>15.37375060002046</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5111525313559319</v>
+        <v>0.1922352820240326</v>
       </c>
       <c r="H5" t="n">
-        <v>0.004163796305411945</v>
+        <v>0.003416055423064361</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0001135783597757324</v>
+        <v>4.271478019564266e-05</v>
       </c>
       <c r="J5" t="n">
-        <v>1.331207539183221</v>
+        <v>1.260711060391065</v>
       </c>
       <c r="K5" t="n">
-        <v>0.03210092064674847</v>
+        <v>0.01505460436522362</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0004891674757343065</v>
+        <v>6.94646110511521e-05</v>
       </c>
       <c r="M5" t="n">
-        <v>0.01049886621315193</v>
+        <v>0.009501133786848073</v>
       </c>
       <c r="N5" t="n">
-        <v>47.24951171875</v>
+        <v>42.75927734375</v>
       </c>
       <c r="O5" t="n">
-        <v>34.76595543223775</v>
+        <v>41.71739241117515</v>
       </c>
       <c r="P5" t="n">
-        <v>6.755779864268177e-12</v>
+        <v>6.482667219691164e-12</v>
       </c>
       <c r="Q5" t="n">
-        <v>4501.129974561822</v>
+        <v>4500.598712920311</v>
       </c>
     </row>
     <row r="6">
@@ -764,40 +764,40 @@
         <v>966</v>
       </c>
       <c r="F6" t="n">
-        <v>6.137620528466492</v>
+        <v>5.640270390569921</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1872804185843038</v>
+        <v>0.3663721760494623</v>
       </c>
       <c r="H6" t="n">
-        <v>0.006351655501765107</v>
+        <v>0.005836961456243255</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0001938113794355215</v>
+        <v>0.0003791485375977861</v>
       </c>
       <c r="J6" t="n">
-        <v>1.072079156092322</v>
+        <v>0.907619697924113</v>
       </c>
       <c r="K6" t="n">
-        <v>0.02693463093490572</v>
+        <v>0.04931460150274743</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0009077351656215396</v>
+        <v>0.002581769715006478</v>
       </c>
       <c r="M6" t="n">
-        <v>0.01800453514739229</v>
+        <v>0.01650793650793651</v>
       </c>
       <c r="N6" t="n">
-        <v>17.3978271484375</v>
+        <v>15.95166015625</v>
       </c>
       <c r="O6" t="n">
-        <v>24.10412405477431</v>
+        <v>28.2915017377736</v>
       </c>
       <c r="P6" t="n">
-        <v>2.059603196508205e-11</v>
+        <v>1.954098754610866e-11</v>
       </c>
       <c r="Q6" t="n">
-        <v>966.5721338914575</v>
+        <v>966.6417869335367</v>
       </c>
     </row>
     <row r="7">
@@ -821,40 +821,40 @@
         <v>3152</v>
       </c>
       <c r="F7" t="n">
-        <v>20.46677603291103</v>
+        <v>20.33151099562044</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2005660799087317</v>
+        <v>0.1190675053548426</v>
       </c>
       <c r="H7" t="n">
-        <v>0.006493425944126177</v>
+        <v>0.006450510855737879</v>
       </c>
       <c r="I7" t="n">
-        <v>6.363293293955125e-05</v>
+        <v>3.777615131617532e-05</v>
       </c>
       <c r="J7" t="n">
-        <v>1.243291384815935</v>
+        <v>1.127051197920187</v>
       </c>
       <c r="K7" t="n">
-        <v>0.01051288534168879</v>
+        <v>0.005673518487236455</v>
       </c>
       <c r="L7" t="n">
-        <v>9.893151436961653e-05</v>
+        <v>2.79682433373301e-05</v>
       </c>
       <c r="M7" t="n">
-        <v>0.01650793650793651</v>
+        <v>0.01600907029478458</v>
       </c>
       <c r="N7" t="n">
-        <v>52.03173828125001</v>
+        <v>50.45935058593749</v>
       </c>
       <c r="O7" t="n">
-        <v>23.35091952012064</v>
+        <v>25.04321508812544</v>
       </c>
       <c r="P7" t="n">
-        <v>1.583734146407318e-10</v>
+        <v>1.554121431441295e-10</v>
       </c>
       <c r="Q7" t="n">
-        <v>3152.508980960771</v>
+        <v>3152.499373308552</v>
       </c>
     </row>
     <row r="8">
@@ -878,40 +878,40 @@
         <v>3954</v>
       </c>
       <c r="F8" t="n">
-        <v>15.53825647486</v>
+        <v>14.51932711652016</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5098892675341249</v>
+        <v>0.2934689583848036</v>
       </c>
       <c r="H8" t="n">
-        <v>0.003929722103890167</v>
+        <v>0.003672028505625193</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0001289541801814846</v>
+        <v>7.422013238333916e-05</v>
       </c>
       <c r="J8" t="n">
-        <v>1.460311260664919</v>
+        <v>1.326045062261043</v>
       </c>
       <c r="K8" t="n">
-        <v>0.04805708251155821</v>
+        <v>0.02468141039560292</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0005595649156774294</v>
+        <v>0.0002143749004068811</v>
       </c>
       <c r="M8" t="n">
-        <v>0.01</v>
+        <v>0.009501133786848073</v>
       </c>
       <c r="N8" t="n">
-        <v>39.54034423828125</v>
+        <v>37.56781005859375</v>
       </c>
       <c r="O8" t="n">
-        <v>33.73452550992971</v>
+        <v>38.79908349221185</v>
       </c>
       <c r="P8" t="n">
-        <v>4.926773925604347e-11</v>
+        <v>4.799001733924926e-11</v>
       </c>
       <c r="Q8" t="n">
-        <v>3944.963974235252</v>
+        <v>3943.679953556278</v>
       </c>
     </row>
     <row r="9">
@@ -935,40 +935,40 @@
         <v>2178</v>
       </c>
       <c r="F9" t="n">
-        <v>23.87533611430924</v>
+        <v>24.5051156207832</v>
       </c>
       <c r="G9" t="n">
-        <v>0.199603620443464</v>
+        <v>0.2138535209922222</v>
       </c>
       <c r="H9" t="n">
-        <v>0.01096433565968014</v>
+        <v>0.01125355101847167</v>
       </c>
       <c r="I9" t="n">
-        <v>9.166451449945803e-05</v>
+        <v>9.820853515682607e-05</v>
       </c>
       <c r="J9" t="n">
-        <v>1.229145680085068</v>
+        <v>1.148446504889286</v>
       </c>
       <c r="K9" t="n">
-        <v>0.008954135430953924</v>
+        <v>0.008229025402798424</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0001070512298754903</v>
+        <v>0.0001130678900154355</v>
       </c>
       <c r="M9" t="n">
-        <v>0.02600907029478458</v>
+        <v>0.02551020408163265</v>
       </c>
       <c r="N9" t="n">
-        <v>56.63592529296875</v>
+        <v>55.54962158203125</v>
       </c>
       <c r="O9" t="n">
-        <v>14.21023832975533</v>
+        <v>14.45949872044094</v>
       </c>
       <c r="P9" t="n">
-        <v>9.650500119140539e-11</v>
+        <v>9.605670030987539e-11</v>
       </c>
       <c r="Q9" t="n">
-        <v>2175.246197569066</v>
+        <v>2175.234931285351</v>
       </c>
     </row>
     <row r="10">
@@ -992,40 +992,40 @@
         <v>3112</v>
       </c>
       <c r="F10" t="n">
-        <v>18.1369995145824</v>
+        <v>18.27886725288525</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2432247810841414</v>
+        <v>0.1021111832822258</v>
       </c>
       <c r="H10" t="n">
-        <v>0.005828931573549382</v>
+        <v>0.005874525517486837</v>
       </c>
       <c r="I10" t="n">
-        <v>7.816842056984703e-05</v>
+        <v>3.281684491239608e-05</v>
       </c>
       <c r="J10" t="n">
-        <v>1.360869933351719</v>
+        <v>1.230377603318903</v>
       </c>
       <c r="K10" t="n">
-        <v>0.01761179210471739</v>
+        <v>0.006089725744580973</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0001563171901731081</v>
+        <v>2.647013930316955e-05</v>
       </c>
       <c r="M10" t="n">
-        <v>0.01551020408163265</v>
+        <v>0.01501133786848073</v>
       </c>
       <c r="N10" t="n">
-        <v>48.2607421875</v>
+        <v>46.70849609375</v>
       </c>
       <c r="O10" t="n">
-        <v>24.17271670332591</v>
+        <v>25.80897301507194</v>
       </c>
       <c r="P10" t="n">
-        <v>7.06937906864068e-11</v>
+        <v>6.949503417742286e-11</v>
       </c>
       <c r="Q10" t="n">
-        <v>3112.93841005744</v>
+        <v>3113.035423262702</v>
       </c>
     </row>
     <row r="11">
@@ -1049,25 +1049,25 @@
         <v>3478</v>
       </c>
       <c r="F11" t="n">
-        <v>21.11625766221708</v>
+        <v>20.67109348467221</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3180059870534072</v>
+        <v>0.0902120146076017</v>
       </c>
       <c r="H11" t="n">
-        <v>0.006072056288090055</v>
+        <v>0.005944047718260454</v>
       </c>
       <c r="I11" t="n">
-        <v>9.144377210328032e-05</v>
+        <v>2.594079118192797e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>1.279115198918998</v>
+        <v>1.133663403847548</v>
       </c>
       <c r="K11" t="n">
-        <v>0.01665715461241262</v>
+        <v>0.004001320087077613</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0002044789298814027</v>
+        <v>1.635982179638845e-05</v>
       </c>
       <c r="M11" t="n">
         <v>0.01448979591836735</v>
@@ -1076,13 +1076,13 @@
         <v>50.389892578125</v>
       </c>
       <c r="O11" t="n">
-        <v>24.60793692397083</v>
+        <v>26.6861854826555</v>
       </c>
       <c r="P11" t="n">
-        <v>5.100088038041753e-11</v>
+        <v>4.992122935719596e-11</v>
       </c>
       <c r="Q11" t="n">
-        <v>3478.017965968106</v>
+        <v>3478.119035054389</v>
       </c>
     </row>
     <row r="12">
@@ -1106,40 +1106,40 @@
         <v>1798</v>
       </c>
       <c r="F12" t="n">
-        <v>10.83138782180633</v>
+        <v>10.44835791661786</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1189343580154598</v>
+        <v>0.1204873514374585</v>
       </c>
       <c r="H12" t="n">
-        <v>0.006024055904262052</v>
+        <v>0.005811027472465509</v>
       </c>
       <c r="I12" t="n">
-        <v>6.614731495258778e-05</v>
+        <v>6.701103799039066e-05</v>
       </c>
       <c r="J12" t="n">
-        <v>1.233487856175178</v>
+        <v>1.124744640322379</v>
       </c>
       <c r="K12" t="n">
-        <v>0.01208949815066053</v>
+        <v>0.01074488411064471</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0001152929336444951</v>
+        <v>0.0001182803543130794</v>
       </c>
       <c r="M12" t="n">
-        <v>0.01650793650793651</v>
+        <v>0.01551020408163265</v>
       </c>
       <c r="N12" t="n">
-        <v>29.681640625</v>
+        <v>27.8876953125</v>
       </c>
       <c r="O12" t="n">
-        <v>23.55275459339331</v>
+        <v>25.34294602451444</v>
       </c>
       <c r="P12" t="n">
-        <v>1.759269509509833e-11</v>
+        <v>1.72439401270541e-11</v>
       </c>
       <c r="Q12" t="n">
-        <v>1793.479704400886</v>
+        <v>1793.035344578808</v>
       </c>
     </row>
     <row r="13">
@@ -1163,40 +1163,40 @@
         <v>2140</v>
       </c>
       <c r="F13" t="n">
-        <v>7.383225339650395</v>
+        <v>5.831130034579246</v>
       </c>
       <c r="G13" t="n">
-        <v>0.3977289205921791</v>
+        <v>0.2630292277422717</v>
       </c>
       <c r="H13" t="n">
-        <v>0.003450327699049675</v>
+        <v>0.002725002766341402</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0001858666163231724</v>
+        <v>0.0001229187771454065</v>
       </c>
       <c r="J13" t="n">
-        <v>1.418070862340206</v>
+        <v>1.44973626858714</v>
       </c>
       <c r="K13" t="n">
-        <v>0.06976038352038443</v>
+        <v>0.06515953483187181</v>
       </c>
       <c r="L13" t="n">
-        <v>0.001307088889552022</v>
+        <v>0.0005669978619138594</v>
       </c>
       <c r="M13" t="n">
-        <v>0.008004535147392289</v>
+        <v>0.006507936507936508</v>
       </c>
       <c r="N13" t="n">
-        <v>17.12860107421875</v>
+        <v>13.92608642578125</v>
       </c>
       <c r="O13" t="n">
-        <v>41.30265573954974</v>
+        <v>48.96958175305302</v>
       </c>
       <c r="P13" t="n">
-        <v>3.539373210432152e-12</v>
+        <v>3.460224849895886e-12</v>
       </c>
       <c r="Q13" t="n">
-        <v>2141.354446457694</v>
+        <v>2141.702265000833</v>
       </c>
     </row>
     <row r="14">
@@ -1220,40 +1220,40 @@
         <v>2417</v>
       </c>
       <c r="F14" t="n">
-        <v>7.685360244948903</v>
+        <v>5.851177172244928</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4288062054925163</v>
+        <v>0.3076679363547534</v>
       </c>
       <c r="H14" t="n">
-        <v>0.003179576237778152</v>
+        <v>0.002420740642851105</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0001774050894350607</v>
+        <v>0.0001272879381552424</v>
       </c>
       <c r="J14" t="n">
-        <v>1.44421366723964</v>
+        <v>1.514628228206574</v>
       </c>
       <c r="K14" t="n">
-        <v>0.07587432245996721</v>
+        <v>0.08387519213289332</v>
       </c>
       <c r="L14" t="n">
-        <v>0.00123986853948281</v>
+        <v>0.0006530386203626407</v>
       </c>
       <c r="M14" t="n">
-        <v>0.007505668934240363</v>
+        <v>0.00600907029478458</v>
       </c>
       <c r="N14" t="n">
-        <v>18.1419677734375</v>
+        <v>14.5245361328125</v>
       </c>
       <c r="O14" t="n">
-        <v>42.34817726778903</v>
+        <v>52.2115254981341</v>
       </c>
       <c r="P14" t="n">
-        <v>2.902234163120909e-12</v>
+        <v>2.816141988184028e-12</v>
       </c>
       <c r="Q14" t="n">
-        <v>2413.939743194736</v>
+        <v>2413.736927509325</v>
       </c>
     </row>
     <row r="15">
@@ -1277,40 +1277,40 @@
         <v>2783</v>
       </c>
       <c r="F15" t="n">
-        <v>222580056.6111855</v>
+        <v>6.23314094429366</v>
       </c>
       <c r="G15" t="n">
-        <v>212851825869879.1</v>
+        <v>0.4071097251252815</v>
       </c>
       <c r="H15" t="n">
-        <v>79973.67613428384</v>
+        <v>0.00223958607418754</v>
       </c>
       <c r="I15" t="n">
-        <v>76478293904.13248</v>
+        <v>0.0001462757346906453</v>
       </c>
       <c r="J15" t="n">
-        <v>0.01931650088908909</v>
+        <v>1.572514400844669</v>
       </c>
       <c r="K15" t="n">
-        <v>0.004113185546243618</v>
+        <v>0.1114084550460969</v>
       </c>
       <c r="L15" t="n">
-        <v>2.729313132736339e-05</v>
+        <v>0.0008459310893722362</v>
       </c>
       <c r="M15" t="n">
-        <v>0.02498866213151927</v>
+        <v>0.005510204081632653</v>
       </c>
       <c r="N15" t="n">
-        <v>69.547607421875</v>
+        <v>15.3358154296875</v>
       </c>
       <c r="O15" t="n">
-        <v>46.27969260680279</v>
+        <v>57.92096445875224</v>
       </c>
       <c r="P15" t="n">
-        <v>3.577109007377321e-12</v>
+        <v>3.498125488706444e-12</v>
       </c>
       <c r="Q15" t="n">
-        <v>2784.865043070137</v>
+        <v>2786.707198943668</v>
       </c>
     </row>
     <row r="16">
@@ -1334,40 +1334,40 @@
         <v>1343</v>
       </c>
       <c r="F16" t="n">
-        <v>4.460025553747603</v>
+        <v>3.281272247384341</v>
       </c>
       <c r="G16" t="n">
-        <v>0.2083667218300633</v>
+        <v>0.1103627918020275</v>
       </c>
       <c r="H16" t="n">
-        <v>0.003321502666936397</v>
+        <v>0.002443652931870229</v>
       </c>
       <c r="I16" t="n">
-        <v>0.0001551763804756254</v>
+        <v>8.219018094929178e-05</v>
       </c>
       <c r="J16" t="n">
-        <v>1.423530552657516</v>
+        <v>1.469618752364346</v>
       </c>
       <c r="K16" t="n">
-        <v>0.06219363852230954</v>
+        <v>0.05282117625686077</v>
       </c>
       <c r="L16" t="n">
-        <v>0.0009635734659170579</v>
+        <v>0.0002921131068832113</v>
       </c>
       <c r="M16" t="n">
-        <v>0.008</v>
+        <v>0.0065</v>
       </c>
       <c r="N16" t="n">
-        <v>10.7421875</v>
+        <v>8.728027343749998</v>
       </c>
       <c r="O16" t="n">
-        <v>42.66633598035457</v>
+        <v>53.61458844414353</v>
       </c>
       <c r="P16" t="n">
-        <v>3.152433682764227e-11</v>
+        <v>3.04650185607582e-11</v>
       </c>
       <c r="Q16" t="n">
-        <v>1345.558150501267</v>
+        <v>1345.084696692057</v>
       </c>
     </row>
     <row r="17">
@@ -1391,40 +1391,40 @@
         <v>1779</v>
       </c>
       <c r="F17" t="n">
-        <v>8.448976852641636</v>
+        <v>7.350380557891555</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1296501109855726</v>
+        <v>0.4334125605700579</v>
       </c>
       <c r="H17" t="n">
-        <v>0.004748817727398991</v>
+        <v>0.004131342540668791</v>
       </c>
       <c r="I17" t="n">
-        <v>7.287092344382921e-05</v>
+        <v>0.0002436031352445911</v>
       </c>
       <c r="J17" t="n">
-        <v>1.239216578257107</v>
+        <v>1.048293548986893</v>
       </c>
       <c r="K17" t="n">
-        <v>0.01667045906770272</v>
+        <v>0.05669120423048122</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0001916137841558003</v>
+        <v>0.001663984636619192</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0135</v>
+        <v>0.0125</v>
       </c>
       <c r="N17" t="n">
-        <v>24.01885986328125</v>
+        <v>22.23968505859375</v>
       </c>
       <c r="O17" t="n">
-        <v>29.42202178338179</v>
+        <v>35.851633366066</v>
       </c>
       <c r="P17" t="n">
-        <v>4.771729493735052e-11</v>
+        <v>4.51091087640196e-11</v>
       </c>
       <c r="Q17" t="n">
-        <v>1782.379762773272</v>
+        <v>1782.911764553223</v>
       </c>
     </row>
     <row r="18">
@@ -1448,40 +1448,40 @@
         <v>3650</v>
       </c>
       <c r="F18" t="n">
-        <v>12.83125968722967</v>
+        <v>9.60066868201886</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5629645986041236</v>
+        <v>0.2593445234930565</v>
       </c>
       <c r="H18" t="n">
-        <v>0.003515507670828946</v>
+        <v>0.002630390563314332</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0001542410030690629</v>
+        <v>7.105519519916787e-05</v>
       </c>
       <c r="J18" t="n">
-        <v>1.396707260296086</v>
+        <v>1.439884857474121</v>
       </c>
       <c r="K18" t="n">
-        <v>0.05635726268570131</v>
+        <v>0.04093645716680879</v>
       </c>
       <c r="L18" t="n">
-        <v>0.0009325137695151844</v>
+        <v>0.0002415233243531928</v>
       </c>
       <c r="M18" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0075</v>
       </c>
       <c r="N18" t="n">
-        <v>31.024169921875</v>
+        <v>27.374267578125</v>
       </c>
       <c r="O18" t="n">
-        <v>38.44768429616745</v>
+        <v>47.93816900205721</v>
       </c>
       <c r="P18" t="n">
-        <v>1.774343353631128e-11</v>
+        <v>1.701087630599641e-11</v>
       </c>
       <c r="Q18" t="n">
-        <v>3644.432330447859</v>
+        <v>3642.55796672938</v>
       </c>
     </row>
     <row r="19">
@@ -1505,40 +1505,40 @@
         <v>4211</v>
       </c>
       <c r="F19" t="n">
-        <v>29.45316993193493</v>
+        <v>26.7963448669328</v>
       </c>
       <c r="G19" t="n">
-        <v>1.068493130930639</v>
+        <v>1.523503310319039</v>
       </c>
       <c r="H19" t="n">
-        <v>0.006993633857461188</v>
+        <v>0.006362772671011986</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0002537129196690955</v>
+        <v>0.0003617547570473498</v>
       </c>
       <c r="J19" t="n">
-        <v>1.054240455752225</v>
+        <v>0.9155110023345389</v>
       </c>
       <c r="K19" t="n">
-        <v>0.03288075129920257</v>
+        <v>0.04264435898252802</v>
       </c>
       <c r="L19" t="n">
-        <v>0.00117551605348218</v>
+        <v>0.002247447669572094</v>
       </c>
       <c r="M19" t="n">
-        <v>0.019</v>
+        <v>0.0175</v>
       </c>
       <c r="N19" t="n">
-        <v>80.01708984374999</v>
+        <v>73.69995117187499</v>
       </c>
       <c r="O19" t="n">
-        <v>23.01318201212892</v>
+        <v>26.85264341342339</v>
       </c>
       <c r="P19" t="n">
-        <v>2.192222132226324e-11</v>
+        <v>2.083924656148668e-11</v>
       </c>
       <c r="Q19" t="n">
-        <v>4210.422772491951</v>
+        <v>4210.276863856082</v>
       </c>
     </row>
     <row r="20">
@@ -1562,40 +1562,40 @@
         <v>1364</v>
       </c>
       <c r="F20" t="n">
-        <v>4.324112552004121</v>
+        <v>3.033334259745948</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1804466842198701</v>
+        <v>0.1805501001931343</v>
       </c>
       <c r="H20" t="n">
-        <v>0.003169855035885259</v>
+        <v>0.002223630805891616</v>
       </c>
       <c r="I20" t="n">
-        <v>0.000132279126365027</v>
+        <v>0.0001323549369827433</v>
       </c>
       <c r="J20" t="n">
-        <v>1.406366121009048</v>
+        <v>1.405155455666326</v>
       </c>
       <c r="K20" t="n">
-        <v>0.05546019479220759</v>
+        <v>0.07607578997560266</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0006551646695073318</v>
+        <v>0.001031079865541631</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0075</v>
+        <v>0.0055</v>
       </c>
       <c r="N20" t="n">
-        <v>10.23101806640625</v>
+        <v>7.502746582031248</v>
       </c>
       <c r="O20" t="n">
-        <v>42.21255991974764</v>
+        <v>56.78861673464202</v>
       </c>
       <c r="P20" t="n">
-        <v>1.71600307853262e-11</v>
+        <v>1.623615066472364e-11</v>
       </c>
       <c r="Q20" t="n">
-        <v>1360.86966387402</v>
+        <v>1361.690454016646</v>
       </c>
     </row>
     <row r="21">
@@ -1619,40 +1619,40 @@
         <v>1776</v>
       </c>
       <c r="F21" t="n">
-        <v>5.771388687597842</v>
+        <v>9.151106894339099</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2101942134629494</v>
+        <v>0.6907282749112966</v>
       </c>
       <c r="H21" t="n">
-        <v>0.003249430661773301</v>
+        <v>0.005152293311232022</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0001183443983978338</v>
+        <v>0.0003888966342318448</v>
       </c>
       <c r="J21" t="n">
-        <v>1.412328663391503</v>
+        <v>0.4232397251775412</v>
       </c>
       <c r="K21" t="n">
-        <v>0.04939513644597964</v>
+        <v>0.07753634883491069</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0006169226326571957</v>
+        <v>2.389388336409196e-05</v>
       </c>
       <c r="M21" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.024</v>
       </c>
       <c r="N21" t="n">
-        <v>15.0970458984375</v>
+        <v>42.62695312499999</v>
       </c>
       <c r="O21" t="n">
-        <v>39.77002884196471</v>
+        <v>52.86667861437866</v>
       </c>
       <c r="P21" t="n">
-        <v>2.101229297986004e-11</v>
+        <v>1.976745565862277e-11</v>
       </c>
       <c r="Q21" t="n">
-        <v>1777.323367602554</v>
+        <v>1776.082548617856</v>
       </c>
     </row>
     <row r="22">
@@ -1676,40 +1676,40 @@
         <v>3607</v>
       </c>
       <c r="F22" t="n">
-        <v>19.88328931692195</v>
+        <v>18.83795214527354</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2461295240289038</v>
+        <v>0.4754896107533951</v>
       </c>
       <c r="H22" t="n">
-        <v>0.005512145721970378</v>
+        <v>0.005222352080341147</v>
       </c>
       <c r="I22" t="n">
-        <v>6.823326771048325e-05</v>
+        <v>0.0001318176274548837</v>
       </c>
       <c r="J22" t="n">
-        <v>1.246398345349658</v>
+        <v>1.102004436959298</v>
       </c>
       <c r="K22" t="n">
-        <v>0.01417945958124356</v>
+        <v>0.02375967644668004</v>
       </c>
       <c r="L22" t="n">
-        <v>0.0001301261287241322</v>
+        <v>0.0004720235663420374</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0155</v>
+        <v>0.0145</v>
       </c>
       <c r="N22" t="n">
-        <v>55.91125488281249</v>
+        <v>52.30407714843749</v>
       </c>
       <c r="O22" t="n">
-        <v>25.50541865779515</v>
+        <v>28.29573562907364</v>
       </c>
       <c r="P22" t="n">
-        <v>3.783068554544835e-11</v>
+        <v>3.67521962382214e-11</v>
       </c>
       <c r="Q22" t="n">
-        <v>3604.758004675124</v>
+        <v>3604.65779914559</v>
       </c>
     </row>
     <row r="23">
@@ -1733,40 +1733,40 @@
         <v>4395</v>
       </c>
       <c r="F23" t="n">
-        <v>15.63666789306943</v>
+        <v>11.0276938261813</v>
       </c>
       <c r="G23" t="n">
-        <v>0.6139322808409924</v>
+        <v>0.3643629379000889</v>
       </c>
       <c r="H23" t="n">
-        <v>0.003558210649445134</v>
+        <v>0.002509412995113257</v>
       </c>
       <c r="I23" t="n">
-        <v>0.0001397037012402614</v>
+        <v>8.291281075770915e-05</v>
       </c>
       <c r="J23" t="n">
-        <v>1.371835470709829</v>
+        <v>1.472075671087335</v>
       </c>
       <c r="K23" t="n">
-        <v>0.04920085661051307</v>
+        <v>0.05192709179797327</v>
       </c>
       <c r="L23" t="n">
-        <v>0.0007264618189268275</v>
+        <v>0.0003259210443666561</v>
       </c>
       <c r="M23" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.007</v>
       </c>
       <c r="N23" t="n">
-        <v>37.35351562499999</v>
+        <v>30.76171874999999</v>
       </c>
       <c r="O23" t="n">
-        <v>39.16627633705617</v>
+        <v>49.48330675147614</v>
       </c>
       <c r="P23" t="n">
-        <v>9.845293129520055e-12</v>
+        <v>9.399595671448294e-12</v>
       </c>
       <c r="Q23" t="n">
-        <v>4390.472362905448</v>
+        <v>4389.147249860212</v>
       </c>
     </row>
     <row r="24">
@@ -1790,40 +1790,40 @@
         <v>1257</v>
       </c>
       <c r="F24" t="n">
-        <v>6.159950049409389</v>
+        <v>5.381061977881228</v>
       </c>
       <c r="G24" t="n">
-        <v>0.2030486871761092</v>
+        <v>0.3365435711089653</v>
       </c>
       <c r="H24" t="n">
-        <v>0.004899253476190459</v>
+        <v>0.004279772788621653</v>
       </c>
       <c r="I24" t="n">
-        <v>0.0001614927034317172</v>
+        <v>0.0002676664984975382</v>
       </c>
       <c r="J24" t="n">
-        <v>1.177873109107223</v>
+        <v>1.053529340380478</v>
       </c>
       <c r="K24" t="n">
-        <v>0.03442875031901588</v>
+        <v>0.06065679945047876</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0009265966075376635</v>
+        <v>0.002166214643397685</v>
       </c>
       <c r="M24" t="n">
-        <v>0.016</v>
+        <v>0.0145</v>
       </c>
       <c r="N24" t="n">
-        <v>20.1171875</v>
+        <v>18.231201171875</v>
       </c>
       <c r="O24" t="n">
-        <v>26.78638101426216</v>
+        <v>32.05041934733295</v>
       </c>
       <c r="P24" t="n">
-        <v>2.689083012062509e-11</v>
+        <v>2.543166777777998e-11</v>
       </c>
       <c r="Q24" t="n">
-        <v>1256.959658401852</v>
+        <v>1256.886955161184</v>
       </c>
     </row>
     <row r="25">
@@ -1841,46 +1841,46 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2578.7353515625</v>
+        <v>1837.158203125</v>
       </c>
       <c r="E25" t="n">
-        <v>2579</v>
+        <v>1837</v>
       </c>
       <c r="F25" t="n">
-        <v>7.628241318316572</v>
+        <v>4.071765875075343</v>
       </c>
       <c r="G25" t="n">
-        <v>0.4484300526328838</v>
+        <v>0.26885998779208</v>
       </c>
       <c r="H25" t="n">
-        <v>0.002958132680693461</v>
+        <v>0.00221633927233337</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0001738953368600514</v>
+        <v>0.0001463455827237687</v>
       </c>
       <c r="J25" t="n">
-        <v>1.470670867844325</v>
+        <v>1.415403855641619</v>
       </c>
       <c r="K25" t="n">
-        <v>0.08363272398763569</v>
+        <v>0.0851631186647574</v>
       </c>
       <c r="L25" t="n">
-        <v>0.001203545420941607</v>
+        <v>0.001284401655880299</v>
       </c>
       <c r="M25" t="n">
-        <v>0.007</v>
+        <v>0.0055</v>
       </c>
       <c r="N25" t="n">
-        <v>18.0511474609375</v>
+        <v>10.1043701171875</v>
       </c>
       <c r="O25" t="n">
-        <v>43.57426733179351</v>
+        <v>58.96841456416316</v>
       </c>
       <c r="P25" t="n">
-        <v>8.757415282657275e-12</v>
+        <v>1.551342266004994e-11</v>
       </c>
       <c r="Q25" t="n">
-        <v>2572.886713729026</v>
+        <v>1839.409458599119</v>
       </c>
     </row>
     <row r="26">
@@ -1898,46 +1898,46 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3567.5048828125</v>
+        <v>2578.7353515625</v>
       </c>
       <c r="E26" t="n">
-        <v>3568</v>
+        <v>2579</v>
       </c>
       <c r="F26" t="n">
-        <v>16.97342499260922</v>
+        <v>5.593086956260102</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1965609959724034</v>
+        <v>0.3098352598119689</v>
       </c>
       <c r="H26" t="n">
-        <v>0.004757786057808547</v>
+        <v>0.002168926312221669</v>
       </c>
       <c r="I26" t="n">
-        <v>5.509761091551509e-05</v>
+        <v>0.0001201500803966698</v>
       </c>
       <c r="J26" t="n">
-        <v>1.28980127584304</v>
+        <v>1.565511876044544</v>
       </c>
       <c r="K26" t="n">
-        <v>0.01426855130046424</v>
+        <v>0.09630729879369919</v>
       </c>
       <c r="L26" t="n">
-        <v>8.938702772880043e-05</v>
+        <v>0.0005829695206930962</v>
       </c>
       <c r="M26" t="n">
-        <v>0.013</v>
+        <v>0.0055</v>
       </c>
       <c r="N26" t="n">
-        <v>46.37756347656249</v>
+        <v>14.18304443359375</v>
       </c>
       <c r="O26" t="n">
-        <v>28.54024203390058</v>
+        <v>56.25049139551957</v>
       </c>
       <c r="P26" t="n">
-        <v>1.757871137128941e-11</v>
+        <v>8.449356218161471e-12</v>
       </c>
       <c r="Q26" t="n">
-        <v>3559.172952959399</v>
+        <v>2569.960344743218</v>
       </c>
     </row>
     <row r="27">
@@ -1947,54 +1947,54 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>tokay_GG3rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1251.220703125</v>
+        <v>3567.5048828125</v>
       </c>
       <c r="E27" t="n">
-        <v>1251</v>
+        <v>3568</v>
       </c>
       <c r="F27" t="n">
-        <v>6.968943536799011</v>
+        <v>15.54468695639827</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2097396321474185</v>
+        <v>0.4096938192712757</v>
       </c>
       <c r="H27" t="n">
-        <v>0.005569715653995854</v>
+        <v>0.004357299419908115</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0001676280064928442</v>
+        <v>0.0001148404368681024</v>
       </c>
       <c r="J27" t="n">
-        <v>1.128208953686543</v>
+        <v>1.154408958598312</v>
       </c>
       <c r="K27" t="n">
-        <v>0.02890609544874574</v>
+        <v>0.02729239579873916</v>
       </c>
       <c r="L27" t="n">
-        <v>0.0008208035871424071</v>
+        <v>0.0004249786484322232</v>
       </c>
       <c r="M27" t="n">
-        <v>0.0165</v>
+        <v>0.0125</v>
       </c>
       <c r="N27" t="n">
-        <v>20.6451416015625</v>
+        <v>44.59381103515625</v>
       </c>
       <c r="O27" t="n">
-        <v>24.92820201618651</v>
+        <v>32.69500667980406</v>
       </c>
       <c r="P27" t="n">
-        <v>3.834120878250849e-11</v>
+        <v>1.697534074561853e-11</v>
       </c>
       <c r="Q27" t="n">
-        <v>1251.287838447055</v>
+        <v>3558.719716264305</v>
       </c>
     </row>
     <row r="28">
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2590.9423828125</v>
+        <v>1251.220703125</v>
       </c>
       <c r="E28" t="n">
-        <v>2591</v>
+        <v>1251</v>
       </c>
       <c r="F28" t="n">
-        <v>10.98963182361519</v>
+        <v>6.368678876598986</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3092448683018977</v>
+        <v>0.3783197927481377</v>
       </c>
       <c r="H28" t="n">
-        <v>0.004241557780874234</v>
+        <v>0.00508997242508282</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0001193561347999598</v>
+        <v>0.0003023605602139262</v>
       </c>
       <c r="J28" t="n">
-        <v>1.32768769695136</v>
+        <v>0.9838123412829922</v>
       </c>
       <c r="K28" t="n">
-        <v>0.03276803607911022</v>
+        <v>0.05114370766409176</v>
       </c>
       <c r="L28" t="n">
-        <v>0.0005233411782563589</v>
+        <v>0.002185769896091414</v>
       </c>
       <c r="M28" t="n">
-        <v>0.0105</v>
+        <v>0.016</v>
       </c>
       <c r="N28" t="n">
-        <v>27.20489501953125</v>
+        <v>20.01953125</v>
       </c>
       <c r="O28" t="n">
-        <v>31.27955333718139</v>
+        <v>28.95706481259828</v>
       </c>
       <c r="P28" t="n">
-        <v>2.053361281504691e-11</v>
+        <v>3.658261502826922e-11</v>
       </c>
       <c r="Q28" t="n">
-        <v>2591.805130181283</v>
+        <v>1251.313681664363</v>
       </c>
     </row>
     <row r="29">
@@ -2069,46 +2069,46 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3216.552734375</v>
+        <v>2590.9423828125</v>
       </c>
       <c r="E29" t="n">
-        <v>3217</v>
+        <v>2591</v>
       </c>
       <c r="F29" t="n">
-        <v>10.18586891539348</v>
+        <v>9.218817703152384</v>
       </c>
       <c r="G29" t="n">
-        <v>0.5054175690872295</v>
+        <v>0.2736022388606677</v>
       </c>
       <c r="H29" t="n">
-        <v>0.003166703535290452</v>
+        <v>0.003558094446370993</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0001571301983287508</v>
+        <v>0.0001055995072200985</v>
       </c>
       <c r="J29" t="n">
-        <v>1.439482130378261</v>
+        <v>1.227992132995891</v>
       </c>
       <c r="K29" t="n">
-        <v>0.06753790519768502</v>
+        <v>0.03500157882271466</v>
       </c>
       <c r="L29" t="n">
-        <v>0.0009697510280074862</v>
+        <v>0.0004442429373882437</v>
       </c>
       <c r="M29" t="n">
-        <v>0.0075</v>
+        <v>0.011</v>
       </c>
       <c r="N29" t="n">
-        <v>24.1241455078125</v>
+        <v>28.50036621093749</v>
       </c>
       <c r="O29" t="n">
-        <v>40.60474868382574</v>
+        <v>37.0862902571676</v>
       </c>
       <c r="P29" t="n">
-        <v>5.761462717113044e-12</v>
+        <v>1.963012563946387e-11</v>
       </c>
       <c r="Q29" t="n">
-        <v>3220.389925054321</v>
+        <v>2591.032561350483</v>
       </c>
     </row>
     <row r="30">
@@ -2126,103 +2126,103 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>3582.763671875</v>
+        <v>3216.552734375</v>
       </c>
       <c r="E30" t="n">
-        <v>3583</v>
+        <v>3217</v>
       </c>
       <c r="F30" t="n">
-        <v>14.31809874100298</v>
+        <v>7.332464020819553</v>
       </c>
       <c r="G30" t="n">
-        <v>0.4232403169228528</v>
+        <v>0.3479640214599756</v>
       </c>
       <c r="H30" t="n">
-        <v>0.003996383812139571</v>
+        <v>0.00227960323561874</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0001181323569414654</v>
+        <v>0.0001081791750967788</v>
       </c>
       <c r="J30" t="n">
-        <v>1.348669525122197</v>
+        <v>1.538314863474834</v>
       </c>
       <c r="K30" t="n">
-        <v>0.03562087547215192</v>
+        <v>0.08007424436075428</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0005381260333174574</v>
+        <v>0.0005153658984501136</v>
       </c>
       <c r="M30" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="N30" t="n">
-        <v>35.82763671874999</v>
+        <v>19.29931640625</v>
       </c>
       <c r="O30" t="n">
-        <v>33.43948673382051</v>
+        <v>52.06785164383463</v>
       </c>
       <c r="P30" t="n">
-        <v>1.950103839622597e-11</v>
+        <v>5.500357191301378e-12</v>
       </c>
       <c r="Q30" t="n">
-        <v>3584.025592853023</v>
+        <v>3221.708715369164</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Tokay</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4350.5859375</v>
+        <v>3582.763671875</v>
       </c>
       <c r="E31" t="n">
-        <v>4351</v>
+        <v>3583</v>
       </c>
       <c r="F31" t="n">
-        <v>6.200537234175052</v>
+        <v>11.78210271864684</v>
       </c>
       <c r="G31" t="n">
-        <v>0.503620119972046</v>
+        <v>0.2179051485751409</v>
       </c>
       <c r="H31" t="n">
-        <v>0.001425218883904658</v>
+        <v>0.003288551464093864</v>
       </c>
       <c r="I31" t="n">
-        <v>0.000115759147665853</v>
+        <v>6.082040807930339e-05</v>
       </c>
       <c r="J31" t="n">
-        <v>1.556984711577556</v>
+        <v>1.332271550521036</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1342492179820402</v>
+        <v>0.02401674671209849</v>
       </c>
       <c r="L31" t="n">
-        <v>0.0006445582041643389</v>
+        <v>0.0001628962640967826</v>
       </c>
       <c r="M31" t="n">
-        <v>0.0035</v>
+        <v>0.0095</v>
       </c>
       <c r="N31" t="n">
-        <v>15.22705078125</v>
+        <v>34.03625488281249</v>
       </c>
       <c r="O31" t="n">
-        <v>87.64883889212321</v>
+        <v>38.90485458695645</v>
       </c>
       <c r="P31" t="n">
-        <v>1.806475847363449e-13</v>
+        <v>1.885060989571352e-11</v>
       </c>
       <c r="Q31" t="n">
-        <v>4347.72734487957</v>
+        <v>3584.419331591613</v>
       </c>
     </row>
     <row r="32">
@@ -2240,46 +2240,46 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>7453.125</v>
+        <v>4350.5859375</v>
       </c>
       <c r="E32" t="n">
-        <v>7453</v>
+        <v>4351</v>
       </c>
       <c r="F32" t="n">
-        <v>13.52609931227873</v>
+        <v>115.1988483164157</v>
       </c>
       <c r="G32" t="n">
-        <v>0.3830227078285064</v>
+        <v>20.180063086368</v>
       </c>
       <c r="H32" t="n">
-        <v>0.001814822549236559</v>
+        <v>0.02647892720000218</v>
       </c>
       <c r="I32" t="n">
-        <v>5.139088742353127e-05</v>
+        <v>0.00463847016844912</v>
       </c>
       <c r="J32" t="n">
-        <v>1.387782360319679</v>
+        <v>0.01724117341343154</v>
       </c>
       <c r="K32" t="n">
-        <v>0.03911632563287751</v>
+        <v>0.002222354963986682</v>
       </c>
       <c r="L32" t="n">
-        <v>0.0001643147067307164</v>
+        <v>1.072628946602527e-05</v>
       </c>
       <c r="M32" t="n">
-        <v>0.005</v>
+        <v>0.0395</v>
       </c>
       <c r="N32" t="n">
-        <v>37.265625</v>
+        <v>171.84814453125</v>
       </c>
       <c r="O32" t="n">
-        <v>68.22161768748448</v>
+        <v>87.64883889212321</v>
       </c>
       <c r="P32" t="n">
-        <v>6.30085870083755e-13</v>
+        <v>1.806475847363449e-13</v>
       </c>
       <c r="Q32" t="n">
-        <v>7456.907112586428</v>
+        <v>4347.72734487957</v>
       </c>
     </row>
     <row r="33">
@@ -2297,46 +2297,46 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>8452.1484375</v>
+        <v>7453.125</v>
       </c>
       <c r="E33" t="n">
-        <v>8452</v>
+        <v>7453</v>
       </c>
       <c r="F33" t="n">
-        <v>17.85863955129348</v>
+        <v>13.04145525992646</v>
       </c>
       <c r="G33" t="n">
-        <v>0.7019742548644242</v>
+        <v>0.4442107380035411</v>
       </c>
       <c r="H33" t="n">
-        <v>0.002112911253671233</v>
+        <v>0.001749796932149462</v>
       </c>
       <c r="I33" t="n">
-        <v>8.30527599053923e-05</v>
+        <v>5.960060216399713e-05</v>
       </c>
       <c r="J33" t="n">
-        <v>1.370490614141937</v>
+        <v>1.416558291439019</v>
       </c>
       <c r="K33" t="n">
-        <v>0.05037830177731586</v>
+        <v>0.04900115219581488</v>
       </c>
       <c r="L33" t="n">
-        <v>0.0004109910990382773</v>
+        <v>0.0002381471114821577</v>
       </c>
       <c r="M33" t="n">
-        <v>0.0055</v>
+        <v>0.005</v>
       </c>
       <c r="N33" t="n">
-        <v>46.48681640625</v>
+        <v>37.265625</v>
       </c>
       <c r="O33" t="n">
-        <v>60.09398519868756</v>
+        <v>68.22161768748448</v>
       </c>
       <c r="P33" t="n">
-        <v>1.784690547665494e-12</v>
+        <v>6.30085870083755e-13</v>
       </c>
       <c r="Q33" t="n">
-        <v>8445.060419516562</v>
+        <v>7456.907112586428</v>
       </c>
     </row>
     <row r="34">
@@ -2354,46 +2354,46 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>9026.3671875</v>
+        <v>8452.1484375</v>
       </c>
       <c r="E34" t="n">
-        <v>9026</v>
+        <v>8452</v>
       </c>
       <c r="F34" t="n">
-        <v>25.26965690636864</v>
+        <v>17.87606543006282</v>
       </c>
       <c r="G34" t="n">
-        <v>0.4451316147322679</v>
+        <v>0.612070537767026</v>
       </c>
       <c r="H34" t="n">
-        <v>0.002799537885115383</v>
+        <v>0.002114972963649258</v>
       </c>
       <c r="I34" t="n">
-        <v>4.931459195995264e-05</v>
+        <v>7.241597119277119e-05</v>
       </c>
       <c r="J34" t="n">
-        <v>1.21040516136573</v>
+        <v>1.359274081391985</v>
       </c>
       <c r="K34" t="n">
-        <v>0.01878987637047191</v>
+        <v>0.04350143861619726</v>
       </c>
       <c r="L34" t="n">
-        <v>0.0001291071634474768</v>
+        <v>0.0003070184462743492</v>
       </c>
       <c r="M34" t="n">
-        <v>0.008</v>
+        <v>0.0055</v>
       </c>
       <c r="N34" t="n">
-        <v>72.2109375</v>
+        <v>46.48681640625</v>
       </c>
       <c r="O34" t="n">
-        <v>48.17177549386727</v>
+        <v>60.09398519868756</v>
       </c>
       <c r="P34" t="n">
-        <v>2.045822095595467e-12</v>
+        <v>1.784690547665494e-12</v>
       </c>
       <c r="Q34" t="n">
-        <v>9030.795774783386</v>
+        <v>8445.060419516562</v>
       </c>
     </row>
     <row r="35">
@@ -2403,54 +2403,54 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6837.890625</v>
+        <v>9026.3671875</v>
       </c>
       <c r="E35" t="n">
-        <v>6838</v>
+        <v>9026</v>
       </c>
       <c r="F35" t="n">
-        <v>10.5977698983937</v>
+        <v>24.59390654983015</v>
       </c>
       <c r="G35" t="n">
-        <v>0.6331896030148532</v>
+        <v>0.5009153151522551</v>
       </c>
       <c r="H35" t="n">
-        <v>0.00154985952241576</v>
+        <v>0.002724673840422598</v>
       </c>
       <c r="I35" t="n">
-        <v>9.260013617355179e-05</v>
+        <v>5.549467518293943e-05</v>
       </c>
       <c r="J35" t="n">
-        <v>1.489588780119523</v>
+        <v>1.221734076400344</v>
       </c>
       <c r="K35" t="n">
-        <v>0.09255996511278757</v>
+        <v>0.02217732678694127</v>
       </c>
       <c r="L35" t="n">
-        <v>0.0004790623519389627</v>
+        <v>0.0001714846673462065</v>
       </c>
       <c r="M35" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
       <c r="N35" t="n">
-        <v>27.3515625</v>
+        <v>72.2109375</v>
       </c>
       <c r="O35" t="n">
-        <v>76.67818748697763</v>
+        <v>48.17177549386727</v>
       </c>
       <c r="P35" t="n">
-        <v>3.885635794226587e-13</v>
+        <v>2.045822095595467e-12</v>
       </c>
       <c r="Q35" t="n">
-        <v>6840.757442741772</v>
+        <v>9030.795774783386</v>
       </c>
     </row>
     <row r="36">
@@ -2468,46 +2468,46 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>7901.3671875</v>
+        <v>6837.890625</v>
       </c>
       <c r="E36" t="n">
-        <v>7901</v>
+        <v>6838</v>
       </c>
       <c r="F36" t="n">
-        <v>19.12436303910451</v>
+        <v>10.48075862048517</v>
       </c>
       <c r="G36" t="n">
-        <v>1.032548472683028</v>
+        <v>0.6783872851377761</v>
       </c>
       <c r="H36" t="n">
-        <v>0.002420386571751701</v>
+        <v>0.001532747333244332</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0001306797226581906</v>
+        <v>9.921002284791243e-05</v>
       </c>
       <c r="J36" t="n">
-        <v>1.174421851631025</v>
+        <v>1.510585900741471</v>
       </c>
       <c r="K36" t="n">
-        <v>0.05926269821551847</v>
+        <v>0.1024079021141574</v>
       </c>
       <c r="L36" t="n">
-        <v>0.0009800467979355896</v>
+        <v>0.000571796373326826</v>
       </c>
       <c r="M36" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="N36" t="n">
-        <v>63.2109375</v>
+        <v>27.3515625</v>
       </c>
       <c r="O36" t="n">
-        <v>51.7303391195944</v>
+        <v>76.67818748697763</v>
       </c>
       <c r="P36" t="n">
-        <v>6.977991565512491e-13</v>
+        <v>3.885635794226587e-13</v>
       </c>
       <c r="Q36" t="n">
-        <v>7901.190467312519</v>
+        <v>6840.757442741772</v>
       </c>
     </row>
     <row r="37">
@@ -2525,46 +2525,46 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8835.9375</v>
+        <v>7901.3671875</v>
       </c>
       <c r="E37" t="n">
-        <v>8836</v>
+        <v>7901</v>
       </c>
       <c r="F37" t="n">
-        <v>22.98015480698477</v>
+        <v>19.07932362556879</v>
       </c>
       <c r="G37" t="n">
-        <v>0.678522834599649</v>
+        <v>0.9602732732386496</v>
       </c>
       <c r="H37" t="n">
-        <v>0.002600760225724183</v>
+        <v>0.002414686366652137</v>
       </c>
       <c r="I37" t="n">
-        <v>7.679126686892579e-05</v>
+        <v>0.0001215325462608302</v>
       </c>
       <c r="J37" t="n">
-        <v>1.215681358694547</v>
+        <v>1.184848100345372</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0326037303704333</v>
+        <v>0.05578656082435941</v>
       </c>
       <c r="L37" t="n">
-        <v>0.0003405400154561213</v>
+        <v>0.000864390475711705</v>
       </c>
       <c r="M37" t="n">
         <v>0.008</v>
       </c>
       <c r="N37" t="n">
-        <v>70.6875</v>
+        <v>63.2109375</v>
       </c>
       <c r="O37" t="n">
-        <v>49.42569815474504</v>
+        <v>51.7303391195944</v>
       </c>
       <c r="P37" t="n">
-        <v>1.292541591210098e-12</v>
+        <v>6.977991565512491e-13</v>
       </c>
       <c r="Q37" t="n">
-        <v>8845.361149512852</v>
+        <v>7901.190467312519</v>
       </c>
     </row>
     <row r="38">
@@ -2582,46 +2582,46 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>9257.8125</v>
+        <v>8835.9375</v>
       </c>
       <c r="E38" t="n">
-        <v>9258</v>
+        <v>8836</v>
       </c>
       <c r="F38" t="n">
-        <v>57.96893269989882</v>
+        <v>23.29466516449487</v>
       </c>
       <c r="G38" t="n">
-        <v>6.118874950467526</v>
+        <v>0.6654409542995549</v>
       </c>
       <c r="H38" t="n">
-        <v>0.006261623110200042</v>
+        <v>0.002636354678209852</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0006609417668015556</v>
+        <v>7.531073576511319e-05</v>
       </c>
       <c r="J38" t="n">
-        <v>0.06859142883780221</v>
+        <v>1.197820997357748</v>
       </c>
       <c r="K38" t="n">
-        <v>0.009411778969351539</v>
+        <v>0.03090963143457713</v>
       </c>
       <c r="L38" t="n">
-        <v>6.093241765296857e-06</v>
+        <v>0.0003138516197605542</v>
       </c>
       <c r="M38" t="n">
-        <v>0.0145</v>
+        <v>0.008</v>
       </c>
       <c r="N38" t="n">
-        <v>134.23828125</v>
+        <v>70.6875</v>
       </c>
       <c r="O38" t="n">
-        <v>89.73515677713675</v>
+        <v>49.42569815474504</v>
       </c>
       <c r="P38" t="n">
-        <v>7.664901288177202e-13</v>
+        <v>1.292541591210098e-12</v>
       </c>
       <c r="Q38" t="n">
-        <v>9253.893064877439</v>
+        <v>8845.361149512852</v>
       </c>
     </row>
     <row r="39">
@@ -2631,54 +2631,54 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5625.54931640625</v>
+        <v>9257.8125</v>
       </c>
       <c r="E39" t="n">
-        <v>5626</v>
+        <v>9258</v>
       </c>
       <c r="F39" t="n">
-        <v>13.7025908628672</v>
+        <v>180.2095390736592</v>
       </c>
       <c r="G39" t="n">
-        <v>1.23349974496892</v>
+        <v>50.37301973358876</v>
       </c>
       <c r="H39" t="n">
-        <v>0.002435778284425524</v>
+        <v>0.01946567173116319</v>
       </c>
       <c r="I39" t="n">
-        <v>0.0002192674307149995</v>
+        <v>0.005441136308775832</v>
       </c>
       <c r="J39" t="n">
-        <v>1.123193040757176</v>
+        <v>0.01402270471350458</v>
       </c>
       <c r="K39" t="n">
-        <v>0.09542756147256611</v>
+        <v>0.002534390042048344</v>
       </c>
       <c r="L39" t="n">
-        <v>0.002768955551456496</v>
+        <v>6.619561169739156e-06</v>
       </c>
       <c r="M39" t="n">
-        <v>0.009501133786848073</v>
+        <v>0.0225</v>
       </c>
       <c r="N39" t="n">
-        <v>53.4490966796875</v>
+        <v>208.30078125</v>
       </c>
       <c r="O39" t="n">
-        <v>55.38194222549402</v>
+        <v>89.73515677713675</v>
       </c>
       <c r="P39" t="n">
-        <v>7.975997509325952e-11</v>
+        <v>7.664901288177202e-13</v>
       </c>
       <c r="Q39" t="n">
-        <v>5623.316734238025</v>
+        <v>9253.893064877439</v>
       </c>
     </row>
     <row r="40">
@@ -2696,46 +2696,46 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8096.484375</v>
+        <v>5625.54931640625</v>
       </c>
       <c r="E40" t="n">
-        <v>8096</v>
+        <v>5626</v>
       </c>
       <c r="F40" t="n">
-        <v>16.61126643733448</v>
+        <v>12.60965856631775</v>
       </c>
       <c r="G40" t="n">
-        <v>0.3634184788855256</v>
+        <v>1.026096584491348</v>
       </c>
       <c r="H40" t="n">
-        <v>0.002051664113454734</v>
+        <v>0.002241498182149638</v>
       </c>
       <c r="I40" t="n">
-        <v>4.488596062850125e-05</v>
+        <v>0.0001823993581389214</v>
       </c>
       <c r="J40" t="n">
-        <v>1.326748703747682</v>
+        <v>1.180994347802232</v>
       </c>
       <c r="K40" t="n">
-        <v>0.0279915396108054</v>
+        <v>0.0930796047895663</v>
       </c>
       <c r="L40" t="n">
-        <v>0.0001302866375262261</v>
+        <v>0.002167337050029934</v>
       </c>
       <c r="M40" t="n">
-        <v>0.00600907029478458</v>
+        <v>0.009002267573696146</v>
       </c>
       <c r="N40" t="n">
-        <v>48.65234375</v>
+        <v>50.6427001953125</v>
       </c>
       <c r="O40" t="n">
-        <v>58.78366132431848</v>
+        <v>55.38194222549402</v>
       </c>
       <c r="P40" t="n">
-        <v>1.299537582437962e-10</v>
+        <v>7.975997509325952e-11</v>
       </c>
       <c r="Q40" t="n">
-        <v>8098.586383255675</v>
+        <v>5623.316734238025</v>
       </c>
     </row>
     <row r="41">
@@ -2753,46 +2753,46 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>8489.46533203125</v>
+        <v>8096.484375</v>
       </c>
       <c r="E41" t="n">
-        <v>8489</v>
+        <v>8096</v>
       </c>
       <c r="F41" t="n">
-        <v>54.8932366315176</v>
+        <v>16.65054003882637</v>
       </c>
       <c r="G41" t="n">
-        <v>2.019460731392774</v>
+        <v>0.4482449422709035</v>
       </c>
       <c r="H41" t="n">
-        <v>0.006466041674544828</v>
+        <v>0.002056514811569233</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0002378784354973723</v>
+        <v>5.536291080298707e-05</v>
       </c>
       <c r="J41" t="n">
-        <v>0.842857790203811</v>
+        <v>1.321354983293454</v>
       </c>
       <c r="K41" t="n">
-        <v>0.02437092987453587</v>
+        <v>0.03467666693226418</v>
       </c>
       <c r="L41" t="n">
-        <v>0.0006957767539891147</v>
+        <v>0.0002134138670315013</v>
       </c>
       <c r="M41" t="n">
-        <v>0.01501133786848073</v>
+        <v>0.006507936507936508</v>
       </c>
       <c r="N41" t="n">
-        <v>127.438232421875</v>
+        <v>52.69140625</v>
       </c>
       <c r="O41" t="n">
-        <v>24.82765613524692</v>
+        <v>58.78366132431848</v>
       </c>
       <c r="P41" t="n">
-        <v>3.706405454296643e-10</v>
+        <v>1.299537582437962e-10</v>
       </c>
       <c r="Q41" t="n">
-        <v>8486.907248855707</v>
+        <v>8098.586383255675</v>
       </c>
     </row>
     <row r="42">
@@ -2810,46 +2810,46 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9864.898681640625</v>
+        <v>8489.46533203125</v>
       </c>
       <c r="E42" t="n">
-        <v>9865</v>
+        <v>8489</v>
       </c>
       <c r="F42" t="n">
-        <v>17.55744318502499</v>
+        <v>56.58543102684771</v>
       </c>
       <c r="G42" t="n">
-        <v>0.7706878262572214</v>
+        <v>2.137975810440625</v>
       </c>
       <c r="H42" t="n">
-        <v>0.001779789509414913</v>
+        <v>0.006665370410707441</v>
       </c>
       <c r="I42" t="n">
-        <v>7.812425156393484e-05</v>
+        <v>0.0002518386879293702</v>
       </c>
       <c r="J42" t="n">
-        <v>1.430540075178475</v>
+        <v>0.8352317995237064</v>
       </c>
       <c r="K42" t="n">
-        <v>0.06310040276667497</v>
+        <v>0.0248886758930339</v>
       </c>
       <c r="L42" t="n">
-        <v>0.0004119904486747436</v>
+        <v>0.0007846416822270095</v>
       </c>
       <c r="M42" t="n">
-        <v>0.005011337868480726</v>
+        <v>0.01600907029478458</v>
       </c>
       <c r="N42" t="n">
-        <v>49.43634033203125</v>
+        <v>135.908447265625</v>
       </c>
       <c r="O42" t="n">
-        <v>63.90181081181339</v>
+        <v>24.82765613524692</v>
       </c>
       <c r="P42" t="n">
-        <v>9.69195629278402e-11</v>
+        <v>3.706405454296643e-10</v>
       </c>
       <c r="Q42" t="n">
-        <v>9856.932898275971</v>
+        <v>8486.907248855707</v>
       </c>
     </row>
     <row r="43">
@@ -2859,54 +2859,54 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4944.561767578125</v>
+        <v>9864.898681640625</v>
       </c>
       <c r="E43" t="n">
-        <v>4945</v>
+        <v>9865</v>
       </c>
       <c r="F43" t="n">
-        <v>7.915838219591966</v>
+        <v>18.26594601669812</v>
       </c>
       <c r="G43" t="n">
-        <v>0.3683099505358468</v>
+        <v>0.5678164452643107</v>
       </c>
       <c r="H43" t="n">
-        <v>0.001600918057389177</v>
+        <v>0.001851610098205319</v>
       </c>
       <c r="I43" t="n">
-        <v>7.448788544838973e-05</v>
+        <v>5.755927796005276e-05</v>
       </c>
       <c r="J43" t="n">
-        <v>1.484261017007512</v>
+        <v>1.378394255452227</v>
       </c>
       <c r="K43" t="n">
-        <v>0.07218371225140059</v>
+        <v>0.04341424078883844</v>
       </c>
       <c r="L43" t="n">
-        <v>0.000374978253079178</v>
+        <v>0.0002511172197664648</v>
       </c>
       <c r="M43" t="n">
-        <v>0.004489795918367347</v>
+        <v>0.00600907029478458</v>
       </c>
       <c r="N43" t="n">
-        <v>22.2000732421875</v>
+        <v>59.27886962890625</v>
       </c>
       <c r="O43" t="n">
-        <v>73.82638021620554</v>
+        <v>63.90181081181339</v>
       </c>
       <c r="P43" t="n">
-        <v>4.610246676062042e-11</v>
+        <v>9.69195629278402e-11</v>
       </c>
       <c r="Q43" t="n">
-        <v>4954.457814883755</v>
+        <v>9856.932898275971</v>
       </c>
     </row>
     <row r="44">
@@ -2924,46 +2924,46 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>5768.206787109375</v>
+        <v>4944.561767578125</v>
       </c>
       <c r="E44" t="n">
-        <v>5768</v>
+        <v>4945</v>
       </c>
       <c r="F44" t="n">
-        <v>31.92543080459712</v>
+        <v>7.800303666230374</v>
       </c>
       <c r="G44" t="n">
-        <v>2.402161376318801</v>
+        <v>0.3863270020012606</v>
       </c>
       <c r="H44" t="n">
-        <v>0.005534723698870014</v>
+        <v>0.001577552072941544</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0004164485541134001</v>
+        <v>7.813169703621395e-05</v>
       </c>
       <c r="J44" t="n">
-        <v>0.8224411756415669</v>
+        <v>1.489400138311102</v>
       </c>
       <c r="K44" t="n">
-        <v>0.04763836043567797</v>
+        <v>0.07776616742319931</v>
       </c>
       <c r="L44" t="n">
-        <v>0.003106225350922567</v>
+        <v>0.0004205819049202851</v>
       </c>
       <c r="M44" t="n">
-        <v>0.01501133786848073</v>
+        <v>0.004489795918367347</v>
       </c>
       <c r="N44" t="n">
-        <v>86.5885009765625</v>
+        <v>22.2000732421875</v>
       </c>
       <c r="O44" t="n">
-        <v>26.63568621305765</v>
+        <v>73.82638021620554</v>
       </c>
       <c r="P44" t="n">
-        <v>2.037326814883841e-10</v>
+        <v>4.610246676062042e-11</v>
       </c>
       <c r="Q44" t="n">
-        <v>5766.206632270292</v>
+        <v>4954.457814883755</v>
       </c>
     </row>
     <row r="45">
@@ -2981,46 +2981,46 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>7184.014892578125</v>
+        <v>5768.206787109375</v>
       </c>
       <c r="E45" t="n">
-        <v>7184</v>
+        <v>5768</v>
       </c>
       <c r="F45" t="n">
-        <v>236.2795024146108</v>
+        <v>31.38676581665101</v>
       </c>
       <c r="G45" t="n">
-        <v>2.40489004794071</v>
+        <v>2.251175744832769</v>
       </c>
       <c r="H45" t="n">
-        <v>0.03288961756729004</v>
+        <v>0.005441338526003136</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0003347557158358936</v>
+        <v>0.0003902730654288665</v>
       </c>
       <c r="J45" t="n">
-        <v>0.9717468225374449</v>
+        <v>0.8275396610434489</v>
       </c>
       <c r="K45" t="n">
-        <v>0.006551192460712446</v>
+        <v>0.04620054180818002</v>
       </c>
       <c r="L45" t="n">
-        <v>0.0004427735154623166</v>
+        <v>0.002893821402532026</v>
       </c>
       <c r="M45" t="n">
-        <v>0.06448979591836734</v>
+        <v>0.01551020408163265</v>
       </c>
       <c r="N45" t="n">
-        <v>463.295654296875</v>
+        <v>89.466064453125</v>
       </c>
       <c r="O45" t="n">
-        <v>5.600274938598027</v>
+        <v>26.63568621305765</v>
       </c>
       <c r="P45" t="n">
-        <v>5.484176416186218e-09</v>
+        <v>2.037326814883841e-10</v>
       </c>
       <c r="Q45" t="n">
-        <v>7182.063356605612</v>
+        <v>5766.206632270292</v>
       </c>
     </row>
     <row r="46">
@@ -3038,103 +3038,103 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9633.416748046875</v>
+        <v>7184.014892578125</v>
       </c>
       <c r="E46" t="n">
-        <v>9633</v>
+        <v>7184</v>
       </c>
       <c r="F46" t="n">
-        <v>135.779151684903</v>
+        <v>234.943036872391</v>
       </c>
       <c r="G46" t="n">
-        <v>1.304228554709577</v>
+        <v>2.437155275047116</v>
       </c>
       <c r="H46" t="n">
-        <v>0.01409459958352072</v>
+        <v>0.0327035843306941</v>
       </c>
       <c r="I46" t="n">
-        <v>0.0001353858748998897</v>
+        <v>0.0003392469686504917</v>
       </c>
       <c r="J46" t="n">
-        <v>0.9042606428263641</v>
+        <v>0.9729455183625914</v>
       </c>
       <c r="K46" t="n">
-        <v>0.00619267527097353</v>
+        <v>0.0067193260855411</v>
       </c>
       <c r="L46" t="n">
-        <v>0.0001631920864378598</v>
+        <v>0.0004650896889898434</v>
       </c>
       <c r="M46" t="n">
-        <v>0.03299319727891156</v>
+        <v>0.06498866213151927</v>
       </c>
       <c r="N46" t="n">
-        <v>317.8372192382812</v>
+        <v>466.8795166015624</v>
       </c>
       <c r="O46" t="n">
-        <v>12.07424623307133</v>
+        <v>5.600274938598027</v>
       </c>
       <c r="P46" t="n">
-        <v>1.899439743021853e-09</v>
+        <v>5.484176416186218e-09</v>
       </c>
       <c r="Q46" t="n">
-        <v>9634.460544446882</v>
+        <v>7182.063356605612</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Human</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2804.69970703125</v>
+        <v>9633.416748046875</v>
       </c>
       <c r="E47" t="n">
-        <v>2805</v>
+        <v>9633</v>
       </c>
       <c r="F47" t="n">
-        <v>112.1591857637033</v>
+        <v>133.1388996670538</v>
       </c>
       <c r="G47" t="n">
-        <v>3.116989985832063</v>
+        <v>1.162136887522884</v>
       </c>
       <c r="H47" t="n">
-        <v>0.03998973062339813</v>
+        <v>0.01382052735277408</v>
       </c>
       <c r="I47" t="n">
-        <v>0.001111345352950947</v>
+        <v>0.0001206360025645627</v>
       </c>
       <c r="J47" t="n">
-        <v>0.7874208216893995</v>
+        <v>0.9099152783636083</v>
       </c>
       <c r="K47" t="n">
-        <v>0.01618327782969985</v>
+        <v>0.005631538189497031</v>
       </c>
       <c r="L47" t="n">
-        <v>0.003078120742162101</v>
+        <v>0.0001298070213976185</v>
       </c>
       <c r="M47" t="n">
-        <v>0.1009977324263039</v>
+        <v>0.03149659863945578</v>
       </c>
       <c r="N47" t="n">
-        <v>283.268310546875</v>
+        <v>303.4198608398438</v>
       </c>
       <c r="O47" t="n">
-        <v>4.548385840690079</v>
+        <v>12.07424623307133</v>
       </c>
       <c r="P47" t="n">
-        <v>7.782864418659612e-12</v>
+        <v>1.899439743021853e-09</v>
       </c>
       <c r="Q47" t="n">
-        <v>2804.093986490997</v>
+        <v>9634.460544446882</v>
       </c>
     </row>
     <row r="48">
@@ -3152,46 +3152,46 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2941.973876953125</v>
+        <v>2804.69970703125</v>
       </c>
       <c r="E48" t="n">
-        <v>2942</v>
+        <v>2805</v>
       </c>
       <c r="F48" t="n">
-        <v>204.8053250741048</v>
+        <v>112.5746103350534</v>
       </c>
       <c r="G48" t="n">
-        <v>2.090545044013624</v>
+        <v>3.128881747718502</v>
       </c>
       <c r="H48" t="n">
-        <v>0.06961493665137938</v>
+        <v>0.04013784793175332</v>
       </c>
       <c r="I48" t="n">
-        <v>0.0007105926603871516</v>
+        <v>0.001115585294166981</v>
       </c>
       <c r="J48" t="n">
-        <v>0.8108312609039502</v>
+        <v>0.7874327304752416</v>
       </c>
       <c r="K48" t="n">
-        <v>0.005845507158385367</v>
+        <v>0.01616607615446883</v>
       </c>
       <c r="L48" t="n">
-        <v>0.0007536322401791502</v>
+        <v>0.003084484398494552</v>
       </c>
       <c r="M48" t="n">
-        <v>0.16</v>
+        <v>0.1009977324263039</v>
       </c>
       <c r="N48" t="n">
-        <v>470.7158203125</v>
+        <v>283.268310546875</v>
       </c>
       <c r="O48" t="n">
-        <v>3.385749687296979</v>
+        <v>4.548385840690079</v>
       </c>
       <c r="P48" t="n">
-        <v>1.649522971510552e-11</v>
+        <v>7.782864418659612e-12</v>
       </c>
       <c r="Q48" t="n">
-        <v>2943.013811279915</v>
+        <v>2804.093986490997</v>
       </c>
     </row>
     <row r="49">
@@ -3209,46 +3209,46 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3862.518310546875</v>
+        <v>2941.973876953125</v>
       </c>
       <c r="E49" t="n">
-        <v>3863</v>
+        <v>2942</v>
       </c>
       <c r="F49" t="n">
-        <v>342.0198920001052</v>
+        <v>205.8300272615321</v>
       </c>
       <c r="G49" t="n">
-        <v>2.265109638389958</v>
+        <v>2.104950987964815</v>
       </c>
       <c r="H49" t="n">
-        <v>0.08854841958061302</v>
+        <v>0.06996324096347901</v>
       </c>
       <c r="I49" t="n">
-        <v>0.0005864333722910564</v>
+        <v>0.0007154893537480427</v>
       </c>
       <c r="J49" t="n">
-        <v>0.8301158019981648</v>
+        <v>0.8098123710989732</v>
       </c>
       <c r="K49" t="n">
-        <v>0.003774163838770095</v>
+        <v>0.005853473207585632</v>
       </c>
       <c r="L49" t="n">
-        <v>0.0004130480838088269</v>
+        <v>0.0007620559535455669</v>
       </c>
       <c r="M49" t="n">
-        <v>0.1919954648526077</v>
+        <v>0.1614965986394558</v>
       </c>
       <c r="N49" t="n">
-        <v>741.5859985351562</v>
+        <v>475.1187744140625</v>
       </c>
       <c r="O49" t="n">
-        <v>3.045758270631805</v>
+        <v>3.385749687296979</v>
       </c>
       <c r="P49" t="n">
-        <v>2.7509079510722e-11</v>
+        <v>1.649522971510552e-11</v>
       </c>
       <c r="Q49" t="n">
-        <v>3862.739037311213</v>
+        <v>2943.013811279915</v>
       </c>
     </row>
     <row r="50">
@@ -3258,54 +3258,54 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2339.044189453125</v>
+        <v>3862.518310546875</v>
       </c>
       <c r="E50" t="n">
-        <v>2339</v>
+        <v>3863</v>
       </c>
       <c r="F50" t="n">
-        <v>833.5315642493954</v>
+        <v>342.2259670039959</v>
       </c>
       <c r="G50" t="n">
-        <v>2.181040615102482</v>
+        <v>2.298600605490263</v>
       </c>
       <c r="H50" t="n">
-        <v>0.3563556293668301</v>
+        <v>0.08860177207950681</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0009324495128980077</v>
+        <v>0.0005951041317302689</v>
       </c>
       <c r="J50" t="n">
-        <v>1.13292288867092</v>
+        <v>0.827754412917569</v>
       </c>
       <c r="K50" t="n">
-        <v>0.002252287858549144</v>
+        <v>0.003803886191487528</v>
       </c>
       <c r="L50" t="n">
-        <v>0.0003927868497291857</v>
+        <v>0.0004181251484451382</v>
       </c>
       <c r="M50" t="n">
-        <v>0.7904988662131519</v>
+        <v>0.19</v>
       </c>
       <c r="N50" t="n">
-        <v>1849.011779785156</v>
+        <v>733.8784790039062</v>
       </c>
       <c r="O50" t="n">
-        <v>1.700255064897827</v>
+        <v>3.045758270631805</v>
       </c>
       <c r="P50" t="n">
-        <v>1.219344120318504e-10</v>
+        <v>2.7509079510722e-11</v>
       </c>
       <c r="Q50" t="n">
-        <v>2340.388090027172</v>
+        <v>3862.739037311213</v>
       </c>
     </row>
     <row r="51">
@@ -3323,46 +3323,46 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4050.933837890625</v>
+        <v>2339.044189453125</v>
       </c>
       <c r="E51" t="n">
-        <v>4051</v>
+        <v>2339</v>
       </c>
       <c r="F51" t="n">
-        <v>916.2758381885071</v>
+        <v>833.5840069916085</v>
       </c>
       <c r="G51" t="n">
-        <v>3.395661205768661</v>
+        <v>2.181407918987861</v>
       </c>
       <c r="H51" t="n">
-        <v>0.2261887937092609</v>
+        <v>0.3563780499531746</v>
       </c>
       <c r="I51" t="n">
-        <v>0.0008382415861762942</v>
+        <v>0.0009326065445124745</v>
       </c>
       <c r="J51" t="n">
-        <v>0.9352741379327487</v>
+        <v>1.132869132998374</v>
       </c>
       <c r="K51" t="n">
-        <v>0.002289990332693098</v>
+        <v>0.002252356036539126</v>
       </c>
       <c r="L51" t="n">
-        <v>0.0004352344504847237</v>
+        <v>0.0003928413067985622</v>
       </c>
       <c r="M51" t="n">
-        <v>0.4734920634920635</v>
+        <v>0.7904988662131519</v>
       </c>
       <c r="N51" t="n">
-        <v>1918.085021972656</v>
+        <v>1849.011779785156</v>
       </c>
       <c r="O51" t="n">
-        <v>1.28095518819708</v>
+        <v>1.700255064897827</v>
       </c>
       <c r="P51" t="n">
-        <v>3.398105938092607e-11</v>
+        <v>1.219344120318504e-10</v>
       </c>
       <c r="Q51" t="n">
-        <v>4050.203365680363</v>
+        <v>2340.388090027172</v>
       </c>
     </row>
     <row r="52">
@@ -3380,46 +3380,46 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5838.189697265625</v>
+        <v>4050.933837890625</v>
       </c>
       <c r="E52" t="n">
-        <v>5838</v>
+        <v>4051</v>
       </c>
       <c r="F52" t="n">
-        <v>555.1450293220936</v>
+        <v>917.0996027788008</v>
       </c>
       <c r="G52" t="n">
-        <v>2.832061453128816</v>
+        <v>3.35460397279866</v>
       </c>
       <c r="H52" t="n">
-        <v>0.09508855623209732</v>
+        <v>0.2263921454852362</v>
       </c>
       <c r="I52" t="n">
-        <v>0.0004850924002101611</v>
+        <v>0.0008281063347471128</v>
       </c>
       <c r="J52" t="n">
-        <v>0.8531948662396553</v>
+        <v>0.9345447395231181</v>
       </c>
       <c r="K52" t="n">
-        <v>0.002966196585971969</v>
+        <v>0.002262307113514107</v>
       </c>
       <c r="L52" t="n">
-        <v>0.0002708919184608968</v>
+        <v>0.0004260595446174934</v>
       </c>
       <c r="M52" t="n">
-        <v>0.2009977324263039</v>
+        <v>0.4765079365079365</v>
       </c>
       <c r="N52" t="n">
-        <v>1173.462890625</v>
+        <v>1930.302124023438</v>
       </c>
       <c r="O52" t="n">
-        <v>2.935485532484775</v>
+        <v>1.28095518819708</v>
       </c>
       <c r="P52" t="n">
-        <v>2.796867277425509e-11</v>
+        <v>3.398105938092607e-11</v>
       </c>
       <c r="Q52" t="n">
-        <v>5839.230198622787</v>
+        <v>4050.203365680363</v>
       </c>
     </row>
     <row r="53">
@@ -3437,46 +3437,46 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>8309.124755859375</v>
+        <v>5838.189697265625</v>
       </c>
       <c r="E53" t="n">
-        <v>8309</v>
+        <v>5838</v>
       </c>
       <c r="F53" t="n">
-        <v>1501.91919676692</v>
+        <v>556.742166996272</v>
       </c>
       <c r="G53" t="n">
-        <v>4.696898412724011</v>
+        <v>2.835407210387547</v>
       </c>
       <c r="H53" t="n">
-        <v>0.1807554033543432</v>
+        <v>0.09536212351185296</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0005652699352494236</v>
+        <v>0.0004856654814960087</v>
       </c>
       <c r="J53" t="n">
-        <v>0.9896115551617721</v>
+        <v>0.852015218070759</v>
       </c>
       <c r="K53" t="n">
-        <v>0.002208303270317655</v>
+        <v>0.00296068497791577</v>
       </c>
       <c r="L53" t="n">
-        <v>0.0002996444111471889</v>
+        <v>0.000271405493377466</v>
       </c>
       <c r="M53" t="n">
-        <v>0.4495011337868481</v>
+        <v>0.2024943310657596</v>
       </c>
       <c r="N53" t="n">
-        <v>3734.960998535156</v>
+        <v>1182.200317382812</v>
       </c>
       <c r="O53" t="n">
-        <v>1.387349873576789</v>
+        <v>2.935485532484775</v>
       </c>
       <c r="P53" t="n">
-        <v>9.021792532535704e-10</v>
+        <v>2.796867277425509e-11</v>
       </c>
       <c r="Q53" t="n">
-        <v>8309.988515326677</v>
+        <v>5839.230198622787</v>
       </c>
     </row>
     <row r="54">
@@ -3486,54 +3486,54 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>732.12890625</v>
+        <v>8309.124755859375</v>
       </c>
       <c r="E54" t="n">
-        <v>732</v>
+        <v>8309</v>
       </c>
       <c r="F54" t="n">
-        <v>426.0242234785599</v>
+        <v>1499.2154847065</v>
       </c>
       <c r="G54" t="n">
-        <v>0.9465588900473837</v>
+        <v>4.721668178412352</v>
       </c>
       <c r="H54" t="n">
-        <v>0.5818978322556294</v>
+        <v>0.1804300126375276</v>
       </c>
       <c r="I54" t="n">
-        <v>0.001292885558768202</v>
+        <v>0.0005682509671169345</v>
       </c>
       <c r="J54" t="n">
-        <v>0.5703322494834494</v>
+        <v>0.9907362329998584</v>
       </c>
       <c r="K54" t="n">
-        <v>0.001021537033707037</v>
+        <v>0.002232722066201099</v>
       </c>
       <c r="L54" t="n">
-        <v>8.321041434927589e-05</v>
+        <v>0.0003019276060763383</v>
       </c>
       <c r="M54" t="n">
-        <v>1.18</v>
+        <v>0.4485034013605442</v>
       </c>
       <c r="N54" t="n">
-        <v>863.912109375</v>
+        <v>3726.670715332031</v>
       </c>
       <c r="O54" t="n">
-        <v>1.869358907589715</v>
+        <v>1.387349873576789</v>
       </c>
       <c r="P54" t="n">
-        <v>8.443746198615233e-11</v>
+        <v>9.021792532535704e-10</v>
       </c>
       <c r="Q54" t="n">
-        <v>732.9333705336513</v>
+        <v>8309.988515326677</v>
       </c>
     </row>
     <row r="55">
@@ -3551,46 +3551,46 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>985.14404296875</v>
+        <v>732.12890625</v>
       </c>
       <c r="E55" t="n">
-        <v>985</v>
+        <v>732</v>
       </c>
       <c r="F55" t="n">
-        <v>694.8643004530124</v>
+        <v>466.8908553782699</v>
       </c>
       <c r="G55" t="n">
-        <v>2.539265973618143</v>
+        <v>2.639720523804578</v>
       </c>
       <c r="H55" t="n">
-        <v>0.7053428434272676</v>
+        <v>0.6377167345702925</v>
       </c>
       <c r="I55" t="n">
-        <v>0.002577558065484533</v>
+        <v>0.003605540638089753</v>
       </c>
       <c r="J55" t="n">
-        <v>0.4967652746459102</v>
+        <v>0.532957557326486</v>
       </c>
       <c r="K55" t="n">
-        <v>0.001374978075252021</v>
+        <v>0.001690174310438221</v>
       </c>
       <c r="L55" t="n">
-        <v>0.0002234264096304524</v>
+        <v>0.0006973145826312394</v>
       </c>
       <c r="M55" t="n">
-        <v>1.369002267573696</v>
+        <v>0.9765079365079365</v>
       </c>
       <c r="N55" t="n">
-        <v>1348.664428710938</v>
+        <v>714.9296875</v>
       </c>
       <c r="O55" t="n">
-        <v>2.111207187761406</v>
+        <v>1.869358907589715</v>
       </c>
       <c r="P55" t="n">
-        <v>4.54303482517407e-11</v>
+        <v>8.443746198615233e-11</v>
       </c>
       <c r="Q55" t="n">
-        <v>984.581668316362</v>
+        <v>732.9333705336513</v>
       </c>
     </row>
     <row r="56">
@@ -3608,46 +3608,46 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1633.831787109375</v>
+        <v>985.14404296875</v>
       </c>
       <c r="E56" t="n">
-        <v>1634</v>
+        <v>985</v>
       </c>
       <c r="F56" t="n">
-        <v>71.64584881729785</v>
+        <v>696.9823548207074</v>
       </c>
       <c r="G56" t="n">
-        <v>2.798029810765954</v>
+        <v>2.554349567951642</v>
       </c>
       <c r="H56" t="n">
-        <v>0.04385142300607082</v>
+        <v>0.7074928380222836</v>
       </c>
       <c r="I56" t="n">
-        <v>0.001712556845106015</v>
+        <v>0.002592869120188822</v>
       </c>
       <c r="J56" t="n">
-        <v>0.687888065524211</v>
+        <v>0.4969721945619245</v>
       </c>
       <c r="K56" t="n">
-        <v>0.01937478657080717</v>
+        <v>0.001379791810360227</v>
       </c>
       <c r="L56" t="n">
-        <v>0.005259074200213454</v>
+        <v>0.0002246153036921674</v>
       </c>
       <c r="M56" t="n">
-        <v>0.1085034013605442</v>
+        <v>1.370997732426304</v>
       </c>
       <c r="N56" t="n">
-        <v>177.2763061523438</v>
+        <v>1350.630249023438</v>
       </c>
       <c r="O56" t="n">
-        <v>5.527666438818121</v>
+        <v>2.111207187761406</v>
       </c>
       <c r="P56" t="n">
-        <v>9.064826848430388e-12</v>
+        <v>4.54303482517407e-11</v>
       </c>
       <c r="Q56" t="n">
-        <v>1634.412669824537</v>
+        <v>984.581668316362</v>
       </c>
     </row>
     <row r="57">
@@ -3665,46 +3665,46 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2225.994873046875</v>
+        <v>1633.831787109375</v>
       </c>
       <c r="E57" t="n">
-        <v>2226</v>
+        <v>1634</v>
       </c>
       <c r="F57" t="n">
-        <v>660.1708006533678</v>
+        <v>71.52513277406614</v>
       </c>
       <c r="G57" t="n">
-        <v>2.006211577553995</v>
+        <v>2.840549459637568</v>
       </c>
       <c r="H57" t="n">
-        <v>0.2965733697983526</v>
+        <v>0.04377753777248426</v>
       </c>
       <c r="I57" t="n">
-        <v>0.0009012651384987032</v>
+        <v>0.001738581341144766</v>
       </c>
       <c r="J57" t="n">
-        <v>0.8058744981350021</v>
+        <v>0.6867258990882481</v>
       </c>
       <c r="K57" t="n">
-        <v>0.001597878152246114</v>
+        <v>0.01967946836773346</v>
       </c>
       <c r="L57" t="n">
-        <v>0.0003043553852052328</v>
+        <v>0.005416107939043553</v>
       </c>
       <c r="M57" t="n">
-        <v>0.6334920634920634</v>
+        <v>0.1085034013605442</v>
       </c>
       <c r="N57" t="n">
-        <v>1410.150085449219</v>
+        <v>177.2763061523438</v>
       </c>
       <c r="O57" t="n">
-        <v>1.833350440871084</v>
+        <v>5.527666438818121</v>
       </c>
       <c r="P57" t="n">
-        <v>3.090843463916614e-11</v>
+        <v>9.064826848430388e-12</v>
       </c>
       <c r="Q57" t="n">
-        <v>2226.429989231169</v>
+        <v>1634.412669824537</v>
       </c>
     </row>
     <row r="58">
@@ -3714,54 +3714,54 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>TH13RearwaveformSOAE.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>904.39453125</v>
+        <v>2225.994873046875</v>
       </c>
       <c r="E58" t="n">
-        <v>904</v>
+        <v>2226</v>
       </c>
       <c r="F58" t="n">
-        <v>343.9176201914185</v>
+        <v>659.6315378637985</v>
       </c>
       <c r="G58" t="n">
-        <v>2.450073601578405</v>
+        <v>2.002654528766652</v>
       </c>
       <c r="H58" t="n">
-        <v>0.3802738830320835</v>
+        <v>0.2963311128209898</v>
       </c>
       <c r="I58" t="n">
-        <v>0.002709076091152454</v>
+        <v>0.0008996671793881892</v>
       </c>
       <c r="J58" t="n">
-        <v>0.5605367190463145</v>
+        <v>0.8053124687165877</v>
       </c>
       <c r="K58" t="n">
-        <v>0.002369263841942123</v>
+        <v>0.00159294414632699</v>
       </c>
       <c r="L58" t="n">
-        <v>0.0008353972374226948</v>
+        <v>0.0003045702927003857</v>
       </c>
       <c r="M58" t="n">
-        <v>0.65</v>
+        <v>0.6334920634920634</v>
       </c>
       <c r="N58" t="n">
-        <v>587.8564453125</v>
+        <v>1410.150085449219</v>
       </c>
       <c r="O58" t="n">
-        <v>2.545154730379255</v>
+        <v>1.833350440871084</v>
       </c>
       <c r="P58" t="n">
-        <v>7.161708852846133e-09</v>
+        <v>3.090843463916614e-11</v>
       </c>
       <c r="Q58" t="n">
-        <v>904.9686777906261</v>
+        <v>2226.429989231169</v>
       </c>
     </row>
     <row r="59">
@@ -3779,46 +3779,46 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1520.782470703125</v>
+        <v>904.39453125</v>
       </c>
       <c r="E59" t="n">
-        <v>1521</v>
+        <v>904</v>
       </c>
       <c r="F59" t="n">
-        <v>724.8780094116786</v>
+        <v>344.4738983224083</v>
       </c>
       <c r="G59" t="n">
-        <v>1.01886750048609</v>
+        <v>2.441175412334436</v>
       </c>
       <c r="H59" t="n">
-        <v>0.4766480567576081</v>
+        <v>0.3808889665070145</v>
       </c>
       <c r="I59" t="n">
-        <v>0.0006699626804713384</v>
+        <v>0.002699237255404883</v>
       </c>
       <c r="J59" t="n">
-        <v>0.7933168937124105</v>
+        <v>0.5612662783873309</v>
       </c>
       <c r="K59" t="n">
-        <v>0.0006971795280635326</v>
+        <v>0.002361355799389056</v>
       </c>
       <c r="L59" t="n">
-        <v>9.284643772323053e-05</v>
+        <v>0.00083175619909374</v>
       </c>
       <c r="M59" t="n">
-        <v>0.9170068027210885</v>
+        <v>0.6519954648526077</v>
       </c>
       <c r="N59" t="n">
-        <v>1394.56787109375</v>
+        <v>589.6611328125</v>
       </c>
       <c r="O59" t="n">
-        <v>1.952430412995464</v>
+        <v>2.545154730379255</v>
       </c>
       <c r="P59" t="n">
-        <v>7.462411328533061e-09</v>
+        <v>7.161708852846133e-09</v>
       </c>
       <c r="Q59" t="n">
-        <v>1520.304279797999</v>
+        <v>904.9686777906261</v>
       </c>
     </row>
     <row r="60">
@@ -3836,45 +3836,102 @@
         </is>
       </c>
       <c r="D60" t="n">
+        <v>1520.782470703125</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1521</v>
+      </c>
+      <c r="F60" t="n">
+        <v>723.72851177462</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1.008838437607111</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.4758921974159843</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.0006633680076156324</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.7936821896442126</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.0006928453911249745</v>
+      </c>
+      <c r="L60" t="n">
+        <v>9.168216013940688e-05</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.9195011337868481</v>
+      </c>
+      <c r="N60" t="n">
+        <v>1398.361206054688</v>
+      </c>
+      <c r="O60" t="n">
+        <v>1.952430412995464</v>
+      </c>
+      <c r="P60" t="n">
+        <v>7.462411328533061e-09</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>1520.304279797999</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TH13RearwaveformSOAE.mat</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
         <v>2037.579345703125</v>
       </c>
-      <c r="E60" t="n">
+      <c r="E61" t="n">
         <v>2038</v>
       </c>
-      <c r="F60" t="n">
-        <v>403.363723287138</v>
-      </c>
-      <c r="G60" t="n">
-        <v>0.6939979087577202</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.1979622163611723</v>
-      </c>
-      <c r="I60" t="n">
-        <v>0.0003405992067112539</v>
-      </c>
-      <c r="J60" t="n">
-        <v>0.9228832326415889</v>
-      </c>
-      <c r="K60" t="n">
-        <v>0.001064998810228081</v>
-      </c>
-      <c r="L60" t="n">
-        <v>7.753620886085926e-05</v>
-      </c>
-      <c r="M60" t="n">
-        <v>0.4160090702947846</v>
-      </c>
-      <c r="N60" t="n">
-        <v>847.6514892578125</v>
-      </c>
-      <c r="O60" t="n">
+      <c r="F61" t="n">
+        <v>403.6925223540505</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.6868993179924254</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.1981235838522621</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.0003371153714533709</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.9217583281829171</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.001053628699861245</v>
+      </c>
+      <c r="L61" t="n">
+        <v>7.611553383772669e-05</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.4185034013605442</v>
+      </c>
+      <c r="N61" t="n">
+        <v>852.73388671875</v>
+      </c>
+      <c r="O61" t="n">
         <v>1.725143363002918</v>
       </c>
-      <c r="P60" t="n">
+      <c r="P61" t="n">
         <v>8.231508706457555e-09</v>
       </c>
-      <c r="Q60" t="n">
+      <c r="Q61" t="n">
         <v>2038.146974608225</v>
       </c>
     </row>

</xml_diff>